<commit_message>
bench_suite: render N/A for skipped (Q, backend) cells
</commit_message>
<xml_diff>
--- a/bm_resultL4.xlsx
+++ b/bm_resultL4.xlsx
@@ -558,7 +558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B93"/>
+  <dimension ref="A1:B101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -922,631 +922,693 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>TPC-H 1.5.7 §5 compliance — auxiliary data structures</t>
+          <t>Origin &amp; methodology</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>Spec rule</t>
+          <t>Q1 / Q5 / Q6</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Each directive may reference no more than one base table and may not reference other auxiliary structures.  Each directive may reference one and only one of: PK column(s), FK column(s), or a date column.  Functions/expressions on those columns are allowed.  Multi-column / multi-table indexes are forbidden.</t>
+          <t>Teacher's reviewer-fixed reference (BitEngine branch).  Ported verbatim — same `context.client.bitmap_*` + `dynamic_cast&lt;rabit::Rabit*&gt;` pattern, same per-table semi-joins.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Q3 / Q4 / Q14 / Q15 / Q17 / Q19</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>COMPLIANT — bitmap_shipdate (date), bitmap_linestatus (varchar→ASCII byte), bitmap_returnflag (varchar→ASCII byte).  Each single column.</t>
+          <t>Ported by following the same teacher pattern + reading TPC-H spec §2.4.x for each query's predicate semantics.  Each port emits an [OK] line confirming the result matches DuckDB SQL ground truth.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q8 / Q10 / Q12</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>COMPLIANT — bitmap_orderkey (FK on l_orderkey), bitmap_shipdate (date).  Customer mktsegment + orders orderdate filters at query-time.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="3" t="inlineStr">
-        <is>
-          <t>Q4</t>
-        </is>
-      </c>
-      <c r="B42" s="5" t="inlineStr">
-        <is>
-          <t>COMPLIANT — bitmap_orderkey (FK on l_orderkey).  l_commitdate &lt; l_receiptdate evaluated at query-time on BMFetch'd cols.</t>
+          <t>Deferred.  These are 4-to-7-table aggregation queries where most of the work is in DuckDB SQL execution; a single bitmap-filter step would be a small fraction of total time and yield limited per-bitmap-op insight.  Old non-compliant pre-joined .bm files were retired pre-port; cells are intentionally blank in this workbook (not 0).</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="3" t="inlineStr">
-        <is>
-          <t>Q5</t>
-        </is>
-      </c>
-      <c r="B43" s="5" t="inlineStr">
-        <is>
-          <t>COMPLIANT — bitmap_orderkey + bitmap_suppkey (both FKs).  Region/nation/customer/orders/supplier semi-joins at query-time.</t>
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Empty / blank cells</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>Q6</t>
+          <t>Blank Q row</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>COMPLIANT — bitmap_shipdate_GE (date, year-bucketed) + bitmap_discount/quantity (single columns).  BPE variants over the SAME columns are TPC-H 1.5.7 explicitly allowed.</t>
+          <t>Q deferred (Q8 / Q10 / Q12) — see Origin &amp; methodology above.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>Q14</t>
+          <t>Blank backend cell</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>COMPLIANT — bitmap_shipdate (date) only.  PROMO% predicate evaluated by part scan at query-time.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="3" t="inlineStr">
-        <is>
-          <t>Q15</t>
-        </is>
-      </c>
-      <c r="B46" s="5" t="inlineStr">
-        <is>
-          <t>COMPLIANT — bitmap_shipdate (date) only.  Per-supplier max revenue computed at query-time.</t>
+          <t>Backend not run for that Q.  Two reasons: (a) PATTERN_BACKENDS_PER_Q gating — Q3/Q4/Q5/Q17 limit to CB/CR/CRR because WAH/EW/Concise per-key bitmap build over high-cardinality FK (orderkey 15M, partkey 2M unique values at SF10) exceeds practical memory budget; (b) BS/BSA only exist for the legacy Q6/Q15 paths.  ComBit's SparseComBit storage is specifically designed to handle these high-cardinality FK bitmaps that defeat per-value-bitvector backends.</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="3" t="inlineStr">
-        <is>
-          <t>Q17</t>
-        </is>
-      </c>
-      <c r="B47" s="5" t="inlineStr">
-        <is>
-          <t>COMPLIANT — bitmap_partkey (FK on l_partkey).  p_brand+p_container scan at query-time.</t>
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>TPC-H 1.5.7 §5 compliance — auxiliary data structures</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>Q19</t>
+          <t>Spec rule</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>COMPLIANT — bitmap_shipmode + bitmap_shipinstruct (each single varchar column).  3 OR-group brand+container+size+quantity predicates evaluated at query-time.</t>
+          <t>Each directive may reference no more than one base table and may not reference other auxiliary structures.  Each directive may reference one and only one of: PK column(s), FK column(s), or a date column.  Functions/expressions on those columns are allowed.  Multi-column / multi-table indexes are forbidden.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>Q8 / Q10</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>NOT BENCHED in this workbook (older bitmap-file pipeline retired pre-port).  The pre-built join_result/0.bm structures they relied on were multi-table — incompatible with TPC-H 1.5.7 §5 — and have been removed.  Future port follows the same pattern as Q3/Q4/Q5.</t>
+          <t>Mixed — bitmap_shipdate (date) is strict-compliant.  bitmap_linestatus + bitmap_returnflag reference VARCHAR columns; under a strict reading of 1.5.7 these are NOT permitted (only PK/FK/date).  Per teacher's BitEngine reference (rabit_linestatus / rabit_returnflag) we keep them — the academic methodology for bitmap research on TPC-H universally indexes these low-cardinality VARCHAR columns.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>Q12</t>
+          <t>Q3</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>PARTIAL — uses bitmap_shipmode + bitmap_receiptdate (single col, OK).  The previous pre-built commit_lt_receipt / ship_lt_commit bitmaps were two-column expressions and have been removed; commit/ship-date predicates are now evaluated at query-time on BMFetch'd cols.</t>
+          <t>COMPLIANT — bitmap_orderkey (FK on l_orderkey), bitmap_shipdate (date).  Customer mktsegment + orders orderdate filters at query-time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>COMPLIANT — bitmap_orderkey (FK on l_orderkey).  l_commitdate &lt; l_receiptdate evaluated at query-time on BMFetch'd cols.</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>Phase-name glossary (TPC-H query → phase semantics)</t>
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>Q5</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>COMPLIANT — bitmap_orderkey + bitmap_suppkey (both FKs).  Region/nation/customer/orders/supplier semi-joins at query-time.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>Q1 PhaseA</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>shipdate complement OR (~90 day-bitmaps for shipdate &gt; '1998-09-02') + flip in byte-stream space.</t>
+          <t>Q6</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>Mixed — bitmap_shipdate_GE (date, year-bucketed) is compliant.  bitmap_discount + bitmap_quantity (and the BPE variants) reference DECIMAL columns; under strict 1.5.7 not permitted.  Kept per teacher's BitEngine reference (rabit_discount / rabit_quantity).</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>Q1 PhaseB</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>Per-(returnflag, linestatus) group: linestatus_btv AND returnflag_btv, then byte-stream AND with shipdate filter.</t>
+          <t>Q14</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>COMPLIANT — bitmap_shipdate (date) only.  PROMO% predicate evaluated by part scan at query-time.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>Q1 PhaseC</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>Single sequential scan of lineitem(qty, price, disc, tax); per-row inline aggregate using the 5 group byte-streams (mirror of teacher's reduce_leadingbits).</t>
+          <t>Q15</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>COMPLIANT — bitmap_shipdate (date) only.  Per-supplier max revenue computed at query-time.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>Q3 PhaseA</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>Customer scan: c_mktsegment='BUILDING' → c_custkey set.</t>
+          <t>Q17</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>COMPLIANT — bitmap_partkey (FK on l_partkey).  p_brand+p_container scan at query-time.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>Q3 PhaseB</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>Orders scan: filter o_orderdate &lt; '1995-03-15' AND o_custkey ∈ set; for each match OR bitmap_orderkey[o_orderkey] into btv_res; build l_orderkey_map for downstream aggregate.</t>
+          <t>Q19</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>Non-strict — bitmap_shipmode + bitmap_shipinstruct (both VARCHAR).  Same caveat as Q1.  3 OR-group brand+container+size+quantity predicates evaluated at query-time on materialised cols (no aux on those — compliant).</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>Q3 PhaseC</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>Shipdate range OR (l_shipdate &gt; cutoff).</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="3" t="inlineStr">
-        <is>
-          <t>Q3 PhaseD</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>btv_res &amp;= shipdate_filter; get_rowids.</t>
+          <t>Q8 / Q10 / Q12</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>Deferred — see Origin &amp; methodology.  Older non-compliant pre-built multi-table bitmaps (join_result / late_lineitem / commit_lt_receipt / ship_lt_commit) were retired.</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="3" t="inlineStr">
-        <is>
-          <t>Q3 PhaseE</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>BMFetch lineitem(orderkey, price, discount) per row; sum revenue per orderkey.</t>
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Phase-name glossary (TPC-H query → phase semantics)</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>Q4 PhaseA</t>
+          <t>Q1 PhaseA</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Orders scan: filter o_orderdate ∈ [1993-07-01, 1993-10-01) → orderkey_priority map.</t>
+          <t>shipdate complement OR (~90 day-bitmaps for shipdate &gt; '1998-09-02') + flip in byte-stream space.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>Q4 PhaseB</t>
+          <t>Q1 PhaseB</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>OR matching orderkey bitmaps from bitmap_orderkey; get_rowids.</t>
+          <t>Per-(returnflag, linestatus) group: linestatus_btv AND returnflag_btv, then byte-stream AND with shipdate filter.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>Q4 PhaseC</t>
+          <t>Q1 PhaseC</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>BMFetch lineitem(orderkey, commitdate, receiptdate); per-row eval EXISTS commit &lt; receipt; collect orderkey set.</t>
+          <t>Single sequential scan of lineitem(qty, price, disc, tax); per-row inline aggregate using the 5 group byte-streams (mirror of teacher's reduce_leadingbits).</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>Q4 PhaseD</t>
+          <t>Q3 PhaseA</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Count by priority for orderkeys in the EXISTS set.</t>
+          <t>Customer scan: c_mktsegment='BUILDING' → c_custkey set.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>Q5 PhaseA</t>
+          <t>Q3 PhaseB</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>5 explicit semi-joins: region(ASIA) → nation → customer → orders(date range) → supplier.</t>
+          <t>Orders scan: filter o_orderdate &lt; '1995-03-15' AND o_custkey ∈ set; for each match OR bitmap_orderkey[o_orderkey] into btv_res; build l_orderkey_map for downstream aggregate.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>Q5 PhaseB</t>
+          <t>Q3 PhaseC</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Multi-OR over l_orderkey bitmaps for qualifying orders + multi-OR over l_suppkey bitmaps for qualifying suppliers; AND.</t>
+          <t>Shipdate range OR (l_shipdate &gt; cutoff).</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>Q5 PhaseC</t>
+          <t>Q3 PhaseD</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>BMFetch lineitem(orderkey, suppkey, price, discount); aggregate revenue per nation.</t>
+          <t>btv_res &amp;= shipdate_filter; get_rowids.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>Q6 ship_GE</t>
+          <t>Q3 PhaseE</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Apply per-year shipdate bitmap (Btvs_GE[1994]).</t>
+          <t>BMFetch lineitem(orderkey, price, discount) per row; sum revenue per orderkey.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>Q6 OR_disc</t>
+          <t>Q4 PhaseA</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Multi-OR over discount bitmaps in [5, 7], or single AND_NOT via discount_BPE.</t>
+          <t>Orders scan: filter o_orderdate ∈ [1993-07-01, 1993-10-01) → orderkey_priority map.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>Q6 OR_qty</t>
+          <t>Q4 PhaseB</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Multi-OR over quantity bitmaps in [0, 2399 raw], or single AND_NOT via quantity_BPE.</t>
+          <t>OR matching orderkey bitmaps from bitmap_orderkey; get_rowids.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>Q6 AND</t>
+          <t>Q4 PhaseC</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>btv_disc &amp;= btv_qty; btv_disc &amp;= btv_ship_GE.</t>
+          <t>BMFetch lineitem(orderkey, commitdate, receiptdate); per-row eval EXISTS commit &lt; receipt; collect orderkey set.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>Q6 GetRowIds</t>
+          <t>Q4 PhaseD</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Extract sorted row IDs from final result bitmap.</t>
+          <t>Count by priority for orderkeys in the EXISTS set.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>Q14 PhaseA</t>
+          <t>Q5 PhaseA</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Shipdate range OR (1 month: l_shipdate ∈ ['1995-09-01', '1995-10-01')).</t>
+          <t>5 explicit semi-joins: region(ASIA) → nation → customer → orders(date range) → supplier.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>Q14 PhaseB</t>
+          <t>Q5 PhaseB</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Part scan: p_type LIKE 'PROMO%' → promo_partkeys.</t>
+          <t>Multi-OR over l_orderkey bitmaps for qualifying orders + multi-OR over l_suppkey bitmaps for qualifying suppliers; AND.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>Q14 PhaseC</t>
+          <t>Q5 PhaseC</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>BMFetch lineitem(partkey, price, discount); accumulate total_rev + promo_rev (if l_partkey ∈ promo_set).</t>
+          <t>BMFetch lineitem(orderkey, suppkey, price, discount); aggregate revenue per nation.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>Q15 OR_ship</t>
+          <t>Q6 ship_GE</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Single-column shipdate range OR ([1996-01-01, 1996-04-01)).</t>
+          <t>Apply per-year shipdate bitmap (Btvs_GE[1994]).</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>Q15 walk</t>
+          <t>Q6 OR_disc</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Walk filter rows; revenue_by_suppkey[col_suppkey[r]] += price * (100 - disc).</t>
+          <t>Multi-OR over discount bitmaps in [5, 7], or single AND_NOT via discount_BPE.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>Q17 PhaseA</t>
+          <t>Q6 OR_qty</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Part scan: p_brand='Brand#23' AND p_container='MED BOX'; per-match OR bitmap_partkey[partkey].</t>
+          <t>Multi-OR over quantity bitmaps in [0, 2399 raw], or single AND_NOT via quantity_BPE.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>Q17 PhaseB</t>
+          <t>Q6 AND</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>BMFetch lineitem(partkey, qty, extprice); compute per-partkey avg(qty).</t>
+          <t>btv_disc &amp;= btv_qty; btv_disc &amp;= btv_ship_GE.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>Q17 PhaseC</t>
+          <t>Q6 GetRowIds</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Filter rows where qty &lt; 0.2 × avg_qty[partkey]; sum extprice.</t>
+          <t>Extract sorted row IDs from final result bitmap.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>Q19 PhaseA</t>
+          <t>Q14 PhaseA</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>bitmap_shipmode[A] AND bitmap_shipinstruct[D] (covers AIR + AIR REG + DELIVER IN PERSON).</t>
+          <t>Shipdate range OR (1 month: l_shipdate ∈ ['1995-09-01', '1995-10-01')).</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>Q19 PhaseB</t>
+          <t>Q14 PhaseB</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Part scan → unordered_map&lt;partkey, GroupSpec&gt; for the 3 OR-groups (brand×container×size×qty range).</t>
+          <t>Part scan: p_type LIKE 'PROMO%' → promo_partkeys.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>Q19 PhaseC</t>
+          <t>Q14 PhaseC</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>BMFetch lineitem(partkey, qty, price, disc); per-row look up partkey → group; check qty range; sum revenue.</t>
+          <t>BMFetch lineitem(partkey, price, discount); accumulate total_rev + promo_rev (if l_partkey ∈ promo_set).</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="3" t="inlineStr">
+        <is>
+          <t>Q15 OR_ship</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Single-column shipdate range OR ([1996-01-01, 1996-04-01)).</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="2" t="inlineStr">
-        <is>
-          <t>Algorithm matrix (per backend k-way OR strategy)</t>
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t>Q15 walk</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Walk filter rows; revenue_by_suppkey[col_suppkey[r]] += price * (100 - disc).</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>Q17 PhaseA</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Pairwise SparseComBit::apply_or_to (no native k-way merge; sparse segment storage already amortises common cases).</t>
+          <t>Part scan: p_brand='Brand#23' AND p_container='MED BOX'; per-match OR bitmap_partkey[partkey].</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>Q17 PhaseB</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Pairwise |= (CRoaring's standard mode — comparison baseline).</t>
+          <t>BMFetch lineitem(partkey, qty, extprice); compute per-partkey avg(qty).</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>CRR</t>
+          <t>Q17 PhaseC</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>fastunion (priority-queue k-way merge over run-optimised bitmaps; CRoaring's advertised path).</t>
+          <t>Filter rows where qty &lt; 0.2 × avg_qty[partkey]; sum extprice.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>WAH</t>
+          <t>Q19 PhaseA</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Pairwise |= (FastBit has no public k-way merge API).</t>
+          <t>bitmap_shipmode[A] AND bitmap_shipinstruct[D] (covers AIR + AIR REG + DELIVER IN PERSON).</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>EW</t>
+          <t>Q19 PhaseB</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>fast_logicalor (k-way priority-queue merge; EWAH's idiomatic path).</t>
+          <t>Part scan → unordered_map&lt;partkey, GroupSpec&gt; for the 3 OR-groups (brand×container×size×qty range).</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
+          <t>Q19 PhaseC</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>BMFetch lineitem(partkey, qty, price, disc); per-row look up partkey → group; check qty range; sum revenue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>Algorithm matrix (per backend k-way OR strategy)</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Pairwise SparseComBit::apply_or_to (no native k-way merge; sparse segment storage already amortises common cases).</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="3" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Pairwise |= (CRoaring's standard mode — comparison baseline).</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="3" t="inlineStr">
+        <is>
+          <t>CRR</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>fastunion (priority-queue k-way merge over run-optimised bitmaps; CRoaring's advertised path).</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="3" t="inlineStr">
+        <is>
+          <t>WAH</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Pairwise |= (FastBit has no public k-way merge API).</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="3" t="inlineStr">
+        <is>
+          <t>EW</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>fast_logicalor (k-way priority-queue merge; EWAH's idiomatic path).</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="3" t="inlineStr">
+        <is>
           <t>CON</t>
         </is>
       </c>
-      <c r="B91" t="inlineStr">
+      <c r="B99" t="inlineStr">
         <is>
           <t>fast_logicalor (k-way merge; Concise's idiomatic path).</t>
         </is>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" s="3" t="inlineStr">
+    <row r="100">
+      <c r="A100" s="3" t="inlineStr">
         <is>
           <t>BS</t>
         </is>
       </c>
-      <c r="B92" t="inlineStr">
+      <c r="B100" t="inlineStr">
         <is>
           <t>Scalar word-level OR (uncompressed reference, single-pass through 64-bit words).</t>
         </is>
       </c>
     </row>
-    <row r="93">
-      <c r="A93" s="3" t="inlineStr">
+    <row r="101">
+      <c r="A101" s="3" t="inlineStr">
         <is>
           <t>BSA</t>
         </is>
       </c>
-      <c r="B93" t="inlineStr">
+      <c r="B101" t="inlineStr">
         <is>
           <t>AVX-512 word-level OR (same data layout as BS, vectorised).</t>
         </is>
@@ -1651,12 +1713,8 @@
       <c r="F2" s="8" t="n">
         <v>1251.543</v>
       </c>
-      <c r="G2" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="G2" s="9" t="n"/>
+      <c r="H2" s="9" t="n"/>
       <c r="I2" s="8" t="n">
         <v>1295.5445</v>
       </c>
@@ -1668,9 +1726,7 @@
           <t>Q3</t>
         </is>
       </c>
-      <c r="B3" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="B3" s="9" t="n"/>
       <c r="C3" s="8" t="n">
         <v>2316.3235</v>
       </c>
@@ -1680,18 +1736,10 @@
       <c r="E3" s="8" t="n">
         <v>4270.994</v>
       </c>
-      <c r="F3" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="F3" s="9" t="n"/>
+      <c r="G3" s="9" t="n"/>
+      <c r="H3" s="9" t="n"/>
+      <c r="I3" s="9" t="n"/>
       <c r="J3" s="9" t="n"/>
     </row>
     <row r="4">
@@ -1700,9 +1748,7 @@
           <t>Q4</t>
         </is>
       </c>
-      <c r="B4" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="B4" s="9" t="n"/>
       <c r="C4" s="8" t="n">
         <v>803.9135</v>
       </c>
@@ -1712,18 +1758,10 @@
       <c r="E4" s="8" t="n">
         <v>692.117</v>
       </c>
-      <c r="F4" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="F4" s="9" t="n"/>
+      <c r="G4" s="9" t="n"/>
+      <c r="H4" s="9" t="n"/>
+      <c r="I4" s="9" t="n"/>
       <c r="J4" s="9" t="n"/>
     </row>
     <row r="5">
@@ -1732,9 +1770,7 @@
           <t>Q5</t>
         </is>
       </c>
-      <c r="B5" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="B5" s="9" t="n"/>
       <c r="C5" s="8" t="n">
         <v>1259.6405</v>
       </c>
@@ -1744,18 +1780,10 @@
       <c r="E5" s="8" t="n">
         <v>912.5085</v>
       </c>
-      <c r="F5" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="F5" s="9" t="n"/>
+      <c r="G5" s="9" t="n"/>
+      <c r="H5" s="9" t="n"/>
+      <c r="I5" s="9" t="n"/>
       <c r="J5" s="9" t="n"/>
     </row>
     <row r="6">
@@ -1779,12 +1807,8 @@
       <c r="F6" s="8" t="n">
         <v>210.889</v>
       </c>
-      <c r="G6" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="G6" s="9" t="n"/>
+      <c r="H6" s="9" t="n"/>
       <c r="I6" s="8" t="n">
         <v>616.513</v>
       </c>
@@ -1859,12 +1883,8 @@
       <c r="F10" s="8" t="n">
         <v>232.1375</v>
       </c>
-      <c r="G10" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="G10" s="9" t="n"/>
+      <c r="H10" s="9" t="n"/>
       <c r="I10" s="8" t="n">
         <v>238.1145</v>
       </c>
@@ -1910,9 +1930,7 @@
           <t>Q17</t>
         </is>
       </c>
-      <c r="B12" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="B12" s="9" t="n"/>
       <c r="C12" s="8" t="n">
         <v>63.095</v>
       </c>
@@ -1922,18 +1940,10 @@
       <c r="E12" s="8" t="n">
         <v>49.318</v>
       </c>
-      <c r="F12" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="F12" s="9" t="n"/>
+      <c r="G12" s="9" t="n"/>
+      <c r="H12" s="9" t="n"/>
+      <c r="I12" s="9" t="n"/>
       <c r="J12" s="9" t="n"/>
     </row>
     <row r="13">
@@ -1957,12 +1967,8 @@
       <c r="F13" s="8" t="n">
         <v>239.8755</v>
       </c>
-      <c r="G13" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="G13" s="9" t="n"/>
+      <c r="H13" s="9" t="n"/>
       <c r="I13" s="8" t="n">
         <v>268.6065</v>
       </c>
@@ -2216,12 +2222,8 @@
       <c r="G2" s="8" t="n">
         <v>77.97750000000001</v>
       </c>
-      <c r="H2" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="H2" s="9" t="n"/>
+      <c r="I2" s="9" t="n"/>
       <c r="J2" s="8" t="n">
         <v>85.383</v>
       </c>
@@ -2248,12 +2250,8 @@
       <c r="G3" s="8" t="n">
         <v>369.6275</v>
       </c>
-      <c r="H3" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="H3" s="9" t="n"/>
+      <c r="I3" s="9" t="n"/>
       <c r="J3" s="8" t="n">
         <v>406.7575</v>
       </c>
@@ -2280,12 +2278,8 @@
       <c r="G4" s="8" t="n">
         <v>804.423</v>
       </c>
-      <c r="H4" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="H4" s="9" t="n"/>
+      <c r="I4" s="9" t="n"/>
       <c r="J4" s="8" t="n">
         <v>802.9745</v>
       </c>
@@ -2312,12 +2306,8 @@
       <c r="G5" s="8" t="n">
         <v>1251.543</v>
       </c>
-      <c r="H5" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="H5" s="9" t="n"/>
+      <c r="I5" s="9" t="n"/>
       <c r="J5" s="8" t="n">
         <v>1295.5445</v>
       </c>
@@ -2333,9 +2323,7 @@
           <t>PhaseA_cust</t>
         </is>
       </c>
-      <c r="C6" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="C6" s="9" t="n"/>
       <c r="D6" s="8" t="n">
         <v>24.2085</v>
       </c>
@@ -2345,18 +2333,10 @@
       <c r="F6" s="8" t="n">
         <v>23.236</v>
       </c>
-      <c r="G6" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="G6" s="9" t="n"/>
+      <c r="H6" s="9" t="n"/>
+      <c r="I6" s="9" t="n"/>
+      <c r="J6" s="9" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="11" t="n"/>
@@ -2365,9 +2345,7 @@
           <t>PhaseB_okey</t>
         </is>
       </c>
-      <c r="C7" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="C7" s="9" t="n"/>
       <c r="D7" s="8" t="n">
         <v>1295.9505</v>
       </c>
@@ -2377,18 +2355,10 @@
       <c r="F7" s="8" t="n">
         <v>4021.0805</v>
       </c>
-      <c r="G7" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="G7" s="9" t="n"/>
+      <c r="H7" s="9" t="n"/>
+      <c r="I7" s="9" t="n"/>
+      <c r="J7" s="9" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="11" t="n"/>
@@ -2397,9 +2367,7 @@
           <t>PhaseC_ship</t>
         </is>
       </c>
-      <c r="C8" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="C8" s="9" t="n"/>
       <c r="D8" s="8" t="n">
         <v>905.0185</v>
       </c>
@@ -2409,18 +2377,10 @@
       <c r="F8" s="8" t="n">
         <v>129.3805</v>
       </c>
-      <c r="G8" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="G8" s="9" t="n"/>
+      <c r="H8" s="9" t="n"/>
+      <c r="I8" s="9" t="n"/>
+      <c r="J8" s="9" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="11" t="n"/>
@@ -2429,9 +2389,7 @@
           <t>PhaseD_AND</t>
         </is>
       </c>
-      <c r="C9" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="C9" s="9" t="n"/>
       <c r="D9" s="8" t="n">
         <v>8.628</v>
       </c>
@@ -2441,18 +2399,10 @@
       <c r="F9" s="8" t="n">
         <v>14.4405</v>
       </c>
-      <c r="G9" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="G9" s="9" t="n"/>
+      <c r="H9" s="9" t="n"/>
+      <c r="I9" s="9" t="n"/>
+      <c r="J9" s="9" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="11" t="n"/>
@@ -2461,9 +2411,7 @@
           <t>PhaseE_agg</t>
         </is>
       </c>
-      <c r="C10" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="C10" s="9" t="n"/>
       <c r="D10" s="8" t="n">
         <v>82.74250000000001</v>
       </c>
@@ -2473,18 +2421,10 @@
       <c r="F10" s="8" t="n">
         <v>82.9225</v>
       </c>
-      <c r="G10" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="G10" s="9" t="n"/>
+      <c r="H10" s="9" t="n"/>
+      <c r="I10" s="9" t="n"/>
+      <c r="J10" s="9" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="12" t="n"/>
@@ -2493,9 +2433,7 @@
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C11" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="C11" s="9" t="n"/>
       <c r="D11" s="8" t="n">
         <v>2316.3235</v>
       </c>
@@ -2505,18 +2443,10 @@
       <c r="F11" s="8" t="n">
         <v>4270.994</v>
       </c>
-      <c r="G11" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="G11" s="9" t="n"/>
+      <c r="H11" s="9" t="n"/>
+      <c r="I11" s="9" t="n"/>
+      <c r="J11" s="9" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -2529,9 +2459,7 @@
           <t>PhaseA_orders</t>
         </is>
       </c>
-      <c r="C12" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="C12" s="9" t="n"/>
       <c r="D12" s="8" t="n">
         <v>243.1395</v>
       </c>
@@ -2541,18 +2469,10 @@
       <c r="F12" s="8" t="n">
         <v>243.415</v>
       </c>
-      <c r="G12" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="G12" s="9" t="n"/>
+      <c r="H12" s="9" t="n"/>
+      <c r="I12" s="9" t="n"/>
+      <c r="J12" s="9" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="11" t="n"/>
@@ -2561,9 +2481,7 @@
           <t>PhaseB_okey</t>
         </is>
       </c>
-      <c r="C13" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="C13" s="9" t="n"/>
       <c r="D13" s="8" t="n">
         <v>267.958</v>
       </c>
@@ -2573,18 +2491,10 @@
       <c r="F13" s="8" t="n">
         <v>155.5355</v>
       </c>
-      <c r="G13" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="G13" s="9" t="n"/>
+      <c r="H13" s="9" t="n"/>
+      <c r="I13" s="9" t="n"/>
+      <c r="J13" s="9" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="11" t="n"/>
@@ -2593,9 +2503,7 @@
           <t>PhaseC_exists</t>
         </is>
       </c>
-      <c r="C14" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="C14" s="9" t="n"/>
       <c r="D14" s="8" t="n">
         <v>234.0405</v>
       </c>
@@ -2605,18 +2513,10 @@
       <c r="F14" s="8" t="n">
         <v>234.898</v>
       </c>
-      <c r="G14" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="G14" s="9" t="n"/>
+      <c r="H14" s="9" t="n"/>
+      <c r="I14" s="9" t="n"/>
+      <c r="J14" s="9" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="11" t="n"/>
@@ -2625,9 +2525,7 @@
           <t>PhaseD_count</t>
         </is>
       </c>
-      <c r="C15" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="C15" s="9" t="n"/>
       <c r="D15" s="8" t="n">
         <v>57.9415</v>
       </c>
@@ -2637,18 +2535,10 @@
       <c r="F15" s="8" t="n">
         <v>57.923</v>
       </c>
-      <c r="G15" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="G15" s="9" t="n"/>
+      <c r="H15" s="9" t="n"/>
+      <c r="I15" s="9" t="n"/>
+      <c r="J15" s="9" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="12" t="n"/>
@@ -2657,9 +2547,7 @@
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C16" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="C16" s="9" t="n"/>
       <c r="D16" s="8" t="n">
         <v>803.9135</v>
       </c>
@@ -2669,18 +2557,10 @@
       <c r="F16" s="8" t="n">
         <v>692.117</v>
       </c>
-      <c r="G16" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="G16" s="9" t="n"/>
+      <c r="H16" s="9" t="n"/>
+      <c r="I16" s="9" t="n"/>
+      <c r="J16" s="9" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -2693,9 +2573,7 @@
           <t>PhaseA</t>
         </is>
       </c>
-      <c r="C17" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="C17" s="9" t="n"/>
       <c r="D17" s="8" t="n">
         <v>278.671</v>
       </c>
@@ -2705,18 +2583,10 @@
       <c r="F17" s="8" t="n">
         <v>281.5675</v>
       </c>
-      <c r="G17" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="G17" s="9" t="n"/>
+      <c r="H17" s="9" t="n"/>
+      <c r="I17" s="9" t="n"/>
+      <c r="J17" s="9" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="11" t="n"/>
@@ -2725,9 +2595,7 @@
           <t>PhaseB</t>
         </is>
       </c>
-      <c r="C18" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="C18" s="9" t="n"/>
       <c r="D18" s="8" t="n">
         <v>859.4335</v>
       </c>
@@ -2737,18 +2605,10 @@
       <c r="F18" s="8" t="n">
         <v>510.023</v>
       </c>
-      <c r="G18" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="G18" s="9" t="n"/>
+      <c r="H18" s="9" t="n"/>
+      <c r="I18" s="9" t="n"/>
+      <c r="J18" s="9" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="11" t="n"/>
@@ -2757,9 +2617,7 @@
           <t>PhaseC</t>
         </is>
       </c>
-      <c r="C19" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="C19" s="9" t="n"/>
       <c r="D19" s="8" t="n">
         <v>121.496</v>
       </c>
@@ -2769,18 +2627,10 @@
       <c r="F19" s="8" t="n">
         <v>121.1895</v>
       </c>
-      <c r="G19" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="G19" s="9" t="n"/>
+      <c r="H19" s="9" t="n"/>
+      <c r="I19" s="9" t="n"/>
+      <c r="J19" s="9" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="12" t="n"/>
@@ -2789,9 +2639,7 @@
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C20" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="C20" s="9" t="n"/>
       <c r="D20" s="8" t="n">
         <v>1259.6405</v>
       </c>
@@ -2801,18 +2649,10 @@
       <c r="F20" s="8" t="n">
         <v>912.5085</v>
       </c>
-      <c r="G20" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H20" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I20" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="G20" s="9" t="n"/>
+      <c r="H20" s="9" t="n"/>
+      <c r="I20" s="9" t="n"/>
+      <c r="J20" s="9" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -2840,12 +2680,8 @@
       <c r="G21" s="8" t="n">
         <v>2.897</v>
       </c>
-      <c r="H21" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I21" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="H21" s="9" t="n"/>
+      <c r="I21" s="9" t="n"/>
       <c r="J21" s="8" t="n">
         <v>1.179</v>
       </c>
@@ -2872,12 +2708,8 @@
       <c r="G22" s="8" t="n">
         <v>5.984</v>
       </c>
-      <c r="H22" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I22" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="H22" s="9" t="n"/>
+      <c r="I22" s="9" t="n"/>
       <c r="J22" s="8" t="n">
         <v>26.877</v>
       </c>
@@ -2904,12 +2736,8 @@
       <c r="G23" s="8" t="n">
         <v>177.358</v>
       </c>
-      <c r="H23" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="H23" s="9" t="n"/>
+      <c r="I23" s="9" t="n"/>
       <c r="J23" s="8" t="n">
         <v>507.12</v>
       </c>
@@ -2936,12 +2764,8 @@
       <c r="G24" s="8" t="n">
         <v>12.418</v>
       </c>
-      <c r="H24" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="H24" s="9" t="n"/>
+      <c r="I24" s="9" t="n"/>
       <c r="J24" s="8" t="n">
         <v>64.56</v>
       </c>
@@ -2968,12 +2792,8 @@
       <c r="G25" s="8" t="n">
         <v>12.222</v>
       </c>
-      <c r="H25" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I25" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="H25" s="9" t="n"/>
+      <c r="I25" s="9" t="n"/>
       <c r="J25" s="8" t="n">
         <v>16.765</v>
       </c>
@@ -3000,12 +2820,8 @@
       <c r="G26" s="8" t="n">
         <v>210.889</v>
       </c>
-      <c r="H26" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I26" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="H26" s="9" t="n"/>
+      <c r="I26" s="9" t="n"/>
       <c r="J26" s="8" t="n">
         <v>616.513</v>
       </c>
@@ -3036,12 +2852,8 @@
       <c r="G27" s="8" t="n">
         <v>62.5325</v>
       </c>
-      <c r="H27" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I27" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="H27" s="9" t="n"/>
+      <c r="I27" s="9" t="n"/>
       <c r="J27" s="8" t="n">
         <v>69.587</v>
       </c>
@@ -3068,12 +2880,8 @@
       <c r="G28" s="8" t="n">
         <v>79.033</v>
       </c>
-      <c r="H28" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I28" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="H28" s="9" t="n"/>
+      <c r="I28" s="9" t="n"/>
       <c r="J28" s="8" t="n">
         <v>78.62649999999999</v>
       </c>
@@ -3100,12 +2908,8 @@
       <c r="G29" s="8" t="n">
         <v>90.7225</v>
       </c>
-      <c r="H29" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I29" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="H29" s="9" t="n"/>
+      <c r="I29" s="9" t="n"/>
       <c r="J29" s="8" t="n">
         <v>89.8925</v>
       </c>
@@ -3132,12 +2936,8 @@
       <c r="G30" s="8" t="n">
         <v>232.1375</v>
       </c>
-      <c r="H30" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I30" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="H30" s="9" t="n"/>
+      <c r="I30" s="9" t="n"/>
       <c r="J30" s="8" t="n">
         <v>238.1145</v>
       </c>
@@ -3253,9 +3053,7 @@
           <t>PhaseA_part</t>
         </is>
       </c>
-      <c r="C34" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="C34" s="9" t="n"/>
       <c r="D34" s="8" t="n">
         <v>41.7295</v>
       </c>
@@ -3265,18 +3063,10 @@
       <c r="F34" s="8" t="n">
         <v>30.4145</v>
       </c>
-      <c r="G34" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H34" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I34" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J34" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="G34" s="9" t="n"/>
+      <c r="H34" s="9" t="n"/>
+      <c r="I34" s="9" t="n"/>
+      <c r="J34" s="9" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="11" t="n"/>
@@ -3285,9 +3075,7 @@
           <t>PhaseB_avg</t>
         </is>
       </c>
-      <c r="C35" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="C35" s="9" t="n"/>
       <c r="D35" s="8" t="n">
         <v>20.3075</v>
       </c>
@@ -3297,18 +3085,10 @@
       <c r="F35" s="8" t="n">
         <v>17.963</v>
       </c>
-      <c r="G35" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H35" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I35" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J35" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="G35" s="9" t="n"/>
+      <c r="H35" s="9" t="n"/>
+      <c r="I35" s="9" t="n"/>
+      <c r="J35" s="9" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="11" t="n"/>
@@ -3317,9 +3097,7 @@
           <t>PhaseC_sum</t>
         </is>
       </c>
-      <c r="C36" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="C36" s="9" t="n"/>
       <c r="D36" s="8" t="n">
         <v>1.071</v>
       </c>
@@ -3329,18 +3107,10 @@
       <c r="F36" s="8" t="n">
         <v>0.9370000000000001</v>
       </c>
-      <c r="G36" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H36" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I36" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J36" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="G36" s="9" t="n"/>
+      <c r="H36" s="9" t="n"/>
+      <c r="I36" s="9" t="n"/>
+      <c r="J36" s="9" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="12" t="n"/>
@@ -3349,9 +3119,7 @@
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C37" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="C37" s="9" t="n"/>
       <c r="D37" s="8" t="n">
         <v>63.095</v>
       </c>
@@ -3361,18 +3129,10 @@
       <c r="F37" s="8" t="n">
         <v>49.318</v>
       </c>
-      <c r="G37" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H37" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I37" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J37" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="G37" s="9" t="n"/>
+      <c r="H37" s="9" t="n"/>
+      <c r="I37" s="9" t="n"/>
+      <c r="J37" s="9" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -3400,12 +3160,8 @@
       <c r="G38" s="8" t="n">
         <v>50.499</v>
       </c>
-      <c r="H38" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I38" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="H38" s="9" t="n"/>
+      <c r="I38" s="9" t="n"/>
       <c r="J38" s="8" t="n">
         <v>80.13549999999999</v>
       </c>
@@ -3432,12 +3188,8 @@
       <c r="G39" s="8" t="n">
         <v>28.0165</v>
       </c>
-      <c r="H39" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I39" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="H39" s="9" t="n"/>
+      <c r="I39" s="9" t="n"/>
       <c r="J39" s="8" t="n">
         <v>28.0805</v>
       </c>
@@ -3464,12 +3216,8 @@
       <c r="G40" s="8" t="n">
         <v>161.2035</v>
       </c>
-      <c r="H40" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I40" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="H40" s="9" t="n"/>
+      <c r="I40" s="9" t="n"/>
       <c r="J40" s="8" t="n">
         <v>160.563</v>
       </c>
@@ -3496,12 +3244,8 @@
       <c r="G41" s="8" t="n">
         <v>239.8755</v>
       </c>
-      <c r="H41" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I41" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="H41" s="9" t="n"/>
+      <c r="I41" s="9" t="n"/>
       <c r="J41" s="8" t="n">
         <v>268.6065</v>
       </c>

</xml_diff>

<commit_message>
bm_resultL4.xlsx: refreshed Q3/Q4/Q5/Q17 with broader backend coverage
</commit_message>
<xml_diff>
--- a/bm_resultL4.xlsx
+++ b/bm_resultL4.xlsx
@@ -989,7 +989,7 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Backend not run for that Q.  Two reasons: (a) PATTERN_BACKENDS_PER_Q gating — Q3/Q4/Q5/Q17 limit to CB/CR/CRR because WAH/EW/Concise per-key bitmap build over high-cardinality FK (orderkey 15M, partkey 2M unique values at SF10) exceeds practical memory budget; (b) BS/BSA only exist for the legacy Q6/Q15 paths.  ComBit's SparseComBit storage is specifically designed to handle these high-cardinality FK bitmaps that defeat per-value-bitvector backends.</t>
+          <t>Backend not run for that Q.  Gating is on runtime OR fan-out per-iteration:  Q3/Q4 (~590k orderkeys after the orders-scan + custkey-set semi-join) — only CB/CR/CRR finish in seconds; WAH has no k-way merge (pairwise OR over a 1.27 GB index = ~60 min/iter); EWAH/Concise's fast_logicalor priority-queue setup is O(K log K) and at K=590k empirically hangs &gt;30 min/iter.  Q5 (~28k orderkeys) — WAH still gated, CR/CRR/EW/CON all run.  Q17 (~200 partkey ORs after Brand#23 + MED BOX) — all 6 run.  BS/BSA cells are blank: the legacy dense-bit-array baseline relied on file-format predicate pre-derivation incompatible with the new per-value PRAGMA load_bitmap pattern.</t>
         </is>
       </c>
     </row>
@@ -1728,13 +1728,13 @@
       </c>
       <c r="B3" s="9" t="n"/>
       <c r="C3" s="8" t="n">
-        <v>2316.3235</v>
+        <v>2311.252</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>2760.6415</v>
+        <v>2817.675</v>
       </c>
       <c r="E3" s="8" t="n">
-        <v>4270.994</v>
+        <v>4330.24</v>
       </c>
       <c r="F3" s="9" t="n"/>
       <c r="G3" s="9" t="n"/>
@@ -1750,13 +1750,13 @@
       </c>
       <c r="B4" s="9" t="n"/>
       <c r="C4" s="8" t="n">
-        <v>803.9135</v>
+        <v>828.6325000000001</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>1015.1315</v>
+        <v>1059.1705</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>692.117</v>
+        <v>702.6345</v>
       </c>
       <c r="F4" s="9" t="n"/>
       <c r="G4" s="9" t="n"/>
@@ -1772,18 +1772,22 @@
       </c>
       <c r="B5" s="9" t="n"/>
       <c r="C5" s="8" t="n">
-        <v>1259.6405</v>
+        <v>1343.0815</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>2968.167</v>
+        <v>2880.6655</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>912.5085</v>
-      </c>
-      <c r="F5" s="9" t="n"/>
+        <v>971.0975</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>3043.593</v>
+      </c>
       <c r="G5" s="9" t="n"/>
       <c r="H5" s="9" t="n"/>
-      <c r="I5" s="9" t="n"/>
+      <c r="I5" s="8" t="n">
+        <v>3077.1495</v>
+      </c>
       <c r="J5" s="9" t="n"/>
     </row>
     <row r="6">
@@ -1869,24 +1873,24 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>275.8775</v>
+        <v>277.389</v>
       </c>
       <c r="C10" s="8" t="n">
-        <v>205.407</v>
+        <v>207.964</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>188.3935</v>
+        <v>190.287</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>176.6925</v>
+        <v>179.7225</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>232.1375</v>
+        <v>229.2315</v>
       </c>
       <c r="G10" s="9" t="n"/>
       <c r="H10" s="9" t="n"/>
       <c r="I10" s="8" t="n">
-        <v>238.1145</v>
+        <v>245.095</v>
       </c>
       <c r="J10" s="9" t="n"/>
     </row>
@@ -1930,20 +1934,26 @@
           <t>Q17</t>
         </is>
       </c>
-      <c r="B12" s="9" t="n"/>
+      <c r="B12" s="8" t="n">
+        <v>468.0545</v>
+      </c>
       <c r="C12" s="8" t="n">
-        <v>63.095</v>
+        <v>56.996</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>52.4</v>
+        <v>52.332</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>49.318</v>
-      </c>
-      <c r="F12" s="9" t="n"/>
+        <v>52.9235</v>
+      </c>
+      <c r="F12" s="8" t="n">
+        <v>495.2225</v>
+      </c>
       <c r="G12" s="9" t="n"/>
       <c r="H12" s="9" t="n"/>
-      <c r="I12" s="9" t="n"/>
+      <c r="I12" s="8" t="n">
+        <v>540.683</v>
+      </c>
       <c r="J12" s="9" t="n"/>
     </row>
     <row r="13">
@@ -2325,13 +2335,13 @@
       </c>
       <c r="C6" s="9" t="n"/>
       <c r="D6" s="8" t="n">
-        <v>24.2085</v>
+        <v>22.327</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>23.022</v>
+        <v>22.917</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>23.236</v>
+        <v>23.222</v>
       </c>
       <c r="G6" s="9" t="n"/>
       <c r="H6" s="9" t="n"/>
@@ -2347,13 +2357,13 @@
       </c>
       <c r="C7" s="9" t="n"/>
       <c r="D7" s="8" t="n">
-        <v>1295.9505</v>
+        <v>1290.917</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>2349.221</v>
+        <v>2398.808</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>4021.0805</v>
+        <v>4082.7515</v>
       </c>
       <c r="G7" s="9" t="n"/>
       <c r="H7" s="9" t="n"/>
@@ -2369,13 +2379,13 @@
       </c>
       <c r="C8" s="9" t="n"/>
       <c r="D8" s="8" t="n">
-        <v>905.0185</v>
+        <v>908.941</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>300.282</v>
+        <v>307.9585</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>129.3805</v>
+        <v>129.2175</v>
       </c>
       <c r="G8" s="9" t="n"/>
       <c r="H8" s="9" t="n"/>
@@ -2391,13 +2401,13 @@
       </c>
       <c r="C9" s="9" t="n"/>
       <c r="D9" s="8" t="n">
-        <v>8.628</v>
+        <v>8.102</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>5.4545</v>
+        <v>5.73</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>14.4405</v>
+        <v>14.244</v>
       </c>
       <c r="G9" s="9" t="n"/>
       <c r="H9" s="9" t="n"/>
@@ -2413,13 +2423,13 @@
       </c>
       <c r="C10" s="9" t="n"/>
       <c r="D10" s="8" t="n">
-        <v>82.74250000000001</v>
+        <v>81.441</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>83.042</v>
+        <v>82.407</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>82.9225</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="G10" s="9" t="n"/>
       <c r="H10" s="9" t="n"/>
@@ -2435,13 +2445,13 @@
       </c>
       <c r="C11" s="9" t="n"/>
       <c r="D11" s="8" t="n">
-        <v>2316.3235</v>
+        <v>2311.252</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>2760.6415</v>
+        <v>2817.675</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>4270.994</v>
+        <v>4330.24</v>
       </c>
       <c r="G11" s="9" t="n"/>
       <c r="H11" s="9" t="n"/>
@@ -2461,13 +2471,13 @@
       </c>
       <c r="C12" s="9" t="n"/>
       <c r="D12" s="8" t="n">
-        <v>243.1395</v>
+        <v>248.2625</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>242.639</v>
+        <v>249.4155</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>243.415</v>
+        <v>245.2065</v>
       </c>
       <c r="G12" s="9" t="n"/>
       <c r="H12" s="9" t="n"/>
@@ -2483,13 +2493,13 @@
       </c>
       <c r="C13" s="9" t="n"/>
       <c r="D13" s="8" t="n">
-        <v>267.958</v>
+        <v>281.15</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>478.916</v>
+        <v>507.4705</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>155.5355</v>
+        <v>159.323</v>
       </c>
       <c r="G13" s="9" t="n"/>
       <c r="H13" s="9" t="n"/>
@@ -2505,13 +2515,13 @@
       </c>
       <c r="C14" s="9" t="n"/>
       <c r="D14" s="8" t="n">
-        <v>234.0405</v>
+        <v>237.2995</v>
       </c>
       <c r="E14" s="8" t="n">
-        <v>234.8675</v>
+        <v>238.5415</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>234.898</v>
+        <v>236.6625</v>
       </c>
       <c r="G14" s="9" t="n"/>
       <c r="H14" s="9" t="n"/>
@@ -2527,13 +2537,13 @@
       </c>
       <c r="C15" s="9" t="n"/>
       <c r="D15" s="8" t="n">
-        <v>57.9415</v>
+        <v>62.2325</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>58.4695</v>
+        <v>62.846</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>57.923</v>
+        <v>61.49</v>
       </c>
       <c r="G15" s="9" t="n"/>
       <c r="H15" s="9" t="n"/>
@@ -2549,13 +2559,13 @@
       </c>
       <c r="C16" s="9" t="n"/>
       <c r="D16" s="8" t="n">
-        <v>803.9135</v>
+        <v>828.6325000000001</v>
       </c>
       <c r="E16" s="8" t="n">
-        <v>1015.1315</v>
+        <v>1059.1705</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>692.117</v>
+        <v>702.6345</v>
       </c>
       <c r="G16" s="9" t="n"/>
       <c r="H16" s="9" t="n"/>
@@ -2575,18 +2585,22 @@
       </c>
       <c r="C17" s="9" t="n"/>
       <c r="D17" s="8" t="n">
-        <v>278.671</v>
+        <v>316.5755</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>321.4535</v>
+        <v>290.7215</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>281.5675</v>
-      </c>
-      <c r="G17" s="9" t="n"/>
+        <v>318.258</v>
+      </c>
+      <c r="G17" s="8" t="n">
+        <v>289.0415</v>
+      </c>
       <c r="H17" s="9" t="n"/>
       <c r="I17" s="9" t="n"/>
-      <c r="J17" s="9" t="n"/>
+      <c r="J17" s="8" t="n">
+        <v>297.051</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="11" t="n"/>
@@ -2597,18 +2611,22 @@
       </c>
       <c r="C18" s="9" t="n"/>
       <c r="D18" s="8" t="n">
-        <v>859.4335</v>
+        <v>901.6325000000001</v>
       </c>
       <c r="E18" s="8" t="n">
-        <v>2516.135</v>
+        <v>2465.5035</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>510.023</v>
-      </c>
-      <c r="G18" s="9" t="n"/>
+        <v>526.7</v>
+      </c>
+      <c r="G18" s="8" t="n">
+        <v>2631.059</v>
+      </c>
       <c r="H18" s="9" t="n"/>
       <c r="I18" s="9" t="n"/>
-      <c r="J18" s="9" t="n"/>
+      <c r="J18" s="8" t="n">
+        <v>2652.7555</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="11" t="n"/>
@@ -2619,18 +2637,22 @@
       </c>
       <c r="C19" s="9" t="n"/>
       <c r="D19" s="8" t="n">
-        <v>121.496</v>
+        <v>125.0115</v>
       </c>
       <c r="E19" s="8" t="n">
-        <v>127.102</v>
+        <v>124.5765</v>
       </c>
       <c r="F19" s="8" t="n">
-        <v>121.1895</v>
-      </c>
-      <c r="G19" s="9" t="n"/>
+        <v>125.8135</v>
+      </c>
+      <c r="G19" s="8" t="n">
+        <v>123.81</v>
+      </c>
       <c r="H19" s="9" t="n"/>
       <c r="I19" s="9" t="n"/>
-      <c r="J19" s="9" t="n"/>
+      <c r="J19" s="8" t="n">
+        <v>125.371</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="12" t="n"/>
@@ -2641,18 +2663,22 @@
       </c>
       <c r="C20" s="9" t="n"/>
       <c r="D20" s="8" t="n">
-        <v>1259.6405</v>
+        <v>1343.0815</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>2968.167</v>
+        <v>2880.6655</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>912.5085</v>
-      </c>
-      <c r="G20" s="9" t="n"/>
+        <v>971.0975</v>
+      </c>
+      <c r="G20" s="8" t="n">
+        <v>3043.593</v>
+      </c>
       <c r="H20" s="9" t="n"/>
       <c r="I20" s="9" t="n"/>
-      <c r="J20" s="9" t="n"/>
+      <c r="J20" s="8" t="n">
+        <v>3077.1495</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -2838,24 +2864,24 @@
         </is>
       </c>
       <c r="C27" s="8" t="n">
-        <v>109.632</v>
+        <v>108.436</v>
       </c>
       <c r="D27" s="8" t="n">
-        <v>33.3545</v>
+        <v>34.4515</v>
       </c>
       <c r="E27" s="8" t="n">
-        <v>19.9275</v>
+        <v>20.9445</v>
       </c>
       <c r="F27" s="8" t="n">
-        <v>10.497</v>
+        <v>11.2175</v>
       </c>
       <c r="G27" s="8" t="n">
-        <v>62.5325</v>
+        <v>62.574</v>
       </c>
       <c r="H27" s="9" t="n"/>
       <c r="I27" s="9" t="n"/>
       <c r="J27" s="8" t="n">
-        <v>69.587</v>
+        <v>69.56999999999999</v>
       </c>
     </row>
     <row r="28">
@@ -2866,24 +2892,24 @@
         </is>
       </c>
       <c r="C28" s="8" t="n">
-        <v>77.4085</v>
+        <v>79.1005</v>
       </c>
       <c r="D28" s="8" t="n">
-        <v>82.6675</v>
+        <v>83.52800000000001</v>
       </c>
       <c r="E28" s="8" t="n">
-        <v>79.4935</v>
+        <v>79.973</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>78.181</v>
+        <v>79.57550000000001</v>
       </c>
       <c r="G28" s="8" t="n">
-        <v>79.033</v>
+        <v>78.408</v>
       </c>
       <c r="H28" s="9" t="n"/>
       <c r="I28" s="9" t="n"/>
       <c r="J28" s="8" t="n">
-        <v>78.62649999999999</v>
+        <v>79.87050000000001</v>
       </c>
     </row>
     <row r="29">
@@ -2894,24 +2920,24 @@
         </is>
       </c>
       <c r="C29" s="8" t="n">
-        <v>88.92</v>
+        <v>89.8605</v>
       </c>
       <c r="D29" s="8" t="n">
-        <v>89.3</v>
+        <v>90.069</v>
       </c>
       <c r="E29" s="8" t="n">
-        <v>88.7535</v>
+        <v>89.125</v>
       </c>
       <c r="F29" s="8" t="n">
-        <v>88.01349999999999</v>
+        <v>88.8445</v>
       </c>
       <c r="G29" s="8" t="n">
-        <v>90.7225</v>
+        <v>88.27800000000001</v>
       </c>
       <c r="H29" s="9" t="n"/>
       <c r="I29" s="9" t="n"/>
       <c r="J29" s="8" t="n">
-        <v>89.8925</v>
+        <v>95.7235</v>
       </c>
     </row>
     <row r="30">
@@ -2922,24 +2948,24 @@
         </is>
       </c>
       <c r="C30" s="8" t="n">
-        <v>275.8775</v>
+        <v>277.389</v>
       </c>
       <c r="D30" s="8" t="n">
-        <v>205.407</v>
+        <v>207.964</v>
       </c>
       <c r="E30" s="8" t="n">
-        <v>188.3935</v>
+        <v>190.287</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>176.6925</v>
+        <v>179.7225</v>
       </c>
       <c r="G30" s="8" t="n">
-        <v>232.1375</v>
+        <v>229.2315</v>
       </c>
       <c r="H30" s="9" t="n"/>
       <c r="I30" s="9" t="n"/>
       <c r="J30" s="8" t="n">
-        <v>238.1145</v>
+        <v>245.095</v>
       </c>
     </row>
     <row r="31">
@@ -3053,20 +3079,26 @@
           <t>PhaseA_part</t>
         </is>
       </c>
-      <c r="C34" s="9" t="n"/>
+      <c r="C34" s="8" t="n">
+        <v>443.5375</v>
+      </c>
       <c r="D34" s="8" t="n">
-        <v>41.7295</v>
+        <v>35.6085</v>
       </c>
       <c r="E34" s="8" t="n">
-        <v>32.1285</v>
+        <v>32.076</v>
       </c>
       <c r="F34" s="8" t="n">
-        <v>30.4145</v>
-      </c>
-      <c r="G34" s="9" t="n"/>
+        <v>32.1655</v>
+      </c>
+      <c r="G34" s="8" t="n">
+        <v>468.0265</v>
+      </c>
       <c r="H34" s="9" t="n"/>
       <c r="I34" s="9" t="n"/>
-      <c r="J34" s="9" t="n"/>
+      <c r="J34" s="8" t="n">
+        <v>515.859</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="11" t="n"/>
@@ -3075,20 +3107,26 @@
           <t>PhaseB_avg</t>
         </is>
       </c>
-      <c r="C35" s="9" t="n"/>
+      <c r="C35" s="8" t="n">
+        <v>23.5965</v>
+      </c>
       <c r="D35" s="8" t="n">
-        <v>20.3075</v>
+        <v>20.3655</v>
       </c>
       <c r="E35" s="8" t="n">
-        <v>19.295</v>
+        <v>19.269</v>
       </c>
       <c r="F35" s="8" t="n">
-        <v>17.963</v>
-      </c>
-      <c r="G35" s="9" t="n"/>
+        <v>19.7855</v>
+      </c>
+      <c r="G35" s="8" t="n">
+        <v>26.008</v>
+      </c>
       <c r="H35" s="9" t="n"/>
       <c r="I35" s="9" t="n"/>
-      <c r="J35" s="9" t="n"/>
+      <c r="J35" s="8" t="n">
+        <v>23.949</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="11" t="n"/>
@@ -3097,20 +3135,26 @@
           <t>PhaseC_sum</t>
         </is>
       </c>
-      <c r="C36" s="9" t="n"/>
+      <c r="C36" s="8" t="n">
+        <v>0.919</v>
+      </c>
       <c r="D36" s="8" t="n">
-        <v>1.071</v>
+        <v>1.023</v>
       </c>
       <c r="E36" s="8" t="n">
-        <v>0.977</v>
+        <v>0.987</v>
       </c>
       <c r="F36" s="8" t="n">
-        <v>0.9370000000000001</v>
-      </c>
-      <c r="G36" s="9" t="n"/>
+        <v>0.975</v>
+      </c>
+      <c r="G36" s="8" t="n">
+        <v>1.186</v>
+      </c>
       <c r="H36" s="9" t="n"/>
       <c r="I36" s="9" t="n"/>
-      <c r="J36" s="9" t="n"/>
+      <c r="J36" s="8" t="n">
+        <v>0.9325</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="12" t="n"/>
@@ -3119,20 +3163,26 @@
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C37" s="9" t="n"/>
+      <c r="C37" s="8" t="n">
+        <v>468.0545</v>
+      </c>
       <c r="D37" s="8" t="n">
-        <v>63.095</v>
+        <v>56.996</v>
       </c>
       <c r="E37" s="8" t="n">
-        <v>52.4</v>
+        <v>52.332</v>
       </c>
       <c r="F37" s="8" t="n">
-        <v>49.318</v>
-      </c>
-      <c r="G37" s="9" t="n"/>
+        <v>52.9235</v>
+      </c>
+      <c r="G37" s="8" t="n">
+        <v>495.2225</v>
+      </c>
       <c r="H37" s="9" t="n"/>
       <c r="I37" s="9" t="n"/>
-      <c r="J37" s="9" t="n"/>
+      <c r="J37" s="8" t="n">
+        <v>540.683</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -4840,15 +4890,27 @@
           <t>Q12</t>
         </is>
       </c>
-      <c r="B9" s="17" t="n"/>
-      <c r="C9" s="17" t="n"/>
-      <c r="D9" s="17" t="n"/>
-      <c r="E9" s="17" t="n"/>
-      <c r="F9" s="17" t="n"/>
+      <c r="B9" s="16" t="n">
+        <v>101.8691584</v>
+      </c>
+      <c r="C9" s="16" t="n">
+        <v>105.70694656</v>
+      </c>
+      <c r="D9" s="16" t="n">
+        <v>50.91885056</v>
+      </c>
+      <c r="E9" s="16" t="n">
+        <v>50.91885056</v>
+      </c>
+      <c r="F9" s="16" t="n">
+        <v>169.869312</v>
+      </c>
       <c r="G9" s="17" t="n"/>
       <c r="H9" s="17" t="n"/>
       <c r="I9" s="17" t="n"/>
-      <c r="J9" s="15" t="n"/>
+      <c r="J9" s="15" t="n">
+        <v>428.36</v>
+      </c>
       <c r="K9" s="15" t="n"/>
       <c r="L9" t="inlineStr"/>
     </row>
@@ -5250,7 +5312,9 @@
           <t>Q17</t>
         </is>
       </c>
-      <c r="B12" s="18" t="n"/>
+      <c r="B12" s="20" t="n">
+        <v>61385</v>
+      </c>
       <c r="C12" s="18" t="n"/>
       <c r="D12" s="18" t="n"/>
       <c r="E12" s="18" t="n"/>

</xml_diff>

<commit_message>
bench_suite: parse [load_bitmap] lines for per-column memory breakdown
</commit_message>
<xml_diff>
--- a/bm_resultL4.xlsx
+++ b/bm_resultL4.xlsx
@@ -173,10 +173,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -3806,14 +3806,14 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="21" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -3863,7 +3863,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="36" customHeight="1">
+    <row r="2" ht="62" customHeight="1">
       <c r="A2" s="7" t="inlineStr">
         <is>
           <t>Q1</t>
@@ -3871,87 +3871,111 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
+          <t>shipdate: 467.13 MB
+linestatus: 15.48 MB
+returnflag: 23.22 MB
+total: 505.83 MB</t>
+        </is>
+      </c>
+      <c r="C2" s="13" t="inlineStr">
+        <is>
+          <t>shipdate: 6586.64 MB
+linestatus: 20.63 MB
+returnflag: 29.78 MB
+total: 6637.05 MB</t>
+        </is>
+      </c>
+      <c r="D2" s="13" t="inlineStr">
+        <is>
+          <t>shipdate: 138.44 MB
+linestatus: 15.02 MB
+returnflag: 22.53 MB
+total: 176.00 MB</t>
+        </is>
+      </c>
+      <c r="E2" s="13" t="inlineStr">
+        <is>
+          <t>shipdate: 138.44 MB
+linestatus: 15.02 MB
+returnflag: 22.53 MB
+total: 175.99 MB</t>
+        </is>
+      </c>
+      <c r="F2" s="13" t="inlineStr">
+        <is>
+          <t>shipdate: 921.39 MB
+linestatus: 15.00 MB
+returnflag: 22.49 MB
+total: 958.88 MB</t>
+        </is>
+      </c>
+      <c r="G2" s="14" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C2" s="13" t="inlineStr">
+      <c r="H2" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D2" s="13" t="inlineStr">
+      <c r="I2" s="13" t="inlineStr">
+        <is>
+          <t>shipdate: 239.94 MB
+linestatus: 239.94 MB
+returnflag: 239.94 MB
+total: 719.83 MB</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="48" customHeight="1">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E2" s="13" t="inlineStr">
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>orderkey: 4448.84 MB
+shipdate: 6586.64 MB
+total: 11035.48 MB</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>orderkey: 359.98 MB
+shipdate: 138.44 MB
+total: 498.42 MB</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>orderkey: 257.15 MB
+shipdate: 138.44 MB
+total: 395.60 MB</t>
+        </is>
+      </c>
+      <c r="F3" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F2" s="13" t="inlineStr">
+      <c r="G3" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G2" s="13" t="inlineStr">
+      <c r="H3" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H2" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I2" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="36" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C3" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D3" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E3" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F3" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G3" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H3" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I3" s="13" t="inlineStr">
+      <c r="I3" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3963,138 +3987,173 @@
           <t>Q4</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
+          <t>orderkey: 4448.84 MB
+total: 4448.84 MB</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>orderkey: 359.98 MB
+total: 359.98 MB</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="inlineStr">
+        <is>
+          <t>orderkey: 257.15 MB
+total: 257.15 MB</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D4" s="13" t="inlineStr">
+      <c r="G4" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E4" s="13" t="inlineStr">
+      <c r="H4" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F4" s="13" t="inlineStr">
+      <c r="I4" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G4" s="13" t="inlineStr">
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Q5</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H4" s="13" t="inlineStr">
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>orderkey: 4448.84 MB
+suppkey: 13176.00 MB
+total: 17624.84 MB</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>orderkey: 359.98 MB
+suppkey: 472.84 MB
+total: 832.81 MB</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>orderkey: 257.15 MB
+suppkey: 472.84 MB
+total: 729.99 MB</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>orderkey: 365.62 MB
+suppkey: 959.97 MB
+total: 1325.59 MB</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I4" s="13" t="inlineStr">
+      <c r="H5" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-    </row>
-    <row r="5" ht="36" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>Q5</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="I5" s="13" t="inlineStr">
+        <is>
+          <t>orderkey: 239.94 MB
+suppkey: 239.94 MB
+total: 479.89 MB</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="90" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Q6</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>shipdate_GE: 50.85 MB
+discount: 84.91 MB
+quantity: 276.43 MB
+total: 412.19 MB</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>shipdate_GE: 48.83 MB
+discount: 89.91 MB
+quantity: 257.20 MB
+discount_BPE: 79.93 MB
+quantity_BPE: 79.58 MB
+total: 555.45 MB</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>shipdate_GE: 52.56 MB
+discount: 82.57 MB
+quantity: 120.34 MB
+discount_BPE: 150.25 MB
+quantity_BPE: 154.94 MB
+total: 560.67 MB</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>shipdate_GE: 52.52 MB
+discount: 82.57 MB
+quantity: 120.34 MB
+total: 255.43 MB</t>
+        </is>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
+        <is>
+          <t>shipdate_GE: 52.26 MB
+discount: 82.48 MB
+quantity: 346.69 MB
+total: 481.44 MB</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C5" s="13" t="inlineStr">
+      <c r="H6" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D5" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E5" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F5" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G5" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H5" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I5" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>Q6</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C6" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E6" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F6" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G6" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H6" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="I6" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>shipdate_GE: 239.94 MB
+discount: 239.94 MB
+quantity: 239.94 MB
+total: 719.83 MB</t>
         </is>
       </c>
     </row>
@@ -4104,42 +4163,42 @@
           <t>Q8</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C7" s="13" t="inlineStr">
+      <c r="C7" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D7" s="13" t="inlineStr">
+      <c r="D7" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E7" s="13" t="inlineStr">
+      <c r="E7" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F7" s="13" t="inlineStr">
+      <c r="F7" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G7" s="13" t="inlineStr">
+      <c r="G7" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H7" s="13" t="inlineStr">
+      <c r="H7" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I7" s="13" t="inlineStr">
+      <c r="I7" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4151,42 +4210,42 @@
           <t>Q10</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C8" s="13" t="inlineStr">
+      <c r="C8" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D8" s="13" t="inlineStr">
+      <c r="D8" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E8" s="13" t="inlineStr">
+      <c r="E8" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F8" s="13" t="inlineStr">
+      <c r="F8" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G8" s="13" t="inlineStr">
+      <c r="G8" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H8" s="13" t="inlineStr">
+      <c r="H8" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I8" s="13" t="inlineStr">
+      <c r="I8" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4198,42 +4257,42 @@
           <t>Q12</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
+      <c r="C9" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D9" s="13" t="inlineStr">
+      <c r="D9" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E9" s="13" t="inlineStr">
+      <c r="E9" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F9" s="13" t="inlineStr">
+      <c r="F9" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G9" s="13" t="inlineStr">
+      <c r="G9" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H9" s="13" t="inlineStr">
+      <c r="H9" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I9" s="13" t="inlineStr">
+      <c r="I9" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4247,42 +4306,48 @@
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
+          <t>shipdate: 467.13 MB
+total: 467.13 MB</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>shipdate: 6586.64 MB
+total: 6586.64 MB</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>shipdate: 138.44 MB
+total: 138.44 MB</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>shipdate: 138.44 MB
+total: 138.44 MB</t>
+        </is>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>shipdate: 921.39 MB
+total: 921.39 MB</t>
+        </is>
+      </c>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C10" s="13" t="inlineStr">
+      <c r="H10" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D10" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E10" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F10" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G10" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H10" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="I10" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>shipdate: 239.94 MB
+total: 239.94 MB</t>
         </is>
       </c>
     </row>
@@ -4292,12 +4357,12 @@
           <t>Q15</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B11" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C11" s="14" t="inlineStr">
+      <c r="C11" s="13" t="inlineStr">
         <is>
           <t>L1: 2.23 MB
 L2: 2.20 MB
@@ -4306,32 +4371,32 @@
 total: 7.79 MB</t>
         </is>
       </c>
-      <c r="D11" s="13" t="inlineStr">
+      <c r="D11" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E11" s="13" t="inlineStr">
+      <c r="E11" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F11" s="13" t="inlineStr">
+      <c r="F11" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G11" s="13" t="inlineStr">
+      <c r="G11" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H11" s="13" t="inlineStr">
+      <c r="H11" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I11" s="13" t="inlineStr">
+      <c r="I11" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4345,89 +4410,107 @@
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
+          <t>partkey: 631.88 MB
+total: 631.88 MB</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>partkey: 13567.30 MB
+total: 13567.30 MB</t>
+        </is>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>partkey: 608.09 MB
+total: 608.09 MB</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>partkey: 608.09 MB
+total: 608.09 MB</t>
+        </is>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>partkey: 975.75 MB
+total: 975.75 MB</t>
+        </is>
+      </c>
+      <c r="G12" s="14" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C12" s="13" t="inlineStr">
+      <c r="H12" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D12" s="13" t="inlineStr">
+      <c r="I12" s="13" t="inlineStr">
+        <is>
+          <t>partkey: 239.94 MB
+total: 239.94 MB</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Q19</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>shipmode: 46.44 MB
+shipinstruct: 30.96 MB
+total: 77.40 MB</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>shipmode: 58.13 MB
+shipinstruct: 42.54 MB
+total: 100.66 MB</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>shipmode: 45.06 MB
+shipinstruct: 30.04 MB
+total: 75.10 MB</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>shipmode: 45.06 MB
+shipinstruct: 30.04 MB
+total: 75.10 MB</t>
+        </is>
+      </c>
+      <c r="F13" s="13" t="inlineStr">
+        <is>
+          <t>shipmode: 44.99 MB
+shipinstruct: 29.99 MB
+total: 74.98 MB</t>
+        </is>
+      </c>
+      <c r="G13" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E12" s="13" t="inlineStr">
+      <c r="H13" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F12" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G12" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H12" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I12" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="36" customHeight="1">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>Q19</t>
-        </is>
-      </c>
-      <c r="B13" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C13" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D13" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E13" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F13" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G13" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H13" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="I13" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>shipmode: 239.94 MB
+shipinstruct: 239.94 MB
+total: 479.89 MB</t>
         </is>
       </c>
     </row>
@@ -4442,14 +4525,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -4482,32 +4565,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Q15</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>WAH</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ComBit</t>
+          <t>WAH (FastBit)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>total</t>
         </is>
       </c>
       <c r="E2" s="15" t="n">
-        <v>2.23346688</v>
+        <v>505.8297</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Q15</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -4522,86 +4605,1111 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>total</t>
         </is>
       </c>
       <c r="E3" s="15" t="n">
-        <v>2.2020096</v>
+        <v>6637.049</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Q15</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ComBit</t>
+          <t>CRoaring</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>L3</t>
+          <t>total</t>
         </is>
       </c>
       <c r="E4" s="15" t="n">
-        <v>2.01326592</v>
+        <v>175.999</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Q15</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>CRR</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ComBit</t>
+          <t>CRoaring+Run</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>L4</t>
+          <t>total</t>
         </is>
       </c>
       <c r="E5" s="15" t="n">
-        <v>1.33169152</v>
+        <v>175.9916</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>EW</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>EWAH</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E6" s="15" t="n">
+        <v>958.8793000000001</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>CON</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Concise</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="n">
+        <v>719.832</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ComBit</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E8" s="15" t="n">
+        <v>11035.48</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CRoaring</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="n">
+        <v>498.421</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CRR</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CRoaring+Run</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E10" s="15" t="n">
+        <v>395.597</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ComBit</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="n">
+        <v>4448.84</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>CRoaring</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E12" s="15" t="n">
+        <v>359.978</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>CRR</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>CRoaring+Run</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="n">
+        <v>257.154</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Q5</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>ComBit</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E14" s="15" t="n">
+        <v>17624.84</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Q5</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>CRoaring</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="n">
+        <v>832.8140000000001</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Q5</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>CRR</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>CRoaring+Run</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E16" s="15" t="n">
+        <v>729.99</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Q5</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>EW</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>EWAH</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="n">
+        <v>1325.591</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Q5</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>CON</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Concise</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E18" s="15" t="n">
+        <v>479.888</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Q6</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>WAH</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>WAH (FastBit)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="n">
+        <v>412.1922</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Q6</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>ComBit</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E20" s="15" t="n">
+        <v>555.4544000000001</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Q6</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>CRoaring</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E21" s="15" t="n">
+        <v>560.6653</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Q6</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>CRR</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>CRoaring+Run</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E22" s="15" t="n">
+        <v>255.4297</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Q6</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>EW</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>EWAH</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E23" s="15" t="n">
+        <v>481.4368</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Q6</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>CON</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Concise</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E24" s="15" t="n">
+        <v>719.832</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Q14</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>WAH</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>WAH (FastBit)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E25" s="15" t="n">
+        <v>467.132</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Q14</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>ComBit</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E26" s="15" t="n">
+        <v>6586.64</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Q14</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>CRoaring</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E27" s="15" t="n">
+        <v>138.443</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Q14</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>CRR</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>CRoaring+Run</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E28" s="15" t="n">
+        <v>138.443</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Q14</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>EW</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>EWAH</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E29" s="15" t="n">
+        <v>921.388</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Q14</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>CON</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Concise</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E30" s="15" t="n">
+        <v>239.944</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>Q15</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>CB</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>ComBit</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="E31" s="15" t="n">
+        <v>2.23346688</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Q15</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>ComBit</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="E32" s="15" t="n">
+        <v>2.2020096</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Q15</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>ComBit</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="E33" s="15" t="n">
+        <v>2.01326592</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Q15</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>ComBit</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="E34" s="15" t="n">
+        <v>1.33169152</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Q15</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>ComBit</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
         <is>
           <t>total</t>
         </is>
       </c>
-      <c r="E6" s="15" t="n">
+      <c r="E35" s="15" t="n">
         <v>7.790919679999999</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Q17</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>WAH</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>WAH (FastBit)</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E36" s="15" t="n">
+        <v>631.881</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Q17</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>ComBit</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E37" s="15" t="n">
+        <v>13567.3</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Q17</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>CRoaring</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E38" s="15" t="n">
+        <v>608.0890000000001</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Q17</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>CRR</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>CRoaring+Run</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E39" s="15" t="n">
+        <v>608.0890000000001</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Q17</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>EW</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>EWAH</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E40" s="15" t="n">
+        <v>975.746</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Q17</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>CON</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Concise</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E41" s="15" t="n">
+        <v>239.944</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Q19</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>WAH</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>WAH (FastBit)</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E42" s="15" t="n">
+        <v>77.3993</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Q19</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>ComBit</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E43" s="15" t="n">
+        <v>100.6633</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Q19</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>CRoaring</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E44" s="15" t="n">
+        <v>75.1007</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Q19</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>CRR</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>CRoaring+Run</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E45" s="15" t="n">
+        <v>75.1007</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Q19</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>EW</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>EWAH</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E46" s="15" t="n">
+        <v>74.98269999999999</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Q19</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>CON</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Concise</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E47" s="15" t="n">
+        <v>479.888</v>
       </c>
     </row>
   </sheetData>
@@ -4701,26 +5809,26 @@
         </is>
       </c>
       <c r="B2" s="16" t="n">
-        <v>505.667627</v>
+        <v>505.8297</v>
       </c>
       <c r="C2" s="16" t="n">
-        <v>566.155143</v>
+        <v>6637.049</v>
       </c>
       <c r="D2" s="16" t="n">
-        <v>176.009407</v>
+        <v>175.999</v>
       </c>
       <c r="E2" s="16" t="n">
-        <v>176.009407</v>
+        <v>175.9916</v>
       </c>
       <c r="F2" s="16" t="n">
-        <v>958.920363</v>
+        <v>958.8793000000001</v>
       </c>
       <c r="G2" s="17" t="n"/>
       <c r="H2" s="17" t="n"/>
-      <c r="I2" s="17" t="n"/>
-      <c r="J2" s="15" t="n">
-        <v>2206.75</v>
-      </c>
+      <c r="I2" s="16" t="n">
+        <v>719.832</v>
+      </c>
+      <c r="J2" s="15" t="n"/>
       <c r="K2" s="15" t="n"/>
       <c r="L2" t="inlineStr"/>
     </row>
@@ -4734,13 +5842,13 @@
         <v>466.970216</v>
       </c>
       <c r="C3" s="16" t="n">
-        <v>531.5854949999999</v>
+        <v>11035.48</v>
       </c>
       <c r="D3" s="16" t="n">
-        <v>138.453312</v>
+        <v>498.421</v>
       </c>
       <c r="E3" s="16" t="n">
-        <v>138.453312</v>
+        <v>395.597</v>
       </c>
       <c r="F3" s="16" t="n">
         <v>921.428872</v>
@@ -4749,7 +5857,7 @@
       <c r="H3" s="17" t="n"/>
       <c r="I3" s="17" t="n"/>
       <c r="J3" s="15" t="n">
-        <v>2058.44</v>
+        <v>1388.4</v>
       </c>
       <c r="K3" s="15" t="n"/>
       <c r="L3" t="inlineStr">
@@ -4768,13 +5876,13 @@
         <v>14.210456</v>
       </c>
       <c r="C4" s="16" t="n">
-        <v>13.821317</v>
+        <v>4448.84</v>
       </c>
       <c r="D4" s="16" t="n">
-        <v>10.70605</v>
+        <v>359.978</v>
       </c>
       <c r="E4" s="16" t="n">
-        <v>10.70605</v>
+        <v>257.154</v>
       </c>
       <c r="F4" s="16" t="n">
         <v>18.318512</v>
@@ -4783,7 +5891,7 @@
       <c r="H4" s="17" t="n"/>
       <c r="I4" s="17" t="n"/>
       <c r="J4" s="15" t="n">
-        <v>57.06</v>
+        <v>32.53</v>
       </c>
       <c r="K4" s="15" t="n"/>
       <c r="L4" t="inlineStr"/>
@@ -4798,20 +5906,22 @@
         <v>0.000125</v>
       </c>
       <c r="C5" s="16" t="n">
-        <v>6.7e-05</v>
+        <v>17624.84</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>0.000125</v>
+        <v>832.8140000000001</v>
       </c>
       <c r="E5" s="16" t="n">
-        <v>0.000125</v>
+        <v>729.99</v>
       </c>
       <c r="F5" s="16" t="n">
-        <v>0.000125</v>
+        <v>1325.591</v>
       </c>
       <c r="G5" s="17" t="n"/>
       <c r="H5" s="17" t="n"/>
-      <c r="I5" s="17" t="n"/>
+      <c r="I5" s="16" t="n">
+        <v>479.888</v>
+      </c>
       <c r="J5" s="15" t="n">
         <v>0</v>
       </c>
@@ -4825,26 +5935,26 @@
         </is>
       </c>
       <c r="B6" s="16" t="n">
-        <v>828.3056439999999</v>
+        <v>412.1922</v>
       </c>
       <c r="C6" s="16" t="n">
-        <v>685.775345</v>
+        <v>555.4544000000001</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>341.366933</v>
+        <v>560.6653</v>
       </c>
       <c r="E6" s="16" t="n">
-        <v>341.366933</v>
+        <v>255.4297</v>
       </c>
       <c r="F6" s="16" t="n">
-        <v>1350.602814</v>
+        <v>481.4368</v>
       </c>
       <c r="G6" s="17" t="n"/>
       <c r="H6" s="17" t="n"/>
-      <c r="I6" s="17" t="n"/>
-      <c r="J6" s="15" t="n">
-        <v>3206.05</v>
-      </c>
+      <c r="I6" s="16" t="n">
+        <v>719.832</v>
+      </c>
+      <c r="J6" s="15" t="n"/>
       <c r="K6" s="15" t="n"/>
       <c r="L6" t="inlineStr"/>
     </row>
@@ -4921,32 +6031,28 @@
         </is>
       </c>
       <c r="B10" s="16" t="n">
-        <v>466.970216</v>
+        <v>467.132</v>
       </c>
       <c r="C10" s="16" t="n">
-        <v>531.5854949999999</v>
+        <v>6586.64</v>
       </c>
       <c r="D10" s="16" t="n">
-        <v>138.453312</v>
+        <v>138.443</v>
       </c>
       <c r="E10" s="16" t="n">
-        <v>138.453312</v>
+        <v>138.443</v>
       </c>
       <c r="F10" s="16" t="n">
-        <v>921.428872</v>
+        <v>921.388</v>
       </c>
       <c r="G10" s="17" t="n"/>
       <c r="H10" s="17" t="n"/>
-      <c r="I10" s="17" t="n"/>
-      <c r="J10" s="15" t="n">
-        <v>2058.44</v>
-      </c>
+      <c r="I10" s="16" t="n">
+        <v>239.944</v>
+      </c>
+      <c r="J10" s="15" t="n"/>
       <c r="K10" s="15" t="n"/>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>symlinked share with another Q</t>
-        </is>
-      </c>
+      <c r="L10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -4989,26 +6095,26 @@
         </is>
       </c>
       <c r="B12" s="16" t="n">
-        <v>1.8e-05</v>
+        <v>631.881</v>
       </c>
       <c r="C12" s="16" t="n">
-        <v>1.8e-05</v>
+        <v>13567.3</v>
       </c>
       <c r="D12" s="16" t="n">
-        <v>1.8e-05</v>
+        <v>608.0890000000001</v>
       </c>
       <c r="E12" s="16" t="n">
-        <v>1.8e-05</v>
+        <v>608.0890000000001</v>
       </c>
       <c r="F12" s="16" t="n">
-        <v>1.8e-05</v>
+        <v>975.746</v>
       </c>
       <c r="G12" s="17" t="n"/>
       <c r="H12" s="17" t="n"/>
-      <c r="I12" s="17" t="n"/>
-      <c r="J12" s="15" t="n">
-        <v>0</v>
-      </c>
+      <c r="I12" s="16" t="n">
+        <v>239.944</v>
+      </c>
+      <c r="J12" s="15" t="n"/>
       <c r="K12" s="15" t="n"/>
       <c r="L12" t="inlineStr"/>
     </row>
@@ -5019,32 +6125,28 @@
         </is>
       </c>
       <c r="B13" s="16" t="n">
-        <v>291.905662</v>
+        <v>77.3993</v>
       </c>
       <c r="C13" s="16" t="n">
-        <v>111.947199</v>
+        <v>100.6633</v>
       </c>
       <c r="D13" s="16" t="n">
-        <v>135.35933</v>
+        <v>75.1007</v>
       </c>
       <c r="E13" s="16" t="n">
-        <v>135.35933</v>
+        <v>75.1007</v>
       </c>
       <c r="F13" s="16" t="n">
-        <v>361.689698</v>
+        <v>74.98269999999999</v>
       </c>
       <c r="G13" s="17" t="n"/>
       <c r="H13" s="17" t="n"/>
-      <c r="I13" s="17" t="n"/>
-      <c r="J13" s="15" t="n">
-        <v>900.9</v>
-      </c>
+      <c r="I13" s="16" t="n">
+        <v>479.888</v>
+      </c>
+      <c r="J13" s="15" t="n"/>
       <c r="K13" s="15" t="n"/>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>symlinked share with another Q</t>
-        </is>
-      </c>
+      <c r="L13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
bm_resultL4.xlsx: full 12-Q × 6-backend bench at SF10
</commit_message>
<xml_diff>
--- a/bm_resultL4.xlsx
+++ b/bm_resultL4.xlsx
@@ -1699,24 +1699,24 @@
         </is>
       </c>
       <c r="B2" s="8" t="n">
-        <v>2044.4535</v>
+        <v>2028.102</v>
       </c>
       <c r="C2" s="8" t="n">
-        <v>1027.2135</v>
+        <v>1001.4835</v>
       </c>
       <c r="D2" s="8" t="n">
-        <v>1604.152</v>
+        <v>1579.266</v>
       </c>
       <c r="E2" s="8" t="n">
-        <v>1580.9035</v>
+        <v>1552.726</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>1251.543</v>
+        <v>1273.0575</v>
       </c>
       <c r="G2" s="9" t="n"/>
       <c r="H2" s="9" t="n"/>
       <c r="I2" s="8" t="n">
-        <v>1295.5445</v>
+        <v>1290.693</v>
       </c>
       <c r="J2" s="9" t="n"/>
     </row>
@@ -1726,20 +1726,26 @@
           <t>Q3</t>
         </is>
       </c>
-      <c r="B3" s="9" t="n"/>
+      <c r="B3" s="8" t="n">
+        <v>3567.423</v>
+      </c>
       <c r="C3" s="8" t="n">
-        <v>2311.252</v>
+        <v>2335.4595</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>2817.675</v>
+        <v>1653.717</v>
       </c>
       <c r="E3" s="8" t="n">
-        <v>4330.24</v>
-      </c>
-      <c r="F3" s="9" t="n"/>
+        <v>1379.7845</v>
+      </c>
+      <c r="F3" s="8" t="n">
+        <v>4120.672</v>
+      </c>
       <c r="G3" s="9" t="n"/>
       <c r="H3" s="9" t="n"/>
-      <c r="I3" s="9" t="n"/>
+      <c r="I3" s="8" t="n">
+        <v>4953.748</v>
+      </c>
       <c r="J3" s="9" t="n"/>
     </row>
     <row r="4">
@@ -1748,20 +1754,26 @@
           <t>Q4</t>
         </is>
       </c>
-      <c r="B4" s="9" t="n"/>
+      <c r="B4" s="8" t="n">
+        <v>1353.263</v>
+      </c>
       <c r="C4" s="8" t="n">
-        <v>828.6325000000001</v>
+        <v>814.4745</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>1059.1705</v>
+        <v>1074.3785</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>702.6345</v>
-      </c>
-      <c r="F4" s="9" t="n"/>
+        <v>703.89</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>897.4485</v>
+      </c>
       <c r="G4" s="9" t="n"/>
       <c r="H4" s="9" t="n"/>
-      <c r="I4" s="9" t="n"/>
+      <c r="I4" s="8" t="n">
+        <v>977.87</v>
+      </c>
       <c r="J4" s="9" t="n"/>
     </row>
     <row r="5">
@@ -1770,23 +1782,25 @@
           <t>Q5</t>
         </is>
       </c>
-      <c r="B5" s="9" t="n"/>
+      <c r="B5" s="8" t="n">
+        <v>3428.306</v>
+      </c>
       <c r="C5" s="8" t="n">
-        <v>1343.0815</v>
+        <v>1284.302</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>2880.6655</v>
+        <v>3029.9815</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>971.0975</v>
+        <v>961.7535</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>3043.593</v>
+        <v>2879.6125</v>
       </c>
       <c r="G5" s="9" t="n"/>
       <c r="H5" s="9" t="n"/>
       <c r="I5" s="8" t="n">
-        <v>3077.1495</v>
+        <v>3036.581</v>
       </c>
       <c r="J5" s="9" t="n"/>
     </row>
@@ -1797,24 +1811,24 @@
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>140.076</v>
+        <v>134.332</v>
       </c>
       <c r="C6" s="8" t="n">
-        <v>28.473</v>
+        <v>28.741</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>25.354</v>
+        <v>24.068</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>24.651</v>
+        <v>24.631</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>210.889</v>
+        <v>228.494</v>
       </c>
       <c r="G6" s="9" t="n"/>
       <c r="H6" s="9" t="n"/>
       <c r="I6" s="8" t="n">
-        <v>616.513</v>
+        <v>628.467</v>
       </c>
       <c r="J6" s="9" t="n"/>
     </row>
@@ -1824,14 +1838,26 @@
           <t>Q8</t>
         </is>
       </c>
-      <c r="B7" s="9" t="n"/>
-      <c r="C7" s="9" t="n"/>
-      <c r="D7" s="9" t="n"/>
-      <c r="E7" s="9" t="n"/>
-      <c r="F7" s="9" t="n"/>
+      <c r="B7" s="8" t="n">
+        <v>1705.5285</v>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>795.7234999999999</v>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>954.004</v>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>932.015</v>
+      </c>
+      <c r="F7" s="8" t="n">
+        <v>1139.955</v>
+      </c>
       <c r="G7" s="9" t="n"/>
       <c r="H7" s="9" t="n"/>
-      <c r="I7" s="9" t="n"/>
+      <c r="I7" s="8" t="n">
+        <v>1241.548</v>
+      </c>
       <c r="J7" s="9" t="n"/>
     </row>
     <row r="8">
@@ -1840,14 +1866,26 @@
           <t>Q10</t>
         </is>
       </c>
-      <c r="B8" s="9" t="n"/>
-      <c r="C8" s="9" t="n"/>
-      <c r="D8" s="9" t="n"/>
-      <c r="E8" s="9" t="n"/>
-      <c r="F8" s="9" t="n"/>
+      <c r="B8" s="8" t="n">
+        <v>1069.076</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>512.638</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>602.7380000000001</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>570.16</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>612.7025</v>
+      </c>
       <c r="G8" s="9" t="n"/>
       <c r="H8" s="9" t="n"/>
-      <c r="I8" s="9" t="n"/>
+      <c r="I8" s="8" t="n">
+        <v>700.9105</v>
+      </c>
       <c r="J8" s="9" t="n"/>
     </row>
     <row r="9">
@@ -1856,14 +1894,26 @@
           <t>Q12</t>
         </is>
       </c>
-      <c r="B9" s="9" t="n"/>
-      <c r="C9" s="9" t="n"/>
-      <c r="D9" s="9" t="n"/>
-      <c r="E9" s="9" t="n"/>
-      <c r="F9" s="9" t="n"/>
+      <c r="B9" s="8" t="n">
+        <v>1977.6165</v>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>1339.277</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>1292.08</v>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>1079.6835</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>2025.361</v>
+      </c>
       <c r="G9" s="9" t="n"/>
       <c r="H9" s="9" t="n"/>
-      <c r="I9" s="9" t="n"/>
+      <c r="I9" s="8" t="n">
+        <v>2192.618</v>
+      </c>
       <c r="J9" s="9" t="n"/>
     </row>
     <row r="10">
@@ -1873,24 +1923,24 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>277.389</v>
+        <v>277.701</v>
       </c>
       <c r="C10" s="8" t="n">
-        <v>207.964</v>
+        <v>208.468</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>190.287</v>
+        <v>189.4175</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>179.7225</v>
+        <v>182.1065</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>229.2315</v>
+        <v>230.836</v>
       </c>
       <c r="G10" s="9" t="n"/>
       <c r="H10" s="9" t="n"/>
       <c r="I10" s="8" t="n">
-        <v>245.095</v>
+        <v>239.195</v>
       </c>
       <c r="J10" s="9" t="n"/>
     </row>
@@ -1935,24 +1985,24 @@
         </is>
       </c>
       <c r="B12" s="8" t="n">
-        <v>468.0545</v>
+        <v>470.2065</v>
       </c>
       <c r="C12" s="8" t="n">
-        <v>56.996</v>
+        <v>57.8865</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>52.332</v>
+        <v>60.9555</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>52.9235</v>
+        <v>56.889</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>495.2225</v>
+        <v>485.102</v>
       </c>
       <c r="G12" s="9" t="n"/>
       <c r="H12" s="9" t="n"/>
       <c r="I12" s="8" t="n">
-        <v>540.683</v>
+        <v>537.5535</v>
       </c>
       <c r="J12" s="9" t="n"/>
     </row>
@@ -1963,24 +2013,24 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>269.872</v>
+        <v>269.1215</v>
       </c>
       <c r="C13" s="8" t="n">
-        <v>219.166</v>
+        <v>220.4715</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>212.2775</v>
+        <v>212.381</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>213.504</v>
+        <v>212.9095</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>239.8755</v>
+        <v>239.585</v>
       </c>
       <c r="G13" s="9" t="n"/>
       <c r="H13" s="9" t="n"/>
       <c r="I13" s="8" t="n">
-        <v>268.6065</v>
+        <v>268.818</v>
       </c>
       <c r="J13" s="9" t="n"/>
     </row>
@@ -2139,7 +2189,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:J60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2218,24 +2268,24 @@
         </is>
       </c>
       <c r="C2" s="8" t="n">
-        <v>247.5725</v>
+        <v>248.0305</v>
       </c>
       <c r="D2" s="8" t="n">
-        <v>41.586</v>
+        <v>42.0995</v>
       </c>
       <c r="E2" s="8" t="n">
-        <v>34.9445</v>
+        <v>37.9835</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>12.776</v>
+        <v>13.078</v>
       </c>
       <c r="G2" s="8" t="n">
-        <v>77.97750000000001</v>
+        <v>78.9965</v>
       </c>
       <c r="H2" s="9" t="n"/>
       <c r="I2" s="9" t="n"/>
       <c r="J2" s="8" t="n">
-        <v>85.383</v>
+        <v>90.9085</v>
       </c>
     </row>
     <row r="3">
@@ -2246,24 +2296,24 @@
         </is>
       </c>
       <c r="C3" s="8" t="n">
-        <v>993.2954999999999</v>
+        <v>1001.5955</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>179.1855</v>
+        <v>178.777</v>
       </c>
       <c r="E3" s="8" t="n">
-        <v>761.8680000000001</v>
+        <v>760.5645</v>
       </c>
       <c r="F3" s="8" t="n">
-        <v>760.7015</v>
+        <v>760.28</v>
       </c>
       <c r="G3" s="8" t="n">
-        <v>369.6275</v>
+        <v>416.8915</v>
       </c>
       <c r="H3" s="9" t="n"/>
       <c r="I3" s="9" t="n"/>
       <c r="J3" s="8" t="n">
-        <v>406.7575</v>
+        <v>420.956</v>
       </c>
     </row>
     <row r="4">
@@ -2274,24 +2324,24 @@
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>802.704</v>
+        <v>777.6145</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>806.5485</v>
+        <v>780.346</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>807.417</v>
+        <v>780.6685</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>806.58</v>
+        <v>779.6900000000001</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>804.423</v>
+        <v>777.2195</v>
       </c>
       <c r="H4" s="9" t="n"/>
       <c r="I4" s="9" t="n"/>
       <c r="J4" s="8" t="n">
-        <v>802.9745</v>
+        <v>778.778</v>
       </c>
     </row>
     <row r="5">
@@ -2302,24 +2352,24 @@
         </is>
       </c>
       <c r="C5" s="8" t="n">
-        <v>2044.4535</v>
+        <v>2028.102</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>1027.2135</v>
+        <v>1001.4835</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>1604.152</v>
+        <v>1579.266</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>1580.9035</v>
+        <v>1552.726</v>
       </c>
       <c r="G5" s="8" t="n">
-        <v>1251.543</v>
+        <v>1273.0575</v>
       </c>
       <c r="H5" s="9" t="n"/>
       <c r="I5" s="9" t="n"/>
       <c r="J5" s="8" t="n">
-        <v>1295.5445</v>
+        <v>1290.693</v>
       </c>
     </row>
     <row r="6">
@@ -2333,20 +2383,26 @@
           <t>PhaseA_cust</t>
         </is>
       </c>
-      <c r="C6" s="9" t="n"/>
+      <c r="C6" s="8" t="n">
+        <v>22.0545</v>
+      </c>
       <c r="D6" s="8" t="n">
-        <v>22.327</v>
+        <v>23.8995</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>22.917</v>
+        <v>22.397</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>23.222</v>
-      </c>
-      <c r="G6" s="9" t="n"/>
+        <v>22.1255</v>
+      </c>
+      <c r="G6" s="8" t="n">
+        <v>21.9745</v>
+      </c>
       <c r="H6" s="9" t="n"/>
       <c r="I6" s="9" t="n"/>
-      <c r="J6" s="9" t="n"/>
+      <c r="J6" s="8" t="n">
+        <v>22.0185</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="11" t="n"/>
@@ -2355,20 +2411,26 @@
           <t>PhaseB_okey</t>
         </is>
       </c>
-      <c r="C7" s="9" t="n"/>
+      <c r="C7" s="8" t="n">
+        <v>2192.3795</v>
+      </c>
       <c r="D7" s="8" t="n">
-        <v>1290.917</v>
+        <v>1297.014</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>2398.808</v>
+        <v>1205.36</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>4082.7515</v>
-      </c>
-      <c r="G7" s="9" t="n"/>
+        <v>1144.781</v>
+      </c>
+      <c r="G7" s="8" t="n">
+        <v>1091.6</v>
+      </c>
       <c r="H7" s="9" t="n"/>
       <c r="I7" s="9" t="n"/>
-      <c r="J7" s="9" t="n"/>
+      <c r="J7" s="8" t="n">
+        <v>1208.4175</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="n"/>
@@ -2377,20 +2439,26 @@
           <t>PhaseC_ship</t>
         </is>
       </c>
-      <c r="C8" s="9" t="n"/>
+      <c r="C8" s="8" t="n">
+        <v>1255.111</v>
+      </c>
       <c r="D8" s="8" t="n">
-        <v>908.941</v>
+        <v>923.3945</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>307.9585</v>
+        <v>337.6395</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>129.2175</v>
-      </c>
-      <c r="G8" s="9" t="n"/>
+        <v>124.2565</v>
+      </c>
+      <c r="G8" s="8" t="n">
+        <v>2914.332</v>
+      </c>
       <c r="H8" s="9" t="n"/>
       <c r="I8" s="9" t="n"/>
-      <c r="J8" s="9" t="n"/>
+      <c r="J8" s="8" t="n">
+        <v>3609.2085</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="11" t="n"/>
@@ -2399,20 +2467,26 @@
           <t>PhaseD_AND</t>
         </is>
       </c>
-      <c r="C9" s="9" t="n"/>
+      <c r="C9" s="8" t="n">
+        <v>14.2595</v>
+      </c>
       <c r="D9" s="8" t="n">
-        <v>8.102</v>
+        <v>8.8705</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>5.73</v>
+        <v>5.4845</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>14.244</v>
-      </c>
-      <c r="G9" s="9" t="n"/>
+        <v>5.367</v>
+      </c>
+      <c r="G9" s="8" t="n">
+        <v>9.938499999999999</v>
+      </c>
       <c r="H9" s="9" t="n"/>
       <c r="I9" s="9" t="n"/>
-      <c r="J9" s="9" t="n"/>
+      <c r="J9" s="8" t="n">
+        <v>28.4905</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="11" t="n"/>
@@ -2421,20 +2495,26 @@
           <t>PhaseE_agg</t>
         </is>
       </c>
-      <c r="C10" s="9" t="n"/>
+      <c r="C10" s="8" t="n">
+        <v>82.53</v>
+      </c>
       <c r="D10" s="8" t="n">
-        <v>81.441</v>
+        <v>82.04949999999999</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>82.407</v>
+        <v>82.32550000000001</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>81.90000000000001</v>
-      </c>
-      <c r="G10" s="9" t="n"/>
+        <v>82.6075</v>
+      </c>
+      <c r="G10" s="8" t="n">
+        <v>82.7615</v>
+      </c>
       <c r="H10" s="9" t="n"/>
       <c r="I10" s="9" t="n"/>
-      <c r="J10" s="9" t="n"/>
+      <c r="J10" s="8" t="n">
+        <v>83.559</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="n"/>
@@ -2443,20 +2523,26 @@
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C11" s="9" t="n"/>
+      <c r="C11" s="8" t="n">
+        <v>3567.423</v>
+      </c>
       <c r="D11" s="8" t="n">
-        <v>2311.252</v>
+        <v>2335.4595</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>2817.675</v>
+        <v>1653.717</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>4330.24</v>
-      </c>
-      <c r="G11" s="9" t="n"/>
+        <v>1379.7845</v>
+      </c>
+      <c r="G11" s="8" t="n">
+        <v>4120.672</v>
+      </c>
       <c r="H11" s="9" t="n"/>
       <c r="I11" s="9" t="n"/>
-      <c r="J11" s="9" t="n"/>
+      <c r="J11" s="8" t="n">
+        <v>4953.748</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -2469,20 +2555,26 @@
           <t>PhaseA_orders</t>
         </is>
       </c>
-      <c r="C12" s="9" t="n"/>
+      <c r="C12" s="8" t="n">
+        <v>243.1965</v>
+      </c>
       <c r="D12" s="8" t="n">
-        <v>248.2625</v>
+        <v>242.0565</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>249.4155</v>
+        <v>242.959</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>245.2065</v>
-      </c>
-      <c r="G12" s="9" t="n"/>
+        <v>245.6165</v>
+      </c>
+      <c r="G12" s="8" t="n">
+        <v>242.5845</v>
+      </c>
       <c r="H12" s="9" t="n"/>
       <c r="I12" s="9" t="n"/>
-      <c r="J12" s="9" t="n"/>
+      <c r="J12" s="8" t="n">
+        <v>243.836</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="11" t="n"/>
@@ -2491,20 +2583,26 @@
           <t>PhaseB_okey</t>
         </is>
       </c>
-      <c r="C13" s="9" t="n"/>
+      <c r="C13" s="8" t="n">
+        <v>814.0235</v>
+      </c>
       <c r="D13" s="8" t="n">
-        <v>281.15</v>
+        <v>277.59</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>507.4705</v>
+        <v>533.6075</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>159.323</v>
-      </c>
-      <c r="G13" s="9" t="n"/>
+        <v>160.3505</v>
+      </c>
+      <c r="G13" s="8" t="n">
+        <v>359.367</v>
+      </c>
       <c r="H13" s="9" t="n"/>
       <c r="I13" s="9" t="n"/>
-      <c r="J13" s="9" t="n"/>
+      <c r="J13" s="8" t="n">
+        <v>438.502</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="11" t="n"/>
@@ -2513,20 +2611,26 @@
           <t>PhaseC_exists</t>
         </is>
       </c>
-      <c r="C14" s="9" t="n"/>
+      <c r="C14" s="8" t="n">
+        <v>235.28</v>
+      </c>
       <c r="D14" s="8" t="n">
-        <v>237.2995</v>
+        <v>235.1395</v>
       </c>
       <c r="E14" s="8" t="n">
-        <v>238.5415</v>
+        <v>236.9025</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>236.6625</v>
-      </c>
-      <c r="G14" s="9" t="n"/>
+        <v>237.129</v>
+      </c>
+      <c r="G14" s="8" t="n">
+        <v>235.073</v>
+      </c>
       <c r="H14" s="9" t="n"/>
       <c r="I14" s="9" t="n"/>
-      <c r="J14" s="9" t="n"/>
+      <c r="J14" s="8" t="n">
+        <v>234.8045</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="11" t="n"/>
@@ -2535,20 +2639,26 @@
           <t>PhaseD_count</t>
         </is>
       </c>
-      <c r="C15" s="9" t="n"/>
+      <c r="C15" s="8" t="n">
+        <v>60.683</v>
+      </c>
       <c r="D15" s="8" t="n">
-        <v>62.2325</v>
+        <v>59.429</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>62.846</v>
+        <v>60.462</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>61.49</v>
-      </c>
-      <c r="G15" s="9" t="n"/>
+        <v>60.418</v>
+      </c>
+      <c r="G15" s="8" t="n">
+        <v>60.707</v>
+      </c>
       <c r="H15" s="9" t="n"/>
       <c r="I15" s="9" t="n"/>
-      <c r="J15" s="9" t="n"/>
+      <c r="J15" s="8" t="n">
+        <v>60.6015</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="12" t="n"/>
@@ -2557,20 +2667,26 @@
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C16" s="9" t="n"/>
+      <c r="C16" s="8" t="n">
+        <v>1353.263</v>
+      </c>
       <c r="D16" s="8" t="n">
-        <v>828.6325000000001</v>
+        <v>814.4745</v>
       </c>
       <c r="E16" s="8" t="n">
-        <v>1059.1705</v>
+        <v>1074.3785</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>702.6345</v>
-      </c>
-      <c r="G16" s="9" t="n"/>
+        <v>703.89</v>
+      </c>
+      <c r="G16" s="8" t="n">
+        <v>897.4485</v>
+      </c>
       <c r="H16" s="9" t="n"/>
       <c r="I16" s="9" t="n"/>
-      <c r="J16" s="9" t="n"/>
+      <c r="J16" s="8" t="n">
+        <v>977.87</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -2583,23 +2699,25 @@
           <t>PhaseA</t>
         </is>
       </c>
-      <c r="C17" s="9" t="n"/>
+      <c r="C17" s="8" t="n">
+        <v>282.358</v>
+      </c>
       <c r="D17" s="8" t="n">
-        <v>316.5755</v>
+        <v>279.9095</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>290.7215</v>
+        <v>279.82</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>318.258</v>
+        <v>313.016</v>
       </c>
       <c r="G17" s="8" t="n">
-        <v>289.0415</v>
+        <v>301.22</v>
       </c>
       <c r="H17" s="9" t="n"/>
       <c r="I17" s="9" t="n"/>
       <c r="J17" s="8" t="n">
-        <v>297.051</v>
+        <v>283.585</v>
       </c>
     </row>
     <row r="18">
@@ -2609,23 +2727,25 @@
           <t>PhaseB</t>
         </is>
       </c>
-      <c r="C18" s="9" t="n"/>
+      <c r="C18" s="8" t="n">
+        <v>3022.255</v>
+      </c>
       <c r="D18" s="8" t="n">
-        <v>901.6325000000001</v>
+        <v>880.579</v>
       </c>
       <c r="E18" s="8" t="n">
-        <v>2465.5035</v>
+        <v>2623.953</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>526.7</v>
+        <v>523.522</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>2631.059</v>
+        <v>2453.86</v>
       </c>
       <c r="H18" s="9" t="n"/>
       <c r="I18" s="9" t="n"/>
       <c r="J18" s="8" t="n">
-        <v>2652.7555</v>
+        <v>2629.2995</v>
       </c>
     </row>
     <row r="19">
@@ -2635,23 +2755,25 @@
           <t>PhaseC</t>
         </is>
       </c>
-      <c r="C19" s="9" t="n"/>
+      <c r="C19" s="8" t="n">
+        <v>123.0745</v>
+      </c>
       <c r="D19" s="8" t="n">
-        <v>125.0115</v>
+        <v>123.813</v>
       </c>
       <c r="E19" s="8" t="n">
-        <v>124.5765</v>
+        <v>123.5125</v>
       </c>
       <c r="F19" s="8" t="n">
-        <v>125.8135</v>
+        <v>125.7185</v>
       </c>
       <c r="G19" s="8" t="n">
-        <v>123.81</v>
+        <v>124.387</v>
       </c>
       <c r="H19" s="9" t="n"/>
       <c r="I19" s="9" t="n"/>
       <c r="J19" s="8" t="n">
-        <v>125.371</v>
+        <v>123.2775</v>
       </c>
     </row>
     <row r="20">
@@ -2661,23 +2783,25 @@
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C20" s="9" t="n"/>
+      <c r="C20" s="8" t="n">
+        <v>3428.306</v>
+      </c>
       <c r="D20" s="8" t="n">
-        <v>1343.0815</v>
+        <v>1284.302</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>2880.6655</v>
+        <v>3029.9815</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>971.0975</v>
+        <v>961.7535</v>
       </c>
       <c r="G20" s="8" t="n">
-        <v>3043.593</v>
+        <v>2879.6125</v>
       </c>
       <c r="H20" s="9" t="n"/>
       <c r="I20" s="9" t="n"/>
       <c r="J20" s="8" t="n">
-        <v>3077.1495</v>
+        <v>3036.581</v>
       </c>
     </row>
     <row r="21">
@@ -2695,21 +2819,21 @@
         <v>0.005</v>
       </c>
       <c r="D21" s="8" t="n">
-        <v>1.991</v>
+        <v>2.011</v>
       </c>
       <c r="E21" s="8" t="n">
-        <v>0.9409999999999999</v>
+        <v>0.944</v>
       </c>
       <c r="F21" s="8" t="n">
-        <v>0.827</v>
+        <v>0.907</v>
       </c>
       <c r="G21" s="8" t="n">
-        <v>2.897</v>
+        <v>2.716</v>
       </c>
       <c r="H21" s="9" t="n"/>
       <c r="I21" s="9" t="n"/>
       <c r="J21" s="8" t="n">
-        <v>1.179</v>
+        <v>1.502</v>
       </c>
     </row>
     <row r="22">
@@ -2720,24 +2844,24 @@
         </is>
       </c>
       <c r="C22" s="8" t="n">
-        <v>11.066</v>
+        <v>12.852</v>
       </c>
       <c r="D22" s="8" t="n">
-        <v>4.655</v>
+        <v>4.523</v>
       </c>
       <c r="E22" s="8" t="n">
-        <v>1.789</v>
+        <v>1.879</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>1.715</v>
+        <v>1.836</v>
       </c>
       <c r="G22" s="8" t="n">
-        <v>5.984</v>
+        <v>7.833</v>
       </c>
       <c r="H22" s="9" t="n"/>
       <c r="I22" s="9" t="n"/>
       <c r="J22" s="8" t="n">
-        <v>26.877</v>
+        <v>27.69</v>
       </c>
     </row>
     <row r="23">
@@ -2748,24 +2872,24 @@
         </is>
       </c>
       <c r="C23" s="8" t="n">
-        <v>91.595</v>
+        <v>84.88</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>10.193</v>
+        <v>10.394</v>
       </c>
       <c r="E23" s="8" t="n">
-        <v>3.157</v>
+        <v>2.864</v>
       </c>
       <c r="F23" s="8" t="n">
-        <v>2.531</v>
+        <v>2.684</v>
       </c>
       <c r="G23" s="8" t="n">
-        <v>177.358</v>
+        <v>192.749</v>
       </c>
       <c r="H23" s="9" t="n"/>
       <c r="I23" s="9" t="n"/>
       <c r="J23" s="8" t="n">
-        <v>507.12</v>
+        <v>517.647</v>
       </c>
     </row>
     <row r="24">
@@ -2776,24 +2900,24 @@
         </is>
       </c>
       <c r="C24" s="8" t="n">
-        <v>3.789</v>
+        <v>3.735</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>3.195</v>
+        <v>3.299</v>
       </c>
       <c r="E24" s="8" t="n">
-        <v>13.697</v>
+        <v>13.134</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>13.776</v>
+        <v>13.398</v>
       </c>
       <c r="G24" s="8" t="n">
-        <v>12.418</v>
+        <v>12.898</v>
       </c>
       <c r="H24" s="9" t="n"/>
       <c r="I24" s="9" t="n"/>
       <c r="J24" s="8" t="n">
-        <v>64.56</v>
+        <v>64.624</v>
       </c>
     </row>
     <row r="25">
@@ -2804,24 +2928,24 @@
         </is>
       </c>
       <c r="C25" s="8" t="n">
-        <v>33.612</v>
+        <v>32.847</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>7.077</v>
+        <v>7.106</v>
       </c>
       <c r="E25" s="8" t="n">
-        <v>5.76</v>
+        <v>5.239</v>
       </c>
       <c r="F25" s="8" t="n">
-        <v>5.793</v>
+        <v>5.797</v>
       </c>
       <c r="G25" s="8" t="n">
-        <v>12.222</v>
+        <v>12.286</v>
       </c>
       <c r="H25" s="9" t="n"/>
       <c r="I25" s="9" t="n"/>
       <c r="J25" s="8" t="n">
-        <v>16.765</v>
+        <v>16.994</v>
       </c>
     </row>
     <row r="26">
@@ -2832,485 +2956,1020 @@
         </is>
       </c>
       <c r="C26" s="8" t="n">
-        <v>140.076</v>
+        <v>134.332</v>
       </c>
       <c r="D26" s="8" t="n">
-        <v>28.473</v>
+        <v>28.741</v>
       </c>
       <c r="E26" s="8" t="n">
-        <v>25.354</v>
+        <v>24.068</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>24.651</v>
+        <v>24.631</v>
       </c>
       <c r="G26" s="8" t="n">
-        <v>210.889</v>
+        <v>228.494</v>
       </c>
       <c r="H26" s="9" t="n"/>
       <c r="I26" s="9" t="n"/>
       <c r="J26" s="8" t="n">
-        <v>616.513</v>
+        <v>628.467</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>Q14</t>
+          <t>Q8</t>
         </is>
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>PhaseA_ship</t>
+          <t>PhaseA_side</t>
         </is>
       </c>
       <c r="C27" s="8" t="n">
-        <v>108.436</v>
+        <v>88.489</v>
       </c>
       <c r="D27" s="8" t="n">
-        <v>34.4515</v>
+        <v>88.1905</v>
       </c>
       <c r="E27" s="8" t="n">
-        <v>20.9445</v>
+        <v>88.1785</v>
       </c>
       <c r="F27" s="8" t="n">
-        <v>11.2175</v>
+        <v>88.3385</v>
       </c>
       <c r="G27" s="8" t="n">
-        <v>62.574</v>
+        <v>88.511</v>
       </c>
       <c r="H27" s="9" t="n"/>
       <c r="I27" s="9" t="n"/>
       <c r="J27" s="8" t="n">
-        <v>69.56999999999999</v>
+        <v>88.45950000000001</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="11" t="n"/>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>PhaseB_part</t>
+          <t>PhaseB_orders</t>
         </is>
       </c>
       <c r="C28" s="8" t="n">
-        <v>79.1005</v>
+        <v>354.0105</v>
       </c>
       <c r="D28" s="8" t="n">
-        <v>83.52800000000001</v>
+        <v>344.3415</v>
       </c>
       <c r="E28" s="8" t="n">
-        <v>79.973</v>
+        <v>357.294</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>79.57550000000001</v>
+        <v>355.584</v>
       </c>
       <c r="G28" s="8" t="n">
-        <v>78.408</v>
+        <v>352.364</v>
       </c>
       <c r="H28" s="9" t="n"/>
       <c r="I28" s="9" t="n"/>
       <c r="J28" s="8" t="n">
-        <v>79.87050000000001</v>
+        <v>356.307</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="11" t="n"/>
       <c r="B29" s="10" t="inlineStr">
         <is>
-          <t>PhaseC_agg</t>
+          <t>PhaseCDE_OR_AND</t>
         </is>
       </c>
       <c r="C29" s="8" t="n">
-        <v>89.8605</v>
+        <v>1233.4145</v>
       </c>
       <c r="D29" s="8" t="n">
-        <v>90.069</v>
+        <v>333.2545</v>
       </c>
       <c r="E29" s="8" t="n">
-        <v>89.125</v>
+        <v>479.129</v>
       </c>
       <c r="F29" s="8" t="n">
-        <v>88.8445</v>
+        <v>458.864</v>
       </c>
       <c r="G29" s="8" t="n">
-        <v>88.27800000000001</v>
+        <v>668.746</v>
       </c>
       <c r="H29" s="9" t="n"/>
       <c r="I29" s="9" t="n"/>
       <c r="J29" s="8" t="n">
-        <v>95.7235</v>
+        <v>768.0765</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="12" t="n"/>
+      <c r="A30" s="11" t="n"/>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>PhaseF_agg</t>
         </is>
       </c>
       <c r="C30" s="8" t="n">
-        <v>277.389</v>
+        <v>29.0035</v>
       </c>
       <c r="D30" s="8" t="n">
-        <v>207.964</v>
+        <v>29.9085</v>
       </c>
       <c r="E30" s="8" t="n">
-        <v>190.287</v>
+        <v>29.2105</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>179.7225</v>
+        <v>29.057</v>
       </c>
       <c r="G30" s="8" t="n">
-        <v>229.2315</v>
+        <v>29.146</v>
       </c>
       <c r="H30" s="9" t="n"/>
       <c r="I30" s="9" t="n"/>
       <c r="J30" s="8" t="n">
-        <v>245.095</v>
+        <v>29.179</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="7" t="inlineStr">
-        <is>
-          <t>Q15</t>
-        </is>
-      </c>
+      <c r="A31" s="11" t="n"/>
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t>OR</t>
-        </is>
-      </c>
-      <c r="C31" s="8" t="n">
-        <v>10.4295</v>
-      </c>
-      <c r="D31" s="8" t="n">
-        <v>22.1345</v>
-      </c>
-      <c r="E31" s="8" t="n">
-        <v>82.34650000000001</v>
-      </c>
-      <c r="F31" s="8" t="n">
-        <v>12.1195</v>
-      </c>
-      <c r="G31" s="8" t="n">
-        <v>189.147</v>
-      </c>
-      <c r="H31" s="8" t="n">
-        <v>90.1255</v>
-      </c>
-      <c r="I31" s="8" t="n">
-        <v>60.573</v>
-      </c>
-      <c r="J31" s="8" t="n">
-        <v>207.621</v>
-      </c>
+          <t>PhaseG_share</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="n"/>
+      <c r="D31" s="9" t="n"/>
+      <c r="E31" s="9" t="n"/>
+      <c r="F31" s="9" t="n"/>
+      <c r="G31" s="9" t="n"/>
+      <c r="H31" s="9" t="n"/>
+      <c r="I31" s="9" t="n"/>
+      <c r="J31" s="9" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="11" t="n"/>
+      <c r="A32" s="12" t="n"/>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>Agg</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="C32" s="8" t="n">
-        <v>72.6315</v>
+        <v>1705.5285</v>
       </c>
       <c r="D32" s="8" t="n">
-        <v>43.8575</v>
+        <v>795.7234999999999</v>
       </c>
       <c r="E32" s="8" t="n">
-        <v>53.5335</v>
+        <v>954.004</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>53.073</v>
+        <v>932.015</v>
       </c>
       <c r="G32" s="8" t="n">
-        <v>50.8185</v>
-      </c>
-      <c r="H32" s="8" t="n">
-        <v>28.1475</v>
-      </c>
-      <c r="I32" s="8" t="n">
-        <v>28.2415</v>
-      </c>
+        <v>1139.955</v>
+      </c>
+      <c r="H32" s="9" t="n"/>
+      <c r="I32" s="9" t="n"/>
       <c r="J32" s="8" t="n">
-        <v>57.9075</v>
+        <v>1241.548</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="12" t="n"/>
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>Q10</t>
+        </is>
+      </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>PhaseA_orders</t>
         </is>
       </c>
       <c r="C33" s="8" t="n">
-        <v>83.1835</v>
+        <v>93.4965</v>
       </c>
       <c r="D33" s="8" t="n">
-        <v>65.8505</v>
+        <v>92.741</v>
       </c>
       <c r="E33" s="8" t="n">
-        <v>135.906</v>
+        <v>99.801</v>
       </c>
       <c r="F33" s="8" t="n">
-        <v>65.24299999999999</v>
+        <v>92.27249999999999</v>
       </c>
       <c r="G33" s="8" t="n">
-        <v>240.268</v>
-      </c>
-      <c r="H33" s="8" t="n">
-        <v>118.411</v>
-      </c>
-      <c r="I33" s="8" t="n">
-        <v>88.82299999999999</v>
-      </c>
+        <v>93.116</v>
+      </c>
+      <c r="H33" s="9" t="n"/>
+      <c r="I33" s="9" t="n"/>
       <c r="J33" s="8" t="n">
-        <v>265.875</v>
+        <v>92.4225</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="7" t="inlineStr">
-        <is>
-          <t>Q17</t>
-        </is>
-      </c>
+      <c r="A34" s="11" t="n"/>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>PhaseA_part</t>
+          <t>PhaseB_okey</t>
         </is>
       </c>
       <c r="C34" s="8" t="n">
-        <v>443.5375</v>
+        <v>714.7265</v>
       </c>
       <c r="D34" s="8" t="n">
-        <v>35.6085</v>
+        <v>191.4745</v>
       </c>
       <c r="E34" s="8" t="n">
-        <v>32.076</v>
+        <v>273.2755</v>
       </c>
       <c r="F34" s="8" t="n">
-        <v>32.1655</v>
+        <v>257.7525</v>
       </c>
       <c r="G34" s="8" t="n">
-        <v>468.0265</v>
+        <v>276.625</v>
       </c>
       <c r="H34" s="9" t="n"/>
       <c r="I34" s="9" t="n"/>
       <c r="J34" s="8" t="n">
-        <v>515.859</v>
+        <v>354.0475</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="11" t="n"/>
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t>PhaseB_avg</t>
+          <t>PhaseC_rf</t>
         </is>
       </c>
       <c r="C35" s="8" t="n">
-        <v>23.5965</v>
+        <v>0.002</v>
       </c>
       <c r="D35" s="8" t="n">
-        <v>20.3655</v>
+        <v>2.963</v>
       </c>
       <c r="E35" s="8" t="n">
-        <v>19.269</v>
+        <v>0.9615</v>
       </c>
       <c r="F35" s="8" t="n">
-        <v>19.7855</v>
+        <v>0.9425</v>
       </c>
       <c r="G35" s="8" t="n">
-        <v>26.008</v>
+        <v>1.663</v>
       </c>
       <c r="H35" s="9" t="n"/>
       <c r="I35" s="9" t="n"/>
       <c r="J35" s="8" t="n">
-        <v>23.949</v>
+        <v>1.4505</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="11" t="n"/>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>PhaseC_sum</t>
+          <t>PhaseD_AND</t>
         </is>
       </c>
       <c r="C36" s="8" t="n">
-        <v>0.919</v>
+        <v>37.551</v>
       </c>
       <c r="D36" s="8" t="n">
-        <v>1.023</v>
+        <v>11.663</v>
       </c>
       <c r="E36" s="8" t="n">
-        <v>0.987</v>
+        <v>8.172000000000001</v>
       </c>
       <c r="F36" s="8" t="n">
-        <v>0.975</v>
+        <v>7.646</v>
       </c>
       <c r="G36" s="8" t="n">
-        <v>1.186</v>
+        <v>19.408</v>
       </c>
       <c r="H36" s="9" t="n"/>
       <c r="I36" s="9" t="n"/>
       <c r="J36" s="8" t="n">
-        <v>0.9325</v>
+        <v>40.8425</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="12" t="n"/>
+      <c r="A37" s="11" t="n"/>
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>PhaseE_agg</t>
         </is>
       </c>
       <c r="C37" s="8" t="n">
-        <v>468.0545</v>
+        <v>212.73</v>
       </c>
       <c r="D37" s="8" t="n">
-        <v>56.996</v>
+        <v>206.2135</v>
       </c>
       <c r="E37" s="8" t="n">
-        <v>52.332</v>
+        <v>211.9825</v>
       </c>
       <c r="F37" s="8" t="n">
-        <v>52.9235</v>
+        <v>203.9285</v>
       </c>
       <c r="G37" s="8" t="n">
-        <v>495.2225</v>
+        <v>214.615</v>
       </c>
       <c r="H37" s="9" t="n"/>
       <c r="I37" s="9" t="n"/>
       <c r="J37" s="8" t="n">
-        <v>540.683</v>
+        <v>205.6075</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="7" t="inlineStr">
-        <is>
-          <t>Q19</t>
-        </is>
-      </c>
+      <c r="A38" s="11" t="n"/>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>PhaseA_ship</t>
+          <t>PhaseF_top20</t>
         </is>
       </c>
       <c r="C38" s="8" t="n">
-        <v>80.48399999999999</v>
+        <v>7.638</v>
       </c>
       <c r="D38" s="8" t="n">
-        <v>29.631</v>
+        <v>7.3125</v>
       </c>
       <c r="E38" s="8" t="n">
-        <v>22.794</v>
+        <v>7.665</v>
       </c>
       <c r="F38" s="8" t="n">
-        <v>23.533</v>
+        <v>7.5845</v>
       </c>
       <c r="G38" s="8" t="n">
-        <v>50.499</v>
+        <v>7.3595</v>
       </c>
       <c r="H38" s="9" t="n"/>
       <c r="I38" s="9" t="n"/>
       <c r="J38" s="8" t="n">
-        <v>80.13549999999999</v>
+        <v>7.3165</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="11" t="n"/>
+      <c r="A39" s="12" t="n"/>
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t>PhaseB_part</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="C39" s="8" t="n">
-        <v>28.236</v>
+        <v>1069.076</v>
       </c>
       <c r="D39" s="8" t="n">
-        <v>28.2265</v>
+        <v>512.638</v>
       </c>
       <c r="E39" s="8" t="n">
-        <v>28.1925</v>
+        <v>602.7380000000001</v>
       </c>
       <c r="F39" s="8" t="n">
-        <v>28.1225</v>
+        <v>570.16</v>
       </c>
       <c r="G39" s="8" t="n">
-        <v>28.0165</v>
+        <v>612.7025</v>
       </c>
       <c r="H39" s="9" t="n"/>
       <c r="I39" s="9" t="n"/>
       <c r="J39" s="8" t="n">
-        <v>28.0805</v>
+        <v>700.9105</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="11" t="n"/>
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>Q12</t>
+        </is>
+      </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>PhaseC_agg</t>
+          <t>PhaseA_orders</t>
         </is>
       </c>
       <c r="C40" s="8" t="n">
-        <v>160.855</v>
+        <v>604.455</v>
       </c>
       <c r="D40" s="8" t="n">
-        <v>161.2325</v>
+        <v>607.1895</v>
       </c>
       <c r="E40" s="8" t="n">
-        <v>160.686</v>
+        <v>606.3869999999999</v>
       </c>
       <c r="F40" s="8" t="n">
-        <v>161.454</v>
+        <v>604.671</v>
       </c>
       <c r="G40" s="8" t="n">
-        <v>161.2035</v>
+        <v>606.222</v>
       </c>
       <c r="H40" s="9" t="n"/>
       <c r="I40" s="9" t="n"/>
       <c r="J40" s="8" t="n">
-        <v>160.563</v>
+        <v>603.728</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="12" t="n"/>
+      <c r="A41" s="11" t="n"/>
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>PhaseB_shipmode</t>
         </is>
       </c>
       <c r="C41" s="8" t="n">
-        <v>269.872</v>
+        <v>17.4005</v>
       </c>
       <c r="D41" s="8" t="n">
-        <v>219.166</v>
+        <v>6.3855</v>
       </c>
       <c r="E41" s="8" t="n">
-        <v>212.2775</v>
+        <v>1.6865</v>
       </c>
       <c r="F41" s="8" t="n">
-        <v>213.504</v>
+        <v>1.6265</v>
       </c>
       <c r="G41" s="8" t="n">
-        <v>239.8755</v>
+        <v>4.0765</v>
       </c>
       <c r="H41" s="9" t="n"/>
       <c r="I41" s="9" t="n"/>
       <c r="J41" s="8" t="n">
-        <v>268.6065</v>
+        <v>33.215</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="11" t="n"/>
+      <c r="B42" s="10" t="inlineStr">
+        <is>
+          <t>PhaseC_rdate</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="n">
+        <v>867.301</v>
+      </c>
+      <c r="D42" s="8" t="n">
+        <v>263.486</v>
+      </c>
+      <c r="E42" s="8" t="n">
+        <v>255.4865</v>
+      </c>
+      <c r="F42" s="8" t="n">
+        <v>38.071</v>
+      </c>
+      <c r="G42" s="8" t="n">
+        <v>955.047</v>
+      </c>
+      <c r="H42" s="9" t="n"/>
+      <c r="I42" s="9" t="n"/>
+      <c r="J42" s="8" t="n">
+        <v>1053.933</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="11" t="n"/>
+      <c r="B43" s="10" t="inlineStr">
+        <is>
+          <t>PhaseD_AND</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="n">
+        <v>75.3425</v>
+      </c>
+      <c r="D43" s="8" t="n">
+        <v>42.6535</v>
+      </c>
+      <c r="E43" s="8" t="n">
+        <v>25.154</v>
+      </c>
+      <c r="F43" s="8" t="n">
+        <v>24.8025</v>
+      </c>
+      <c r="G43" s="8" t="n">
+        <v>49.0955</v>
+      </c>
+      <c r="H43" s="9" t="n"/>
+      <c r="I43" s="9" t="n"/>
+      <c r="J43" s="8" t="n">
+        <v>88.64400000000001</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="11" t="n"/>
+      <c r="B44" s="10" t="inlineStr">
+        <is>
+          <t>PhaseE_agg</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="n">
+        <v>413.2565</v>
+      </c>
+      <c r="D44" s="8" t="n">
+        <v>419.0115</v>
+      </c>
+      <c r="E44" s="8" t="n">
+        <v>403.369</v>
+      </c>
+      <c r="F44" s="8" t="n">
+        <v>409.7575</v>
+      </c>
+      <c r="G44" s="8" t="n">
+        <v>411.2285</v>
+      </c>
+      <c r="H44" s="9" t="n"/>
+      <c r="I44" s="9" t="n"/>
+      <c r="J44" s="8" t="n">
+        <v>413.478</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="12" t="n"/>
+      <c r="B45" s="10" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="n">
+        <v>1977.6165</v>
+      </c>
+      <c r="D45" s="8" t="n">
+        <v>1339.277</v>
+      </c>
+      <c r="E45" s="8" t="n">
+        <v>1292.08</v>
+      </c>
+      <c r="F45" s="8" t="n">
+        <v>1079.6835</v>
+      </c>
+      <c r="G45" s="8" t="n">
+        <v>2025.361</v>
+      </c>
+      <c r="H45" s="9" t="n"/>
+      <c r="I45" s="9" t="n"/>
+      <c r="J45" s="8" t="n">
+        <v>2192.618</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="7" t="inlineStr">
+        <is>
+          <t>Q14</t>
+        </is>
+      </c>
+      <c r="B46" s="10" t="inlineStr">
+        <is>
+          <t>PhaseA_ship</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="n">
+        <v>108.834</v>
+      </c>
+      <c r="D46" s="8" t="n">
+        <v>34.511</v>
+      </c>
+      <c r="E46" s="8" t="n">
+        <v>19.769</v>
+      </c>
+      <c r="F46" s="8" t="n">
+        <v>11.008</v>
+      </c>
+      <c r="G46" s="8" t="n">
+        <v>63.611</v>
+      </c>
+      <c r="H46" s="9" t="n"/>
+      <c r="I46" s="9" t="n"/>
+      <c r="J46" s="8" t="n">
+        <v>69.32850000000001</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="11" t="n"/>
+      <c r="B47" s="10" t="inlineStr">
+        <is>
+          <t>PhaseB_part</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="n">
+        <v>78.89400000000001</v>
+      </c>
+      <c r="D47" s="8" t="n">
+        <v>83.90900000000001</v>
+      </c>
+      <c r="E47" s="8" t="n">
+        <v>79.56999999999999</v>
+      </c>
+      <c r="F47" s="8" t="n">
+        <v>80.16500000000001</v>
+      </c>
+      <c r="G47" s="8" t="n">
+        <v>78.27200000000001</v>
+      </c>
+      <c r="H47" s="9" t="n"/>
+      <c r="I47" s="9" t="n"/>
+      <c r="J47" s="8" t="n">
+        <v>79.371</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="11" t="n"/>
+      <c r="B48" s="10" t="inlineStr">
+        <is>
+          <t>PhaseC_agg</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="n">
+        <v>89.98399999999999</v>
+      </c>
+      <c r="D48" s="8" t="n">
+        <v>90.1735</v>
+      </c>
+      <c r="E48" s="8" t="n">
+        <v>89.9315</v>
+      </c>
+      <c r="F48" s="8" t="n">
+        <v>91.13849999999999</v>
+      </c>
+      <c r="G48" s="8" t="n">
+        <v>89.0185</v>
+      </c>
+      <c r="H48" s="9" t="n"/>
+      <c r="I48" s="9" t="n"/>
+      <c r="J48" s="8" t="n">
+        <v>90.349</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="12" t="n"/>
+      <c r="B49" s="10" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="n">
+        <v>277.701</v>
+      </c>
+      <c r="D49" s="8" t="n">
+        <v>208.468</v>
+      </c>
+      <c r="E49" s="8" t="n">
+        <v>189.4175</v>
+      </c>
+      <c r="F49" s="8" t="n">
+        <v>182.1065</v>
+      </c>
+      <c r="G49" s="8" t="n">
+        <v>230.836</v>
+      </c>
+      <c r="H49" s="9" t="n"/>
+      <c r="I49" s="9" t="n"/>
+      <c r="J49" s="8" t="n">
+        <v>239.195</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="7" t="inlineStr">
+        <is>
+          <t>Q15</t>
+        </is>
+      </c>
+      <c r="B50" s="10" t="inlineStr">
+        <is>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="n">
+        <v>10.4295</v>
+      </c>
+      <c r="D50" s="8" t="n">
+        <v>22.1345</v>
+      </c>
+      <c r="E50" s="8" t="n">
+        <v>82.34650000000001</v>
+      </c>
+      <c r="F50" s="8" t="n">
+        <v>12.1195</v>
+      </c>
+      <c r="G50" s="8" t="n">
+        <v>189.147</v>
+      </c>
+      <c r="H50" s="8" t="n">
+        <v>90.1255</v>
+      </c>
+      <c r="I50" s="8" t="n">
+        <v>60.573</v>
+      </c>
+      <c r="J50" s="8" t="n">
+        <v>207.621</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="11" t="n"/>
+      <c r="B51" s="10" t="inlineStr">
+        <is>
+          <t>Agg</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="n">
+        <v>72.6315</v>
+      </c>
+      <c r="D51" s="8" t="n">
+        <v>43.8575</v>
+      </c>
+      <c r="E51" s="8" t="n">
+        <v>53.5335</v>
+      </c>
+      <c r="F51" s="8" t="n">
+        <v>53.073</v>
+      </c>
+      <c r="G51" s="8" t="n">
+        <v>50.8185</v>
+      </c>
+      <c r="H51" s="8" t="n">
+        <v>28.1475</v>
+      </c>
+      <c r="I51" s="8" t="n">
+        <v>28.2415</v>
+      </c>
+      <c r="J51" s="8" t="n">
+        <v>57.9075</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="12" t="n"/>
+      <c r="B52" s="10" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C52" s="8" t="n">
+        <v>83.1835</v>
+      </c>
+      <c r="D52" s="8" t="n">
+        <v>65.8505</v>
+      </c>
+      <c r="E52" s="8" t="n">
+        <v>135.906</v>
+      </c>
+      <c r="F52" s="8" t="n">
+        <v>65.24299999999999</v>
+      </c>
+      <c r="G52" s="8" t="n">
+        <v>240.268</v>
+      </c>
+      <c r="H52" s="8" t="n">
+        <v>118.411</v>
+      </c>
+      <c r="I52" s="8" t="n">
+        <v>88.82299999999999</v>
+      </c>
+      <c r="J52" s="8" t="n">
+        <v>265.875</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="7" t="inlineStr">
+        <is>
+          <t>Q17</t>
+        </is>
+      </c>
+      <c r="B53" s="10" t="inlineStr">
+        <is>
+          <t>PhaseA_part</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="n">
+        <v>444.8</v>
+      </c>
+      <c r="D53" s="8" t="n">
+        <v>36.411</v>
+      </c>
+      <c r="E53" s="8" t="n">
+        <v>35.5265</v>
+      </c>
+      <c r="F53" s="8" t="n">
+        <v>34.5895</v>
+      </c>
+      <c r="G53" s="8" t="n">
+        <v>459.6365</v>
+      </c>
+      <c r="H53" s="9" t="n"/>
+      <c r="I53" s="9" t="n"/>
+      <c r="J53" s="8" t="n">
+        <v>511.877</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="11" t="n"/>
+      <c r="B54" s="10" t="inlineStr">
+        <is>
+          <t>PhaseB_avg</t>
+        </is>
+      </c>
+      <c r="C54" s="8" t="n">
+        <v>24.5715</v>
+      </c>
+      <c r="D54" s="8" t="n">
+        <v>20.463</v>
+      </c>
+      <c r="E54" s="8" t="n">
+        <v>24.442</v>
+      </c>
+      <c r="F54" s="8" t="n">
+        <v>21.323</v>
+      </c>
+      <c r="G54" s="8" t="n">
+        <v>24.369</v>
+      </c>
+      <c r="H54" s="9" t="n"/>
+      <c r="I54" s="9" t="n"/>
+      <c r="J54" s="8" t="n">
+        <v>24.846</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="11" t="n"/>
+      <c r="B55" s="10" t="inlineStr">
+        <is>
+          <t>PhaseC_sum</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="n">
+        <v>0.907</v>
+      </c>
+      <c r="D55" s="8" t="n">
+        <v>1.0115</v>
+      </c>
+      <c r="E55" s="8" t="n">
+        <v>0.9775</v>
+      </c>
+      <c r="F55" s="8" t="n">
+        <v>0.973</v>
+      </c>
+      <c r="G55" s="8" t="n">
+        <v>0.904</v>
+      </c>
+      <c r="H55" s="9" t="n"/>
+      <c r="I55" s="9" t="n"/>
+      <c r="J55" s="8" t="n">
+        <v>0.904</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="12" t="n"/>
+      <c r="B56" s="10" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C56" s="8" t="n">
+        <v>470.2065</v>
+      </c>
+      <c r="D56" s="8" t="n">
+        <v>57.8865</v>
+      </c>
+      <c r="E56" s="8" t="n">
+        <v>60.9555</v>
+      </c>
+      <c r="F56" s="8" t="n">
+        <v>56.889</v>
+      </c>
+      <c r="G56" s="8" t="n">
+        <v>485.102</v>
+      </c>
+      <c r="H56" s="9" t="n"/>
+      <c r="I56" s="9" t="n"/>
+      <c r="J56" s="8" t="n">
+        <v>537.5535</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="7" t="inlineStr">
+        <is>
+          <t>Q19</t>
+        </is>
+      </c>
+      <c r="B57" s="10" t="inlineStr">
+        <is>
+          <t>PhaseA_ship</t>
+        </is>
+      </c>
+      <c r="C57" s="8" t="n">
+        <v>80.377</v>
+      </c>
+      <c r="D57" s="8" t="n">
+        <v>30.196</v>
+      </c>
+      <c r="E57" s="8" t="n">
+        <v>23.4155</v>
+      </c>
+      <c r="F57" s="8" t="n">
+        <v>22.856</v>
+      </c>
+      <c r="G57" s="8" t="n">
+        <v>51.2205</v>
+      </c>
+      <c r="H57" s="9" t="n"/>
+      <c r="I57" s="9" t="n"/>
+      <c r="J57" s="8" t="n">
+        <v>80.6755</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="11" t="n"/>
+      <c r="B58" s="10" t="inlineStr">
+        <is>
+          <t>PhaseB_part</t>
+        </is>
+      </c>
+      <c r="C58" s="8" t="n">
+        <v>27.9565</v>
+      </c>
+      <c r="D58" s="8" t="n">
+        <v>28.104</v>
+      </c>
+      <c r="E58" s="8" t="n">
+        <v>28.0375</v>
+      </c>
+      <c r="F58" s="8" t="n">
+        <v>28.1695</v>
+      </c>
+      <c r="G58" s="8" t="n">
+        <v>27.9915</v>
+      </c>
+      <c r="H58" s="9" t="n"/>
+      <c r="I58" s="9" t="n"/>
+      <c r="J58" s="8" t="n">
+        <v>28.1395</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="11" t="n"/>
+      <c r="B59" s="10" t="inlineStr">
+        <is>
+          <t>PhaseC_agg</t>
+        </is>
+      </c>
+      <c r="C59" s="8" t="n">
+        <v>160.4965</v>
+      </c>
+      <c r="D59" s="8" t="n">
+        <v>162.0105</v>
+      </c>
+      <c r="E59" s="8" t="n">
+        <v>159.9325</v>
+      </c>
+      <c r="F59" s="8" t="n">
+        <v>160.873</v>
+      </c>
+      <c r="G59" s="8" t="n">
+        <v>159.9815</v>
+      </c>
+      <c r="H59" s="9" t="n"/>
+      <c r="I59" s="9" t="n"/>
+      <c r="J59" s="8" t="n">
+        <v>160.236</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="12" t="n"/>
+      <c r="B60" s="10" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C60" s="8" t="n">
+        <v>269.1215</v>
+      </c>
+      <c r="D60" s="8" t="n">
+        <v>220.4715</v>
+      </c>
+      <c r="E60" s="8" t="n">
+        <v>212.381</v>
+      </c>
+      <c r="F60" s="8" t="n">
+        <v>212.9095</v>
+      </c>
+      <c r="G60" s="8" t="n">
+        <v>239.585</v>
+      </c>
+      <c r="H60" s="9" t="n"/>
+      <c r="I60" s="9" t="n"/>
+      <c r="J60" s="8" t="n">
+        <v>268.818</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="A27:A30"/>
+  <mergeCells count="12">
     <mergeCell ref="A12:A16"/>
+    <mergeCell ref="A40:A45"/>
     <mergeCell ref="A21:A26"/>
-    <mergeCell ref="A38:A41"/>
+    <mergeCell ref="A46:A49"/>
     <mergeCell ref="A2:A5"/>
     <mergeCell ref="A17:A20"/>
-    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="A33:A39"/>
     <mergeCell ref="A6:A11"/>
-    <mergeCell ref="A31:A33"/>
+    <mergeCell ref="A53:A56"/>
+    <mergeCell ref="A50:A52"/>
+    <mergeCell ref="A57:A60"/>
+    <mergeCell ref="A27:A32"/>
   </mergeCells>
   <conditionalFormatting sqref="C2:J2">
     <cfRule type="colorScale" priority="1">
@@ -3792,6 +4451,234 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="C42:J42">
+    <cfRule type="colorScale" priority="41">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C43:J43">
+    <cfRule type="colorScale" priority="42">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C44:J44">
+    <cfRule type="colorScale" priority="43">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C45:J45">
+    <cfRule type="colorScale" priority="44">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C46:J46">
+    <cfRule type="colorScale" priority="45">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C47:J47">
+    <cfRule type="colorScale" priority="46">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C48:J48">
+    <cfRule type="colorScale" priority="47">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C49:J49">
+    <cfRule type="colorScale" priority="48">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C50:J50">
+    <cfRule type="colorScale" priority="49">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C51:J51">
+    <cfRule type="colorScale" priority="50">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C52:J52">
+    <cfRule type="colorScale" priority="51">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C53:J53">
+    <cfRule type="colorScale" priority="52">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C54:J54">
+    <cfRule type="colorScale" priority="53">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C55:J55">
+    <cfRule type="colorScale" priority="54">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C56:J56">
+    <cfRule type="colorScale" priority="55">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C57:J57">
+    <cfRule type="colorScale" priority="56">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C58:J58">
+    <cfRule type="colorScale" priority="57">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C59:J59">
+    <cfRule type="colorScale" priority="58">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C60:J60">
+    <cfRule type="colorScale" priority="59">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3807,7 +4694,7 @@
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
     <col width="25" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
@@ -3934,9 +4821,11 @@
           <t>Q3</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>orderkey: 1265.80 MB
+shipdate: 467.13 MB
+total: 1732.93 MB</t>
         </is>
       </c>
       <c r="C3" s="13" t="inlineStr">
@@ -3960,24 +4849,28 @@
 total: 395.60 MB</t>
         </is>
       </c>
-      <c r="F3" s="14" t="inlineStr">
+      <c r="F3" s="13" t="inlineStr">
+        <is>
+          <t>orderkey: 365.62 MB
+shipdate: 921.39 MB
+total: 1287.01 MB</t>
+        </is>
+      </c>
+      <c r="G3" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G3" s="14" t="inlineStr">
+      <c r="H3" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H3" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I3" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="I3" s="13" t="inlineStr">
+        <is>
+          <t>orderkey: 239.94 MB
+shipdate: 239.94 MB
+total: 479.89 MB</t>
         </is>
       </c>
     </row>
@@ -3987,9 +4880,10 @@
           <t>Q4</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>orderkey: 1265.80 MB
+total: 1265.80 MB</t>
         </is>
       </c>
       <c r="C4" s="13" t="inlineStr">
@@ -4010,24 +4904,26 @@
 total: 257.15 MB</t>
         </is>
       </c>
-      <c r="F4" s="14" t="inlineStr">
+      <c r="F4" s="13" t="inlineStr">
+        <is>
+          <t>orderkey: 365.62 MB
+total: 365.62 MB</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G4" s="14" t="inlineStr">
+      <c r="H4" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H4" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I4" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="I4" s="13" t="inlineStr">
+        <is>
+          <t>orderkey: 239.94 MB
+total: 239.94 MB</t>
         </is>
       </c>
     </row>
@@ -4037,9 +4933,11 @@
           <t>Q5</t>
         </is>
       </c>
-      <c r="B5" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>orderkey: 1265.80 MB
+suppkey: 487.34 MB
+total: 1753.14 MB</t>
         </is>
       </c>
       <c r="C5" s="13" t="inlineStr">
@@ -4157,144 +5055,180 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="36" customHeight="1">
+    <row r="7" ht="48" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Q8</t>
         </is>
       </c>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>orderkey: 1265.80 MB
+partkey: 631.88 MB
+total: 1897.68 MB</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>orderkey: 4448.84 MB
+partkey: 13567.30 MB
+total: 18016.14 MB</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>orderkey: 359.98 MB
+partkey: 608.09 MB
+total: 968.07 MB</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>orderkey: 257.15 MB
+partkey: 608.09 MB
+total: 865.24 MB</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="inlineStr">
+        <is>
+          <t>orderkey: 365.62 MB
+partkey: 975.75 MB
+total: 1341.37 MB</t>
+        </is>
+      </c>
+      <c r="G7" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C7" s="14" t="inlineStr">
+      <c r="H7" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D7" s="14" t="inlineStr">
+      <c r="I7" s="13" t="inlineStr">
+        <is>
+          <t>orderkey: 239.94 MB
+partkey: 239.94 MB
+total: 479.89 MB</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Q10</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>orderkey: 1265.80 MB
+returnflag: 23.22 MB
+total: 1289.02 MB</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>orderkey: 4448.84 MB
+returnflag: 29.78 MB
+total: 4478.62 MB</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>orderkey: 359.98 MB
+returnflag: 22.53 MB
+total: 382.51 MB</t>
+        </is>
+      </c>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>orderkey: 257.15 MB
+returnflag: 22.53 MB
+total: 279.69 MB</t>
+        </is>
+      </c>
+      <c r="F8" s="13" t="inlineStr">
+        <is>
+          <t>orderkey: 365.62 MB
+returnflag: 22.49 MB
+total: 388.12 MB</t>
+        </is>
+      </c>
+      <c r="G8" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E7" s="14" t="inlineStr">
+      <c r="H8" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F7" s="14" t="inlineStr">
+      <c r="I8" s="13" t="inlineStr">
+        <is>
+          <t>orderkey: 239.94 MB
+returnflag: 239.94 MB
+total: 479.89 MB</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Q12</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>shipmode: 46.44 MB
+receiptdate: 467.73 MB
+total: 514.17 MB</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>shipmode: 58.13 MB
+receiptdate: 6593.20 MB
+total: 6651.33 MB</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>shipmode: 45.06 MB
+receiptdate: 138.52 MB
+total: 183.57 MB</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>shipmode: 45.06 MB
+receiptdate: 138.52 MB
+total: 183.57 MB</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>shipmode: 44.99 MB
+receiptdate: 922.61 MB
+total: 967.60 MB</t>
+        </is>
+      </c>
+      <c r="G9" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G7" s="14" t="inlineStr">
+      <c r="H9" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H7" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I7" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>Q10</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C8" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D8" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E8" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F8" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G8" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H8" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I8" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="36" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>Q12</t>
-        </is>
-      </c>
-      <c r="B9" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C9" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D9" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E9" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F9" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G9" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H9" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I9" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="I9" s="13" t="inlineStr">
+        <is>
+          <t>shipmode: 239.94 MB
+receiptdate: 239.94 MB
+total: 479.89 MB</t>
         </is>
       </c>
     </row>
@@ -4525,7 +5459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4720,12 +5654,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>WAH</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ComBit</t>
+          <t>WAH (FastBit)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -4734,7 +5668,7 @@
         </is>
       </c>
       <c r="E8" s="15" t="n">
-        <v>11035.48</v>
+        <v>1732.932</v>
       </c>
     </row>
     <row r="9">
@@ -4745,12 +5679,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>CRoaring</t>
+          <t>ComBit</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -4759,7 +5693,7 @@
         </is>
       </c>
       <c r="E9" s="15" t="n">
-        <v>498.421</v>
+        <v>11035.48</v>
       </c>
     </row>
     <row r="10">
@@ -4770,12 +5704,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CRR</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CRoaring+Run</t>
+          <t>CRoaring</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -4784,23 +5718,23 @@
         </is>
       </c>
       <c r="E10" s="15" t="n">
-        <v>395.597</v>
+        <v>498.421</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Q4</t>
+          <t>Q3</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>CRR</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ComBit</t>
+          <t>CRoaring+Run</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -4809,23 +5743,23 @@
         </is>
       </c>
       <c r="E11" s="15" t="n">
-        <v>4448.84</v>
+        <v>395.597</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Q4</t>
+          <t>Q3</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>EW</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>CRoaring</t>
+          <t>EWAH</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -4834,23 +5768,23 @@
         </is>
       </c>
       <c r="E12" s="15" t="n">
-        <v>359.978</v>
+        <v>1287.01</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Q4</t>
+          <t>Q3</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CRR</t>
+          <t>CON</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CRoaring+Run</t>
+          <t>Concise</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -4859,23 +5793,23 @@
         </is>
       </c>
       <c r="E13" s="15" t="n">
-        <v>257.154</v>
+        <v>479.888</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Q5</t>
+          <t>Q4</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>WAH</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ComBit</t>
+          <t>WAH (FastBit)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -4884,23 +5818,23 @@
         </is>
       </c>
       <c r="E14" s="15" t="n">
-        <v>17624.84</v>
+        <v>1265.8</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Q5</t>
+          <t>Q4</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>CRoaring</t>
+          <t>ComBit</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -4909,23 +5843,23 @@
         </is>
       </c>
       <c r="E15" s="15" t="n">
-        <v>832.8140000000001</v>
+        <v>4448.84</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Q5</t>
+          <t>Q4</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CRR</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CRoaring+Run</t>
+          <t>CRoaring</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -4934,23 +5868,23 @@
         </is>
       </c>
       <c r="E16" s="15" t="n">
-        <v>729.99</v>
+        <v>359.978</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Q5</t>
+          <t>Q4</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>EW</t>
+          <t>CRR</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>EWAH</t>
+          <t>CRoaring+Run</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -4959,23 +5893,23 @@
         </is>
       </c>
       <c r="E17" s="15" t="n">
-        <v>1325.591</v>
+        <v>257.154</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Q5</t>
+          <t>Q4</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CON</t>
+          <t>EW</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Concise</t>
+          <t>EWAH</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -4984,23 +5918,23 @@
         </is>
       </c>
       <c r="E18" s="15" t="n">
-        <v>479.888</v>
+        <v>365.622</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Q6</t>
+          <t>Q4</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>WAH</t>
+          <t>CON</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>WAH (FastBit)</t>
+          <t>Concise</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -5009,23 +5943,23 @@
         </is>
       </c>
       <c r="E19" s="15" t="n">
-        <v>412.1922</v>
+        <v>239.944</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Q6</t>
+          <t>Q5</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>WAH</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ComBit</t>
+          <t>WAH (FastBit)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -5034,23 +5968,23 @@
         </is>
       </c>
       <c r="E20" s="15" t="n">
-        <v>555.4544000000001</v>
+        <v>1753.143</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Q6</t>
+          <t>Q5</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>CRoaring</t>
+          <t>ComBit</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -5059,23 +5993,23 @@
         </is>
       </c>
       <c r="E21" s="15" t="n">
-        <v>560.6653</v>
+        <v>17624.84</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Q6</t>
+          <t>Q5</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CRR</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>CRoaring+Run</t>
+          <t>CRoaring</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -5084,23 +6018,23 @@
         </is>
       </c>
       <c r="E22" s="15" t="n">
-        <v>255.4297</v>
+        <v>832.8140000000001</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Q6</t>
+          <t>Q5</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>EW</t>
+          <t>CRR</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>EWAH</t>
+          <t>CRoaring+Run</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -5109,23 +6043,23 @@
         </is>
       </c>
       <c r="E23" s="15" t="n">
-        <v>481.4368</v>
+        <v>729.99</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Q6</t>
+          <t>Q5</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CON</t>
+          <t>EW</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Concise</t>
+          <t>EWAH</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -5134,23 +6068,23 @@
         </is>
       </c>
       <c r="E24" s="15" t="n">
-        <v>719.832</v>
+        <v>1325.591</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Q14</t>
+          <t>Q5</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>WAH</t>
+          <t>CON</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>WAH (FastBit)</t>
+          <t>Concise</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -5159,23 +6093,23 @@
         </is>
       </c>
       <c r="E25" s="15" t="n">
-        <v>467.132</v>
+        <v>479.888</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Q14</t>
+          <t>Q6</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>WAH</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ComBit</t>
+          <t>WAH (FastBit)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -5184,23 +6118,23 @@
         </is>
       </c>
       <c r="E26" s="15" t="n">
-        <v>6586.64</v>
+        <v>412.1922</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Q14</t>
+          <t>Q6</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>CRoaring</t>
+          <t>ComBit</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -5209,23 +6143,23 @@
         </is>
       </c>
       <c r="E27" s="15" t="n">
-        <v>138.443</v>
+        <v>555.4544000000001</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Q14</t>
+          <t>Q6</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CRR</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>CRoaring+Run</t>
+          <t>CRoaring</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -5234,23 +6168,23 @@
         </is>
       </c>
       <c r="E28" s="15" t="n">
-        <v>138.443</v>
+        <v>560.6653</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Q14</t>
+          <t>Q6</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>EW</t>
+          <t>CRR</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>EWAH</t>
+          <t>CRoaring+Run</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -5259,23 +6193,23 @@
         </is>
       </c>
       <c r="E29" s="15" t="n">
-        <v>921.388</v>
+        <v>255.4297</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Q14</t>
+          <t>Q6</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CON</t>
+          <t>EW</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Concise</t>
+          <t>EWAH</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -5284,63 +6218,63 @@
         </is>
       </c>
       <c r="E30" s="15" t="n">
-        <v>239.944</v>
+        <v>481.4368</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Q15</t>
+          <t>Q6</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>CON</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ComBit</t>
+          <t>Concise</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>total</t>
         </is>
       </c>
       <c r="E31" s="15" t="n">
-        <v>2.23346688</v>
+        <v>719.832</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Q15</t>
+          <t>Q8</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>WAH</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ComBit</t>
+          <t>WAH (FastBit)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>total</t>
         </is>
       </c>
       <c r="E32" s="15" t="n">
-        <v>2.2020096</v>
+        <v>1897.681</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Q15</t>
+          <t>Q8</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -5355,52 +6289,52 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>L3</t>
+          <t>total</t>
         </is>
       </c>
       <c r="E33" s="15" t="n">
-        <v>2.01326592</v>
+        <v>18016.14</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Q15</t>
+          <t>Q8</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ComBit</t>
+          <t>CRoaring</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>L4</t>
+          <t>total</t>
         </is>
       </c>
       <c r="E34" s="15" t="n">
-        <v>1.33169152</v>
+        <v>968.067</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Q15</t>
+          <t>Q8</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>CRR</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ComBit</t>
+          <t>CRoaring+Run</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -5409,23 +6343,23 @@
         </is>
       </c>
       <c r="E35" s="15" t="n">
-        <v>7.790919679999999</v>
+        <v>865.2430000000001</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Q17</t>
+          <t>Q8</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>WAH</t>
+          <t>EW</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>WAH (FastBit)</t>
+          <t>EWAH</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -5434,23 +6368,23 @@
         </is>
       </c>
       <c r="E36" s="15" t="n">
-        <v>631.881</v>
+        <v>1341.368</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Q17</t>
+          <t>Q8</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>CON</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ComBit</t>
+          <t>Concise</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -5459,23 +6393,23 @@
         </is>
       </c>
       <c r="E37" s="15" t="n">
-        <v>13567.3</v>
+        <v>479.888</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Q17</t>
+          <t>Q10</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>WAH</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>CRoaring</t>
+          <t>WAH (FastBit)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -5484,23 +6418,23 @@
         </is>
       </c>
       <c r="E38" s="15" t="n">
-        <v>608.0890000000001</v>
+        <v>1289.018</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Q17</t>
+          <t>Q10</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>CRR</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>CRoaring+Run</t>
+          <t>ComBit</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -5509,23 +6443,23 @@
         </is>
       </c>
       <c r="E39" s="15" t="n">
-        <v>608.0890000000001</v>
+        <v>4478.6165</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Q17</t>
+          <t>Q10</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>EW</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>EWAH</t>
+          <t>CRoaring</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -5534,23 +6468,23 @@
         </is>
       </c>
       <c r="E40" s="15" t="n">
-        <v>975.746</v>
+        <v>382.5116</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Q17</t>
+          <t>Q10</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>CON</t>
+          <t>CRR</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Concise</t>
+          <t>CRoaring+Run</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -5559,23 +6493,23 @@
         </is>
       </c>
       <c r="E41" s="15" t="n">
-        <v>239.944</v>
+        <v>279.6851</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Q19</t>
+          <t>Q10</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>WAH</t>
+          <t>EW</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>WAH (FastBit)</t>
+          <t>EWAH</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -5584,23 +6518,23 @@
         </is>
       </c>
       <c r="E42" s="15" t="n">
-        <v>77.3993</v>
+        <v>388.1168</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Q19</t>
+          <t>Q10</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>CON</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>ComBit</t>
+          <t>Concise</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -5609,23 +6543,23 @@
         </is>
       </c>
       <c r="E43" s="15" t="n">
-        <v>100.6633</v>
+        <v>479.888</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Q19</t>
+          <t>Q12</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>WAH</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>CRoaring</t>
+          <t>WAH (FastBit)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -5634,23 +6568,23 @@
         </is>
       </c>
       <c r="E44" s="15" t="n">
-        <v>75.1007</v>
+        <v>514.1715</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Q19</t>
+          <t>Q12</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>CRR</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>CRoaring+Run</t>
+          <t>ComBit</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -5659,23 +6593,23 @@
         </is>
       </c>
       <c r="E45" s="15" t="n">
-        <v>75.1007</v>
+        <v>6651.326</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Q19</t>
+          <t>Q12</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>EW</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>EWAH</t>
+          <t>CRoaring</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -5684,31 +6618,656 @@
         </is>
       </c>
       <c r="E46" s="15" t="n">
-        <v>74.98269999999999</v>
+        <v>183.5719</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
+          <t>Q12</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>CRR</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>CRoaring+Run</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E47" s="15" t="n">
+        <v>183.5719</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Q12</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>EW</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>EWAH</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E48" s="15" t="n">
+        <v>967.6016</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Q12</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>CON</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Concise</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E49" s="15" t="n">
+        <v>479.888</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Q14</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>WAH</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>WAH (FastBit)</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E50" s="15" t="n">
+        <v>467.132</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Q14</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>ComBit</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E51" s="15" t="n">
+        <v>6586.64</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Q14</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>CRoaring</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E52" s="15" t="n">
+        <v>138.443</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Q14</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>CRR</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>CRoaring+Run</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E53" s="15" t="n">
+        <v>138.443</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Q14</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>EW</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>EWAH</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E54" s="15" t="n">
+        <v>921.388</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Q14</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>CON</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Concise</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E55" s="15" t="n">
+        <v>239.944</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Q15</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>ComBit</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="E56" s="15" t="n">
+        <v>2.23346688</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Q15</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>ComBit</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="E57" s="15" t="n">
+        <v>2.2020096</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Q15</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>ComBit</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="E58" s="15" t="n">
+        <v>2.01326592</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Q15</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>ComBit</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="E59" s="15" t="n">
+        <v>1.33169152</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Q15</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>ComBit</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E60" s="15" t="n">
+        <v>7.790919679999999</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Q17</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>WAH</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>WAH (FastBit)</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E61" s="15" t="n">
+        <v>631.881</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Q17</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>ComBit</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E62" s="15" t="n">
+        <v>13567.3</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Q17</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>CRoaring</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E63" s="15" t="n">
+        <v>608.0890000000001</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Q17</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>CRR</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>CRoaring+Run</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E64" s="15" t="n">
+        <v>608.0890000000001</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Q17</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>EW</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>EWAH</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E65" s="15" t="n">
+        <v>975.746</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Q17</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>CON</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Concise</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E66" s="15" t="n">
+        <v>239.944</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
           <t>Q19</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>WAH</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>WAH (FastBit)</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E67" s="15" t="n">
+        <v>77.3993</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Q19</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>ComBit</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E68" s="15" t="n">
+        <v>100.6633</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Q19</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>CRoaring</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E69" s="15" t="n">
+        <v>75.1007</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Q19</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>CRR</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>CRoaring+Run</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E70" s="15" t="n">
+        <v>75.1007</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Q19</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>EW</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>EWAH</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E71" s="15" t="n">
+        <v>74.98269999999999</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Q19</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
         <is>
           <t>CON</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C72" t="inlineStr">
         <is>
           <t>Concise</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D72" t="inlineStr">
         <is>
           <t>total</t>
         </is>
       </c>
-      <c r="E47" s="15" t="n">
+      <c r="E72" s="15" t="n">
         <v>479.888</v>
       </c>
     </row>
@@ -5839,7 +7398,7 @@
         </is>
       </c>
       <c r="B3" s="16" t="n">
-        <v>466.970216</v>
+        <v>1732.932</v>
       </c>
       <c r="C3" s="16" t="n">
         <v>11035.48</v>
@@ -5851,20 +7410,16 @@
         <v>395.597</v>
       </c>
       <c r="F3" s="16" t="n">
-        <v>921.428872</v>
+        <v>1287.01</v>
       </c>
       <c r="G3" s="17" t="n"/>
       <c r="H3" s="17" t="n"/>
-      <c r="I3" s="17" t="n"/>
-      <c r="J3" s="15" t="n">
-        <v>1388.4</v>
-      </c>
+      <c r="I3" s="16" t="n">
+        <v>479.888</v>
+      </c>
+      <c r="J3" s="15" t="n"/>
       <c r="K3" s="15" t="n"/>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>symlinked share with another Q</t>
-        </is>
-      </c>
+      <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
@@ -5873,7 +7428,7 @@
         </is>
       </c>
       <c r="B4" s="16" t="n">
-        <v>14.210456</v>
+        <v>1265.8</v>
       </c>
       <c r="C4" s="16" t="n">
         <v>4448.84</v>
@@ -5885,14 +7440,14 @@
         <v>257.154</v>
       </c>
       <c r="F4" s="16" t="n">
-        <v>18.318512</v>
+        <v>365.622</v>
       </c>
       <c r="G4" s="17" t="n"/>
       <c r="H4" s="17" t="n"/>
-      <c r="I4" s="17" t="n"/>
-      <c r="J4" s="15" t="n">
-        <v>32.53</v>
-      </c>
+      <c r="I4" s="16" t="n">
+        <v>239.944</v>
+      </c>
+      <c r="J4" s="15" t="n"/>
       <c r="K4" s="15" t="n"/>
       <c r="L4" t="inlineStr"/>
     </row>
@@ -5903,7 +7458,7 @@
         </is>
       </c>
       <c r="B5" s="16" t="n">
-        <v>0.000125</v>
+        <v>1753.143</v>
       </c>
       <c r="C5" s="16" t="n">
         <v>17624.84</v>
@@ -5922,9 +7477,7 @@
       <c r="I5" s="16" t="n">
         <v>479.888</v>
       </c>
-      <c r="J5" s="15" t="n">
-        <v>0</v>
-      </c>
+      <c r="J5" s="15" t="n"/>
       <c r="K5" s="15" t="n"/>
       <c r="L5" t="inlineStr"/>
     </row>
@@ -5964,14 +7517,26 @@
           <t>Q8</t>
         </is>
       </c>
-      <c r="B7" s="17" t="n"/>
-      <c r="C7" s="17" t="n"/>
-      <c r="D7" s="17" t="n"/>
-      <c r="E7" s="17" t="n"/>
-      <c r="F7" s="17" t="n"/>
+      <c r="B7" s="16" t="n">
+        <v>1897.681</v>
+      </c>
+      <c r="C7" s="16" t="n">
+        <v>18016.14</v>
+      </c>
+      <c r="D7" s="16" t="n">
+        <v>968.067</v>
+      </c>
+      <c r="E7" s="16" t="n">
+        <v>865.2430000000001</v>
+      </c>
+      <c r="F7" s="16" t="n">
+        <v>1341.368</v>
+      </c>
       <c r="G7" s="17" t="n"/>
       <c r="H7" s="17" t="n"/>
-      <c r="I7" s="17" t="n"/>
+      <c r="I7" s="16" t="n">
+        <v>479.888</v>
+      </c>
       <c r="J7" s="15" t="n"/>
       <c r="K7" s="15" t="n"/>
       <c r="L7" t="inlineStr"/>
@@ -5982,14 +7547,26 @@
           <t>Q10</t>
         </is>
       </c>
-      <c r="B8" s="17" t="n"/>
-      <c r="C8" s="17" t="n"/>
-      <c r="D8" s="17" t="n"/>
-      <c r="E8" s="17" t="n"/>
-      <c r="F8" s="17" t="n"/>
+      <c r="B8" s="16" t="n">
+        <v>1289.018</v>
+      </c>
+      <c r="C8" s="16" t="n">
+        <v>4478.6165</v>
+      </c>
+      <c r="D8" s="16" t="n">
+        <v>382.5116</v>
+      </c>
+      <c r="E8" s="16" t="n">
+        <v>279.6851</v>
+      </c>
+      <c r="F8" s="16" t="n">
+        <v>388.1168</v>
+      </c>
       <c r="G8" s="17" t="n"/>
       <c r="H8" s="17" t="n"/>
-      <c r="I8" s="17" t="n"/>
+      <c r="I8" s="16" t="n">
+        <v>479.888</v>
+      </c>
       <c r="J8" s="15" t="n"/>
       <c r="K8" s="15" t="n"/>
       <c r="L8" t="inlineStr"/>
@@ -6001,26 +7578,26 @@
         </is>
       </c>
       <c r="B9" s="16" t="n">
-        <v>101.8691584</v>
+        <v>514.1715</v>
       </c>
       <c r="C9" s="16" t="n">
-        <v>105.70694656</v>
+        <v>6651.326</v>
       </c>
       <c r="D9" s="16" t="n">
-        <v>50.91885056</v>
+        <v>183.5719</v>
       </c>
       <c r="E9" s="16" t="n">
-        <v>50.91885056</v>
+        <v>183.5719</v>
       </c>
       <c r="F9" s="16" t="n">
-        <v>169.869312</v>
+        <v>967.6016</v>
       </c>
       <c r="G9" s="17" t="n"/>
       <c r="H9" s="17" t="n"/>
-      <c r="I9" s="17" t="n"/>
-      <c r="J9" s="15" t="n">
-        <v>428.36</v>
-      </c>
+      <c r="I9" s="16" t="n">
+        <v>479.888</v>
+      </c>
+      <c r="J9" s="15" t="n"/>
       <c r="K9" s="15" t="n"/>
       <c r="L9" t="inlineStr"/>
     </row>
@@ -6255,7 +7832,9 @@
           <t>Q3</t>
         </is>
       </c>
-      <c r="B3" s="18" t="n"/>
+      <c r="B3" s="20" t="n">
+        <v>302114</v>
+      </c>
       <c r="C3" s="18" t="n"/>
       <c r="D3" s="18" t="n"/>
       <c r="E3" s="18" t="n"/>
@@ -6272,7 +7851,9 @@
           <t>Q4</t>
         </is>
       </c>
-      <c r="B4" s="18" t="n"/>
+      <c r="B4" s="20" t="n">
+        <v>2294856</v>
+      </c>
       <c r="C4" s="18" t="n"/>
       <c r="D4" s="18" t="n"/>
       <c r="E4" s="18" t="n"/>
@@ -6289,7 +7870,9 @@
           <t>Q5</t>
         </is>
       </c>
-      <c r="B5" s="18" t="n"/>
+      <c r="B5" s="20" t="n">
+        <v>72985</v>
+      </c>
       <c r="C5" s="18" t="n"/>
       <c r="D5" s="18" t="n"/>
       <c r="E5" s="18" t="n"/>
@@ -6323,7 +7906,9 @@
           <t>Q8</t>
         </is>
       </c>
-      <c r="B7" s="18" t="n"/>
+      <c r="B7" s="20" t="n">
+        <v>24254</v>
+      </c>
       <c r="C7" s="18" t="n"/>
       <c r="D7" s="18" t="n"/>
       <c r="E7" s="18" t="n"/>
@@ -6340,7 +7925,9 @@
           <t>Q10</t>
         </is>
       </c>
-      <c r="B8" s="18" t="n"/>
+      <c r="B8" s="20" t="n">
+        <v>1147084</v>
+      </c>
       <c r="C8" s="18" t="n"/>
       <c r="D8" s="18" t="n"/>
       <c r="E8" s="18" t="n"/>
@@ -6357,7 +7944,9 @@
           <t>Q12</t>
         </is>
       </c>
-      <c r="B9" s="18" t="n"/>
+      <c r="B9" s="20" t="n">
+        <v>2600101</v>
+      </c>
       <c r="C9" s="18" t="n"/>
       <c r="D9" s="18" t="n"/>
       <c r="E9" s="18" t="n"/>

</xml_diff>

<commit_message>
Q3: use shipdate_BPE for DDC + CRoaring shipdate
</commit_message>
<xml_diff>
--- a/bm_resultL4.xlsx
+++ b/bm_resultL4.xlsx
@@ -1727,24 +1727,24 @@
         </is>
       </c>
       <c r="B3" s="8" t="n">
-        <v>3567.423</v>
+        <v>3545.4935</v>
       </c>
       <c r="C3" s="8" t="n">
-        <v>2335.4595</v>
+        <v>1447.822</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>1653.717</v>
+        <v>1333.2165</v>
       </c>
       <c r="E3" s="8" t="n">
-        <v>1379.7845</v>
+        <v>1294.4165</v>
       </c>
       <c r="F3" s="8" t="n">
-        <v>4120.672</v>
+        <v>4480.026</v>
       </c>
       <c r="G3" s="9" t="n"/>
       <c r="H3" s="9" t="n"/>
       <c r="I3" s="8" t="n">
-        <v>4953.748</v>
+        <v>4960.3875</v>
       </c>
       <c r="J3" s="9" t="n"/>
     </row>
@@ -2384,24 +2384,24 @@
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>22.0545</v>
+        <v>22.246</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>23.8995</v>
+        <v>24.1925</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>22.397</v>
+        <v>23.115</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>22.1255</v>
+        <v>23.521</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>21.9745</v>
+        <v>22.04</v>
       </c>
       <c r="H6" s="9" t="n"/>
       <c r="I6" s="9" t="n"/>
       <c r="J6" s="8" t="n">
-        <v>22.0185</v>
+        <v>21.9655</v>
       </c>
     </row>
     <row r="7">
@@ -2412,24 +2412,24 @@
         </is>
       </c>
       <c r="C7" s="8" t="n">
-        <v>2192.3795</v>
+        <v>2168.553</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>1297.014</v>
+        <v>1301.8655</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>1205.36</v>
+        <v>1201.8255</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>1144.781</v>
+        <v>1171.5375</v>
       </c>
       <c r="G7" s="8" t="n">
-        <v>1091.6</v>
+        <v>1305.4145</v>
       </c>
       <c r="H7" s="9" t="n"/>
       <c r="I7" s="9" t="n"/>
       <c r="J7" s="8" t="n">
-        <v>1208.4175</v>
+        <v>1219.989</v>
       </c>
     </row>
     <row r="8">
@@ -2440,24 +2440,24 @@
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>1255.111</v>
+        <v>1256.6725</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>923.3945</v>
+        <v>32.684</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>337.6395</v>
+        <v>19.96</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>124.2565</v>
+        <v>11.033</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>2914.332</v>
+        <v>3059.743</v>
       </c>
       <c r="H8" s="9" t="n"/>
       <c r="I8" s="9" t="n"/>
       <c r="J8" s="8" t="n">
-        <v>3609.2085</v>
+        <v>3600.548</v>
       </c>
     </row>
     <row r="9">
@@ -2468,24 +2468,24 @@
         </is>
       </c>
       <c r="C9" s="8" t="n">
-        <v>14.2595</v>
+        <v>14.2075</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>8.8705</v>
+        <v>7.976</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>5.4845</v>
+        <v>5.2735</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>5.367</v>
+        <v>5.4175</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>9.938499999999999</v>
+        <v>10.0405</v>
       </c>
       <c r="H9" s="9" t="n"/>
       <c r="I9" s="9" t="n"/>
       <c r="J9" s="8" t="n">
-        <v>28.4905</v>
+        <v>28.6695</v>
       </c>
     </row>
     <row r="10">
@@ -2496,24 +2496,24 @@
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>82.53</v>
+        <v>83.048</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>82.04949999999999</v>
+        <v>80.98099999999999</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>82.32550000000001</v>
+        <v>82.42449999999999</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>82.6075</v>
+        <v>83.0565</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>82.7615</v>
+        <v>82.706</v>
       </c>
       <c r="H10" s="9" t="n"/>
       <c r="I10" s="9" t="n"/>
       <c r="J10" s="8" t="n">
-        <v>83.559</v>
+        <v>89.315</v>
       </c>
     </row>
     <row r="11">
@@ -2524,24 +2524,24 @@
         </is>
       </c>
       <c r="C11" s="8" t="n">
-        <v>3567.423</v>
+        <v>3545.4935</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>2335.4595</v>
+        <v>1447.822</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>1653.717</v>
+        <v>1333.2165</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>1379.7845</v>
+        <v>1294.4165</v>
       </c>
       <c r="G11" s="8" t="n">
-        <v>4120.672</v>
+        <v>4480.026</v>
       </c>
       <c r="H11" s="9" t="n"/>
       <c r="I11" s="9" t="n"/>
       <c r="J11" s="8" t="n">
-        <v>4953.748</v>
+        <v>4960.3875</v>
       </c>
     </row>
     <row r="12">
@@ -4815,7 +4815,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="48" customHeight="1">
+    <row r="3" ht="62" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Q3</t>
@@ -4832,14 +4832,16 @@
         <is>
           <t>orderkey: 4448.84 MB
 shipdate: 6586.64 MB
-total: 11035.48 MB</t>
+shipdate_BPE: 188.47 MB
+total: 11223.95 MB</t>
         </is>
       </c>
       <c r="D3" s="13" t="inlineStr">
         <is>
           <t>orderkey: 359.98 MB
 shipdate: 138.44 MB
-total: 498.42 MB</t>
+shipdate_BPE: 354.33 MB
+total: 852.75 MB</t>
         </is>
       </c>
       <c r="E3" s="13" t="inlineStr">
@@ -5693,7 +5695,7 @@
         </is>
       </c>
       <c r="E9" s="15" t="n">
-        <v>11035.48</v>
+        <v>11223.952</v>
       </c>
     </row>
     <row r="10">
@@ -5718,7 +5720,7 @@
         </is>
       </c>
       <c r="E10" s="15" t="n">
-        <v>498.421</v>
+        <v>852.75</v>
       </c>
     </row>
     <row r="11">
@@ -7401,10 +7403,10 @@
         <v>1732.932</v>
       </c>
       <c r="C3" s="16" t="n">
-        <v>11035.48</v>
+        <v>11223.952</v>
       </c>
       <c r="D3" s="16" t="n">
-        <v>498.421</v>
+        <v>852.75</v>
       </c>
       <c r="E3" s="16" t="n">
         <v>395.597</v>

</xml_diff>

<commit_message>
SparseDDC::or_many: implement scatter-by-output-segment k-way OR
</commit_message>
<xml_diff>
--- a/bm_resultL4.xlsx
+++ b/bm_resultL4.xlsx
@@ -1727,24 +1727,24 @@
         </is>
       </c>
       <c r="B3" s="8" t="n">
-        <v>3545.4935</v>
+        <v>3603.054</v>
       </c>
       <c r="C3" s="8" t="n">
-        <v>1447.822</v>
+        <v>943.283</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>1333.2165</v>
+        <v>1325.1885</v>
       </c>
       <c r="E3" s="8" t="n">
-        <v>1294.4165</v>
+        <v>1282.534</v>
       </c>
       <c r="F3" s="8" t="n">
-        <v>4480.026</v>
+        <v>4583.751</v>
       </c>
       <c r="G3" s="9" t="n"/>
       <c r="H3" s="9" t="n"/>
       <c r="I3" s="8" t="n">
-        <v>4960.3875</v>
+        <v>4966.076</v>
       </c>
       <c r="J3" s="9" t="n"/>
     </row>
@@ -2384,24 +2384,24 @@
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>22.246</v>
+        <v>22.0915</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>24.1925</v>
+        <v>24.45</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>23.115</v>
+        <v>22.25</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>23.521</v>
+        <v>23.4705</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>22.04</v>
+        <v>21.995</v>
       </c>
       <c r="H6" s="9" t="n"/>
       <c r="I6" s="9" t="n"/>
       <c r="J6" s="8" t="n">
-        <v>21.9655</v>
+        <v>22.1495</v>
       </c>
     </row>
     <row r="7">
@@ -2412,24 +2412,24 @@
         </is>
       </c>
       <c r="C7" s="8" t="n">
-        <v>2168.553</v>
+        <v>2197.456</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>1301.8655</v>
+        <v>796.7605</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>1201.8255</v>
+        <v>1195.838</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>1171.5375</v>
+        <v>1159.9735</v>
       </c>
       <c r="G7" s="8" t="n">
-        <v>1305.4145</v>
+        <v>1299.308</v>
       </c>
       <c r="H7" s="9" t="n"/>
       <c r="I7" s="9" t="n"/>
       <c r="J7" s="8" t="n">
-        <v>1219.989</v>
+        <v>1226.864</v>
       </c>
     </row>
     <row r="8">
@@ -2440,24 +2440,24 @@
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>1256.6725</v>
+        <v>1277.042</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>32.684</v>
+        <v>34.0175</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>19.96</v>
+        <v>19.576</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>11.033</v>
+        <v>10.8475</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>3059.743</v>
+        <v>3171.57</v>
       </c>
       <c r="H8" s="9" t="n"/>
       <c r="I8" s="9" t="n"/>
       <c r="J8" s="8" t="n">
-        <v>3600.548</v>
+        <v>3605.0055</v>
       </c>
     </row>
     <row r="9">
@@ -2468,24 +2468,24 @@
         </is>
       </c>
       <c r="C9" s="8" t="n">
-        <v>14.2075</v>
+        <v>14.367</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>7.976</v>
+        <v>5.5065</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>5.2735</v>
+        <v>5.2325</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>5.4175</v>
+        <v>5.3295</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>10.0405</v>
+        <v>9.773</v>
       </c>
       <c r="H9" s="9" t="n"/>
       <c r="I9" s="9" t="n"/>
       <c r="J9" s="8" t="n">
-        <v>28.6695</v>
+        <v>28.5115</v>
       </c>
     </row>
     <row r="10">
@@ -2496,24 +2496,24 @@
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>83.048</v>
+        <v>83.1515</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>80.98099999999999</v>
+        <v>82.4295</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>82.42449999999999</v>
+        <v>82.315</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>83.0565</v>
+        <v>82.2825</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>82.706</v>
+        <v>82.645</v>
       </c>
       <c r="H10" s="9" t="n"/>
       <c r="I10" s="9" t="n"/>
       <c r="J10" s="8" t="n">
-        <v>89.315</v>
+        <v>82.99250000000001</v>
       </c>
     </row>
     <row r="11">
@@ -2524,24 +2524,24 @@
         </is>
       </c>
       <c r="C11" s="8" t="n">
-        <v>3545.4935</v>
+        <v>3603.054</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>1447.822</v>
+        <v>943.283</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>1333.2165</v>
+        <v>1325.1885</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>1294.4165</v>
+        <v>1282.534</v>
       </c>
       <c r="G11" s="8" t="n">
-        <v>4480.026</v>
+        <v>4583.751</v>
       </c>
       <c r="H11" s="9" t="n"/>
       <c r="I11" s="9" t="n"/>
       <c r="J11" s="8" t="n">
-        <v>4960.3875</v>
+        <v>4966.076</v>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
Q4 / Q5 / Q8 / Q10 /
</commit_message>
<xml_diff>
--- a/bm_resultL4.xlsx
+++ b/bm_resultL4.xlsx
@@ -1755,24 +1755,24 @@
         </is>
       </c>
       <c r="B4" s="8" t="n">
-        <v>1353.263</v>
+        <v>1372.8635</v>
       </c>
       <c r="C4" s="8" t="n">
-        <v>814.4745</v>
+        <v>710.62</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>1074.3785</v>
+        <v>720.902</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>703.89</v>
+        <v>711.241</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>897.4485</v>
+        <v>920.9405</v>
       </c>
       <c r="G4" s="9" t="n"/>
       <c r="H4" s="9" t="n"/>
       <c r="I4" s="8" t="n">
-        <v>977.87</v>
+        <v>987.221</v>
       </c>
       <c r="J4" s="9" t="n"/>
     </row>
@@ -1783,24 +1783,24 @@
         </is>
       </c>
       <c r="B5" s="8" t="n">
-        <v>3428.306</v>
+        <v>3420.4895</v>
       </c>
       <c r="C5" s="8" t="n">
-        <v>1284.302</v>
+        <v>1290.4755</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>3029.9815</v>
+        <v>1006.026</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>961.7535</v>
+        <v>930.6085</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>2879.6125</v>
+        <v>2943.378</v>
       </c>
       <c r="G5" s="9" t="n"/>
       <c r="H5" s="9" t="n"/>
       <c r="I5" s="8" t="n">
-        <v>3036.581</v>
+        <v>3056.4685</v>
       </c>
       <c r="J5" s="9" t="n"/>
     </row>
@@ -1839,24 +1839,24 @@
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>1705.5285</v>
+        <v>1707.148</v>
       </c>
       <c r="C7" s="8" t="n">
-        <v>795.7234999999999</v>
+        <v>718.393</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>954.004</v>
+        <v>1154.8775</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>932.015</v>
+        <v>1109.8655</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>1139.955</v>
+        <v>1132.7815</v>
       </c>
       <c r="G7" s="9" t="n"/>
       <c r="H7" s="9" t="n"/>
       <c r="I7" s="8" t="n">
-        <v>1241.548</v>
+        <v>1244.1125</v>
       </c>
       <c r="J7" s="9" t="n"/>
     </row>
@@ -1867,24 +1867,24 @@
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>1069.076</v>
+        <v>1044.876</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>512.638</v>
+        <v>431.346</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>602.7380000000001</v>
+        <v>628.7455</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>570.16</v>
+        <v>604.7910000000001</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>612.7025</v>
+        <v>719.223</v>
       </c>
       <c r="G8" s="9" t="n"/>
       <c r="H8" s="9" t="n"/>
       <c r="I8" s="8" t="n">
-        <v>700.9105</v>
+        <v>813.5465</v>
       </c>
       <c r="J8" s="9" t="n"/>
     </row>
@@ -1985,24 +1985,24 @@
         </is>
       </c>
       <c r="B12" s="8" t="n">
-        <v>470.2065</v>
+        <v>59.1735</v>
       </c>
       <c r="C12" s="8" t="n">
-        <v>57.8865</v>
+        <v>69.6125</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>60.9555</v>
+        <v>52.9695</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>56.889</v>
+        <v>55.96</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>485.102</v>
+        <v>59.709</v>
       </c>
       <c r="G12" s="9" t="n"/>
       <c r="H12" s="9" t="n"/>
       <c r="I12" s="8" t="n">
-        <v>537.5535</v>
+        <v>54.347</v>
       </c>
       <c r="J12" s="9" t="n"/>
     </row>
@@ -2556,24 +2556,24 @@
         </is>
       </c>
       <c r="C12" s="8" t="n">
-        <v>243.1965</v>
+        <v>248.096</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>242.0565</v>
+        <v>248.6595</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>242.959</v>
+        <v>244.94</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>245.6165</v>
+        <v>244.906</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>242.5845</v>
+        <v>254.489</v>
       </c>
       <c r="H12" s="9" t="n"/>
       <c r="I12" s="9" t="n"/>
       <c r="J12" s="8" t="n">
-        <v>243.836</v>
+        <v>245.92</v>
       </c>
     </row>
     <row r="13">
@@ -2584,24 +2584,24 @@
         </is>
       </c>
       <c r="C13" s="8" t="n">
-        <v>814.0235</v>
+        <v>825.231</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>277.59</v>
+        <v>160.1735</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>533.6075</v>
+        <v>179.194</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>160.3505</v>
+        <v>169.853</v>
       </c>
       <c r="G13" s="8" t="n">
-        <v>359.367</v>
+        <v>363.2235</v>
       </c>
       <c r="H13" s="9" t="n"/>
       <c r="I13" s="9" t="n"/>
       <c r="J13" s="8" t="n">
-        <v>438.502</v>
+        <v>440.3245</v>
       </c>
     </row>
     <row r="14">
@@ -2612,24 +2612,24 @@
         </is>
       </c>
       <c r="C14" s="8" t="n">
-        <v>235.28</v>
+        <v>237.7165</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>235.1395</v>
+        <v>237.1095</v>
       </c>
       <c r="E14" s="8" t="n">
-        <v>236.9025</v>
+        <v>237.7255</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>237.129</v>
+        <v>235.049</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>235.073</v>
+        <v>237.1875</v>
       </c>
       <c r="H14" s="9" t="n"/>
       <c r="I14" s="9" t="n"/>
       <c r="J14" s="8" t="n">
-        <v>234.8045</v>
+        <v>236.3645</v>
       </c>
     </row>
     <row r="15">
@@ -2640,24 +2640,24 @@
         </is>
       </c>
       <c r="C15" s="8" t="n">
-        <v>60.683</v>
+        <v>63.421</v>
       </c>
       <c r="D15" s="8" t="n">
-        <v>59.429</v>
+        <v>64.346</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>60.462</v>
+        <v>59.9845</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>60.418</v>
+        <v>61.601</v>
       </c>
       <c r="G15" s="8" t="n">
-        <v>60.707</v>
+        <v>63.959</v>
       </c>
       <c r="H15" s="9" t="n"/>
       <c r="I15" s="9" t="n"/>
       <c r="J15" s="8" t="n">
-        <v>60.6015</v>
+        <v>62.981</v>
       </c>
     </row>
     <row r="16">
@@ -2668,24 +2668,24 @@
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>1353.263</v>
+        <v>1372.8635</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>814.4745</v>
+        <v>710.62</v>
       </c>
       <c r="E16" s="8" t="n">
-        <v>1074.3785</v>
+        <v>720.902</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>703.89</v>
+        <v>711.241</v>
       </c>
       <c r="G16" s="8" t="n">
-        <v>897.4485</v>
+        <v>920.9405</v>
       </c>
       <c r="H16" s="9" t="n"/>
       <c r="I16" s="9" t="n"/>
       <c r="J16" s="8" t="n">
-        <v>977.87</v>
+        <v>987.221</v>
       </c>
     </row>
     <row r="17">
@@ -2700,24 +2700,24 @@
         </is>
       </c>
       <c r="C17" s="8" t="n">
-        <v>282.358</v>
+        <v>286.2415</v>
       </c>
       <c r="D17" s="8" t="n">
-        <v>279.9095</v>
+        <v>289.7485</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>279.82</v>
+        <v>316.9215</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>313.016</v>
+        <v>280.6995</v>
       </c>
       <c r="G17" s="8" t="n">
-        <v>301.22</v>
+        <v>290.349</v>
       </c>
       <c r="H17" s="9" t="n"/>
       <c r="I17" s="9" t="n"/>
       <c r="J17" s="8" t="n">
-        <v>283.585</v>
+        <v>287.2305</v>
       </c>
     </row>
     <row r="18">
@@ -2728,24 +2728,24 @@
         </is>
       </c>
       <c r="C18" s="8" t="n">
-        <v>3022.255</v>
+        <v>3010.6125</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>880.579</v>
+        <v>872.3145</v>
       </c>
       <c r="E18" s="8" t="n">
-        <v>2623.953</v>
+        <v>561.0415</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>523.522</v>
+        <v>527.3185</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>2453.86</v>
+        <v>2528.5685</v>
       </c>
       <c r="H18" s="9" t="n"/>
       <c r="I18" s="9" t="n"/>
       <c r="J18" s="8" t="n">
-        <v>2629.2995</v>
+        <v>2644.287</v>
       </c>
     </row>
     <row r="19">
@@ -2756,24 +2756,24 @@
         </is>
       </c>
       <c r="C19" s="8" t="n">
-        <v>123.0745</v>
+        <v>122.7625</v>
       </c>
       <c r="D19" s="8" t="n">
-        <v>123.813</v>
+        <v>121.8615</v>
       </c>
       <c r="E19" s="8" t="n">
-        <v>123.5125</v>
+        <v>126.5285</v>
       </c>
       <c r="F19" s="8" t="n">
-        <v>125.7185</v>
+        <v>122.011</v>
       </c>
       <c r="G19" s="8" t="n">
-        <v>124.387</v>
+        <v>124.3115</v>
       </c>
       <c r="H19" s="9" t="n"/>
       <c r="I19" s="9" t="n"/>
       <c r="J19" s="8" t="n">
-        <v>123.2775</v>
+        <v>123.1775</v>
       </c>
     </row>
     <row r="20">
@@ -2784,24 +2784,24 @@
         </is>
       </c>
       <c r="C20" s="8" t="n">
-        <v>3428.306</v>
+        <v>3420.4895</v>
       </c>
       <c r="D20" s="8" t="n">
-        <v>1284.302</v>
+        <v>1290.4755</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>3029.9815</v>
+        <v>1006.026</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>961.7535</v>
+        <v>930.6085</v>
       </c>
       <c r="G20" s="8" t="n">
-        <v>2879.6125</v>
+        <v>2943.378</v>
       </c>
       <c r="H20" s="9" t="n"/>
       <c r="I20" s="9" t="n"/>
       <c r="J20" s="8" t="n">
-        <v>3036.581</v>
+        <v>3056.4685</v>
       </c>
     </row>
     <row r="21">
@@ -2988,24 +2988,24 @@
         </is>
       </c>
       <c r="C27" s="8" t="n">
-        <v>88.489</v>
+        <v>89.1935</v>
       </c>
       <c r="D27" s="8" t="n">
-        <v>88.1905</v>
+        <v>89.0235</v>
       </c>
       <c r="E27" s="8" t="n">
-        <v>88.1785</v>
+        <v>140.038</v>
       </c>
       <c r="F27" s="8" t="n">
-        <v>88.3385</v>
+        <v>138.958</v>
       </c>
       <c r="G27" s="8" t="n">
-        <v>88.511</v>
+        <v>89.1425</v>
       </c>
       <c r="H27" s="9" t="n"/>
       <c r="I27" s="9" t="n"/>
       <c r="J27" s="8" t="n">
-        <v>88.45950000000001</v>
+        <v>89.31</v>
       </c>
     </row>
     <row r="28">
@@ -3016,24 +3016,24 @@
         </is>
       </c>
       <c r="C28" s="8" t="n">
-        <v>354.0105</v>
+        <v>355.2395</v>
       </c>
       <c r="D28" s="8" t="n">
-        <v>344.3415</v>
+        <v>352.3605</v>
       </c>
       <c r="E28" s="8" t="n">
-        <v>357.294</v>
+        <v>437.408</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>355.584</v>
+        <v>428.826</v>
       </c>
       <c r="G28" s="8" t="n">
-        <v>352.364</v>
+        <v>351.9555</v>
       </c>
       <c r="H28" s="9" t="n"/>
       <c r="I28" s="9" t="n"/>
       <c r="J28" s="8" t="n">
-        <v>356.307</v>
+        <v>355.8005</v>
       </c>
     </row>
     <row r="29">
@@ -3044,24 +3044,24 @@
         </is>
       </c>
       <c r="C29" s="8" t="n">
-        <v>1233.4145</v>
+        <v>1233.663</v>
       </c>
       <c r="D29" s="8" t="n">
-        <v>333.2545</v>
+        <v>248.3075</v>
       </c>
       <c r="E29" s="8" t="n">
-        <v>479.129</v>
+        <v>540.5365</v>
       </c>
       <c r="F29" s="8" t="n">
-        <v>458.864</v>
+        <v>511.323</v>
       </c>
       <c r="G29" s="8" t="n">
-        <v>668.746</v>
+        <v>659.9450000000001</v>
       </c>
       <c r="H29" s="9" t="n"/>
       <c r="I29" s="9" t="n"/>
       <c r="J29" s="8" t="n">
-        <v>768.0765</v>
+        <v>769.6325000000001</v>
       </c>
     </row>
     <row r="30">
@@ -3072,24 +3072,24 @@
         </is>
       </c>
       <c r="C30" s="8" t="n">
-        <v>29.0035</v>
+        <v>28.838</v>
       </c>
       <c r="D30" s="8" t="n">
-        <v>29.9085</v>
+        <v>29.663</v>
       </c>
       <c r="E30" s="8" t="n">
-        <v>29.2105</v>
+        <v>30.732</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>29.057</v>
+        <v>30.7325</v>
       </c>
       <c r="G30" s="8" t="n">
-        <v>29.146</v>
+        <v>28.8075</v>
       </c>
       <c r="H30" s="9" t="n"/>
       <c r="I30" s="9" t="n"/>
       <c r="J30" s="8" t="n">
-        <v>29.179</v>
+        <v>29.0645</v>
       </c>
     </row>
     <row r="31">
@@ -3116,24 +3116,24 @@
         </is>
       </c>
       <c r="C32" s="8" t="n">
-        <v>1705.5285</v>
+        <v>1707.148</v>
       </c>
       <c r="D32" s="8" t="n">
-        <v>795.7234999999999</v>
+        <v>718.393</v>
       </c>
       <c r="E32" s="8" t="n">
-        <v>954.004</v>
+        <v>1154.8775</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>932.015</v>
+        <v>1109.8655</v>
       </c>
       <c r="G32" s="8" t="n">
-        <v>1139.955</v>
+        <v>1132.7815</v>
       </c>
       <c r="H32" s="9" t="n"/>
       <c r="I32" s="9" t="n"/>
       <c r="J32" s="8" t="n">
-        <v>1241.548</v>
+        <v>1244.1125</v>
       </c>
     </row>
     <row r="33">
@@ -3148,24 +3148,24 @@
         </is>
       </c>
       <c r="C33" s="8" t="n">
-        <v>93.4965</v>
+        <v>91.0385</v>
       </c>
       <c r="D33" s="8" t="n">
-        <v>92.741</v>
+        <v>89.5325</v>
       </c>
       <c r="E33" s="8" t="n">
-        <v>99.801</v>
+        <v>92.1405</v>
       </c>
       <c r="F33" s="8" t="n">
-        <v>92.27249999999999</v>
+        <v>90.604</v>
       </c>
       <c r="G33" s="8" t="n">
-        <v>93.116</v>
+        <v>99.27500000000001</v>
       </c>
       <c r="H33" s="9" t="n"/>
       <c r="I33" s="9" t="n"/>
       <c r="J33" s="8" t="n">
-        <v>92.4225</v>
+        <v>99.30249999999999</v>
       </c>
     </row>
     <row r="34">
@@ -3176,24 +3176,24 @@
         </is>
       </c>
       <c r="C34" s="8" t="n">
-        <v>714.7265</v>
+        <v>700.961</v>
       </c>
       <c r="D34" s="8" t="n">
-        <v>191.4745</v>
+        <v>112.4955</v>
       </c>
       <c r="E34" s="8" t="n">
-        <v>273.2755</v>
+        <v>312.994</v>
       </c>
       <c r="F34" s="8" t="n">
-        <v>257.7525</v>
+        <v>292.641</v>
       </c>
       <c r="G34" s="8" t="n">
-        <v>276.625</v>
+        <v>386.91</v>
       </c>
       <c r="H34" s="9" t="n"/>
       <c r="I34" s="9" t="n"/>
       <c r="J34" s="8" t="n">
-        <v>354.0475</v>
+        <v>458.493</v>
       </c>
     </row>
     <row r="35">
@@ -3207,21 +3207,21 @@
         <v>0.002</v>
       </c>
       <c r="D35" s="8" t="n">
-        <v>2.963</v>
+        <v>2.8435</v>
       </c>
       <c r="E35" s="8" t="n">
-        <v>0.9615</v>
+        <v>0.952</v>
       </c>
       <c r="F35" s="8" t="n">
-        <v>0.9425</v>
+        <v>0.9235</v>
       </c>
       <c r="G35" s="8" t="n">
-        <v>1.663</v>
+        <v>1.672</v>
       </c>
       <c r="H35" s="9" t="n"/>
       <c r="I35" s="9" t="n"/>
       <c r="J35" s="8" t="n">
-        <v>1.4505</v>
+        <v>1.3795</v>
       </c>
     </row>
     <row r="36">
@@ -3232,24 +3232,24 @@
         </is>
       </c>
       <c r="C36" s="8" t="n">
-        <v>37.551</v>
+        <v>37.1105</v>
       </c>
       <c r="D36" s="8" t="n">
-        <v>11.663</v>
+        <v>11.608</v>
       </c>
       <c r="E36" s="8" t="n">
-        <v>8.172000000000001</v>
+        <v>8.598000000000001</v>
       </c>
       <c r="F36" s="8" t="n">
-        <v>7.646</v>
+        <v>8.893000000000001</v>
       </c>
       <c r="G36" s="8" t="n">
-        <v>19.408</v>
+        <v>18.4955</v>
       </c>
       <c r="H36" s="9" t="n"/>
       <c r="I36" s="9" t="n"/>
       <c r="J36" s="8" t="n">
-        <v>40.8425</v>
+        <v>39.7435</v>
       </c>
     </row>
     <row r="37">
@@ -3260,24 +3260,24 @@
         </is>
       </c>
       <c r="C37" s="8" t="n">
-        <v>212.73</v>
+        <v>208.238</v>
       </c>
       <c r="D37" s="8" t="n">
-        <v>206.2135</v>
+        <v>207.7695</v>
       </c>
       <c r="E37" s="8" t="n">
-        <v>211.9825</v>
+        <v>206.6585</v>
       </c>
       <c r="F37" s="8" t="n">
-        <v>203.9285</v>
+        <v>203.825</v>
       </c>
       <c r="G37" s="8" t="n">
-        <v>214.615</v>
+        <v>204.854</v>
       </c>
       <c r="H37" s="9" t="n"/>
       <c r="I37" s="9" t="n"/>
       <c r="J37" s="8" t="n">
-        <v>205.6075</v>
+        <v>206.15</v>
       </c>
     </row>
     <row r="38">
@@ -3288,24 +3288,24 @@
         </is>
       </c>
       <c r="C38" s="8" t="n">
-        <v>7.638</v>
+        <v>7.547</v>
       </c>
       <c r="D38" s="8" t="n">
-        <v>7.3125</v>
+        <v>7.371</v>
       </c>
       <c r="E38" s="8" t="n">
-        <v>7.665</v>
+        <v>7.7785</v>
       </c>
       <c r="F38" s="8" t="n">
-        <v>7.5845</v>
+        <v>7.4515</v>
       </c>
       <c r="G38" s="8" t="n">
-        <v>7.3595</v>
+        <v>7.159</v>
       </c>
       <c r="H38" s="9" t="n"/>
       <c r="I38" s="9" t="n"/>
       <c r="J38" s="8" t="n">
-        <v>7.3165</v>
+        <v>7.28</v>
       </c>
     </row>
     <row r="39">
@@ -3316,24 +3316,24 @@
         </is>
       </c>
       <c r="C39" s="8" t="n">
-        <v>1069.076</v>
+        <v>1044.876</v>
       </c>
       <c r="D39" s="8" t="n">
-        <v>512.638</v>
+        <v>431.346</v>
       </c>
       <c r="E39" s="8" t="n">
-        <v>602.7380000000001</v>
+        <v>628.7455</v>
       </c>
       <c r="F39" s="8" t="n">
-        <v>570.16</v>
+        <v>604.7910000000001</v>
       </c>
       <c r="G39" s="8" t="n">
-        <v>612.7025</v>
+        <v>719.223</v>
       </c>
       <c r="H39" s="9" t="n"/>
       <c r="I39" s="9" t="n"/>
       <c r="J39" s="8" t="n">
-        <v>700.9105</v>
+        <v>813.5465</v>
       </c>
     </row>
     <row r="40">
@@ -3736,24 +3736,24 @@
         </is>
       </c>
       <c r="C53" s="8" t="n">
-        <v>444.8</v>
+        <v>39.0755</v>
       </c>
       <c r="D53" s="8" t="n">
-        <v>36.411</v>
+        <v>44.7315</v>
       </c>
       <c r="E53" s="8" t="n">
-        <v>35.5265</v>
+        <v>32.192</v>
       </c>
       <c r="F53" s="8" t="n">
-        <v>34.5895</v>
+        <v>33.0795</v>
       </c>
       <c r="G53" s="8" t="n">
-        <v>459.6365</v>
+        <v>37.267</v>
       </c>
       <c r="H53" s="9" t="n"/>
       <c r="I53" s="9" t="n"/>
       <c r="J53" s="8" t="n">
-        <v>511.877</v>
+        <v>34.0715</v>
       </c>
     </row>
     <row r="54">
@@ -3764,24 +3764,24 @@
         </is>
       </c>
       <c r="C54" s="8" t="n">
-        <v>24.5715</v>
+        <v>19.165</v>
       </c>
       <c r="D54" s="8" t="n">
-        <v>20.463</v>
+        <v>23.8685</v>
       </c>
       <c r="E54" s="8" t="n">
-        <v>24.442</v>
+        <v>19.7655</v>
       </c>
       <c r="F54" s="8" t="n">
-        <v>21.323</v>
+        <v>21.875</v>
       </c>
       <c r="G54" s="8" t="n">
-        <v>24.369</v>
+        <v>21.257</v>
       </c>
       <c r="H54" s="9" t="n"/>
       <c r="I54" s="9" t="n"/>
       <c r="J54" s="8" t="n">
-        <v>24.846</v>
+        <v>19.19</v>
       </c>
     </row>
     <row r="55">
@@ -3792,24 +3792,24 @@
         </is>
       </c>
       <c r="C55" s="8" t="n">
-        <v>0.907</v>
+        <v>0.9409999999999999</v>
       </c>
       <c r="D55" s="8" t="n">
-        <v>1.0115</v>
+        <v>1.0075</v>
       </c>
       <c r="E55" s="8" t="n">
-        <v>0.9775</v>
+        <v>1.007</v>
       </c>
       <c r="F55" s="8" t="n">
-        <v>0.973</v>
+        <v>1</v>
       </c>
       <c r="G55" s="8" t="n">
-        <v>0.904</v>
+        <v>1.1835</v>
       </c>
       <c r="H55" s="9" t="n"/>
       <c r="I55" s="9" t="n"/>
       <c r="J55" s="8" t="n">
-        <v>0.904</v>
+        <v>0.9419999999999999</v>
       </c>
     </row>
     <row r="56">
@@ -3820,24 +3820,24 @@
         </is>
       </c>
       <c r="C56" s="8" t="n">
-        <v>470.2065</v>
+        <v>59.1735</v>
       </c>
       <c r="D56" s="8" t="n">
-        <v>57.8865</v>
+        <v>69.6125</v>
       </c>
       <c r="E56" s="8" t="n">
-        <v>60.9555</v>
+        <v>52.9695</v>
       </c>
       <c r="F56" s="8" t="n">
-        <v>56.889</v>
+        <v>55.96</v>
       </c>
       <c r="G56" s="8" t="n">
-        <v>485.102</v>
+        <v>59.709</v>
       </c>
       <c r="H56" s="9" t="n"/>
       <c r="I56" s="9" t="n"/>
       <c r="J56" s="8" t="n">
-        <v>537.5535</v>
+        <v>54.347</v>
       </c>
     </row>
     <row r="57">

</xml_diff>

<commit_message>
Apples-to-apples Plan A: every backend uses its natural
</commit_message>
<xml_diff>
--- a/bm_resultL4.xlsx
+++ b/bm_resultL4.xlsx
@@ -1699,24 +1699,24 @@
         </is>
       </c>
       <c r="B2" s="8" t="n">
-        <v>2028.102</v>
+        <v>1771.5575</v>
       </c>
       <c r="C2" s="8" t="n">
-        <v>1001.4835</v>
+        <v>1012.2755</v>
       </c>
       <c r="D2" s="8" t="n">
-        <v>1579.266</v>
+        <v>1544.949</v>
       </c>
       <c r="E2" s="8" t="n">
-        <v>1552.726</v>
+        <v>1517.6855</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>1273.0575</v>
+        <v>1184.7615</v>
       </c>
       <c r="G2" s="9" t="n"/>
       <c r="H2" s="9" t="n"/>
       <c r="I2" s="8" t="n">
-        <v>1290.693</v>
+        <v>1247.413</v>
       </c>
       <c r="J2" s="9" t="n"/>
     </row>
@@ -1727,24 +1727,24 @@
         </is>
       </c>
       <c r="B3" s="8" t="n">
-        <v>3603.054</v>
+        <v>986.3</v>
       </c>
       <c r="C3" s="8" t="n">
-        <v>943.283</v>
+        <v>2733.8415</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>1325.1885</v>
+        <v>2658.403</v>
       </c>
       <c r="E3" s="8" t="n">
-        <v>1282.534</v>
+        <v>1387.7285</v>
       </c>
       <c r="F3" s="8" t="n">
-        <v>4583.751</v>
+        <v>5220.1315</v>
       </c>
       <c r="G3" s="9" t="n"/>
       <c r="H3" s="9" t="n"/>
       <c r="I3" s="8" t="n">
-        <v>4966.076</v>
+        <v>5505.849</v>
       </c>
       <c r="J3" s="9" t="n"/>
     </row>
@@ -1755,24 +1755,24 @@
         </is>
       </c>
       <c r="B4" s="8" t="n">
-        <v>1372.8635</v>
+        <v>712.918</v>
       </c>
       <c r="C4" s="8" t="n">
-        <v>710.62</v>
+        <v>706.628</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>720.902</v>
+        <v>1011.319</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>711.241</v>
+        <v>727.4915</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>920.9405</v>
+        <v>1156.5055</v>
       </c>
       <c r="G4" s="9" t="n"/>
       <c r="H4" s="9" t="n"/>
       <c r="I4" s="8" t="n">
-        <v>987.221</v>
+        <v>1137.0765</v>
       </c>
       <c r="J4" s="9" t="n"/>
     </row>
@@ -1783,24 +1783,24 @@
         </is>
       </c>
       <c r="B5" s="8" t="n">
-        <v>3420.4895</v>
+        <v>589.2085</v>
       </c>
       <c r="C5" s="8" t="n">
-        <v>1290.4755</v>
+        <v>2208.1095</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>1006.026</v>
+        <v>2829.593</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>930.6085</v>
+        <v>915.737</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>2943.378</v>
+        <v>3057.966</v>
       </c>
       <c r="G5" s="9" t="n"/>
       <c r="H5" s="9" t="n"/>
       <c r="I5" s="8" t="n">
-        <v>3056.4685</v>
+        <v>3008.5785</v>
       </c>
       <c r="J5" s="9" t="n"/>
     </row>
@@ -1811,24 +1811,24 @@
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>134.332</v>
+        <v>140.626</v>
       </c>
       <c r="C6" s="8" t="n">
-        <v>28.741</v>
+        <v>43.008</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>24.068</v>
+        <v>55.75</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>24.631</v>
+        <v>38.737</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>228.494</v>
+        <v>210.698</v>
       </c>
       <c r="G6" s="9" t="n"/>
       <c r="H6" s="9" t="n"/>
       <c r="I6" s="8" t="n">
-        <v>628.467</v>
+        <v>596.005</v>
       </c>
       <c r="J6" s="9" t="n"/>
     </row>
@@ -1839,24 +1839,24 @@
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>1707.148</v>
+        <v>637.175</v>
       </c>
       <c r="C7" s="8" t="n">
-        <v>718.393</v>
+        <v>851.3105</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>1154.8775</v>
+        <v>1877.5465</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>1109.8655</v>
+        <v>930.5575</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>1132.7815</v>
+        <v>1444.4775</v>
       </c>
       <c r="G7" s="9" t="n"/>
       <c r="H7" s="9" t="n"/>
       <c r="I7" s="8" t="n">
-        <v>1244.1125</v>
+        <v>1421.486</v>
       </c>
       <c r="J7" s="9" t="n"/>
     </row>
@@ -1867,24 +1867,24 @@
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>1044.876</v>
+        <v>437.0685</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>431.346</v>
+        <v>454.524</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>628.7455</v>
+        <v>1027.5375</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>604.7910000000001</v>
+        <v>572.5855</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>719.223</v>
+        <v>878.981</v>
       </c>
       <c r="G8" s="9" t="n"/>
       <c r="H8" s="9" t="n"/>
       <c r="I8" s="8" t="n">
-        <v>813.5465</v>
+        <v>912.8895</v>
       </c>
       <c r="J8" s="9" t="n"/>
     </row>
@@ -1895,24 +1895,24 @@
         </is>
       </c>
       <c r="B9" s="8" t="n">
-        <v>1977.6165</v>
+        <v>1401.4595</v>
       </c>
       <c r="C9" s="8" t="n">
-        <v>1339.277</v>
+        <v>1553.859</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>1292.08</v>
+        <v>1245.2665</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>1079.6835</v>
+        <v>1094.998</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>2025.361</v>
+        <v>1918.92</v>
       </c>
       <c r="G9" s="9" t="n"/>
       <c r="H9" s="9" t="n"/>
       <c r="I9" s="8" t="n">
-        <v>2192.618</v>
+        <v>2077.558</v>
       </c>
       <c r="J9" s="9" t="n"/>
     </row>
@@ -1923,24 +1923,24 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>277.701</v>
+        <v>199.152</v>
       </c>
       <c r="C10" s="8" t="n">
-        <v>208.468</v>
+        <v>207.4225</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>189.4175</v>
+        <v>187.7505</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>182.1065</v>
+        <v>178.521</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>230.836</v>
+        <v>231.076</v>
       </c>
       <c r="G10" s="9" t="n"/>
       <c r="H10" s="9" t="n"/>
       <c r="I10" s="8" t="n">
-        <v>239.195</v>
+        <v>238.156</v>
       </c>
       <c r="J10" s="9" t="n"/>
     </row>
@@ -1985,24 +1985,24 @@
         </is>
       </c>
       <c r="B12" s="8" t="n">
-        <v>59.1735</v>
+        <v>48.2825</v>
       </c>
       <c r="C12" s="8" t="n">
-        <v>69.6125</v>
+        <v>59.3815</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>52.9695</v>
+        <v>51.8015</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>55.96</v>
+        <v>51.3375</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>59.709</v>
+        <v>61.514</v>
       </c>
       <c r="G12" s="9" t="n"/>
       <c r="H12" s="9" t="n"/>
       <c r="I12" s="8" t="n">
-        <v>54.347</v>
+        <v>54.7575</v>
       </c>
       <c r="J12" s="9" t="n"/>
     </row>
@@ -2013,24 +2013,24 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>269.1215</v>
+        <v>271.2215</v>
       </c>
       <c r="C13" s="8" t="n">
-        <v>220.4715</v>
+        <v>219.5055</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>212.381</v>
+        <v>213.709</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>212.9095</v>
+        <v>213.5735</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>239.585</v>
+        <v>239.0605</v>
       </c>
       <c r="G13" s="9" t="n"/>
       <c r="H13" s="9" t="n"/>
       <c r="I13" s="8" t="n">
-        <v>268.818</v>
+        <v>268.0645</v>
       </c>
       <c r="J13" s="9" t="n"/>
     </row>
@@ -2268,24 +2268,24 @@
         </is>
       </c>
       <c r="C2" s="8" t="n">
-        <v>248.0305</v>
+        <v>25.379</v>
       </c>
       <c r="D2" s="8" t="n">
-        <v>42.0995</v>
+        <v>75.07250000000001</v>
       </c>
       <c r="E2" s="8" t="n">
-        <v>37.9835</v>
+        <v>35.203</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>13.078</v>
+        <v>12.917</v>
       </c>
       <c r="G2" s="8" t="n">
-        <v>78.9965</v>
+        <v>77.955</v>
       </c>
       <c r="H2" s="9" t="n"/>
       <c r="I2" s="9" t="n"/>
       <c r="J2" s="8" t="n">
-        <v>90.9085</v>
+        <v>84.04000000000001</v>
       </c>
     </row>
     <row r="3">
@@ -2296,24 +2296,24 @@
         </is>
       </c>
       <c r="C3" s="8" t="n">
-        <v>1001.5955</v>
+        <v>993.7465</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>178.777</v>
+        <v>179.395</v>
       </c>
       <c r="E3" s="8" t="n">
-        <v>760.5645</v>
+        <v>752.8535000000001</v>
       </c>
       <c r="F3" s="8" t="n">
-        <v>760.28</v>
+        <v>748.6395</v>
       </c>
       <c r="G3" s="8" t="n">
-        <v>416.8915</v>
+        <v>351.736</v>
       </c>
       <c r="H3" s="9" t="n"/>
       <c r="I3" s="9" t="n"/>
       <c r="J3" s="8" t="n">
-        <v>420.956</v>
+        <v>406.8655</v>
       </c>
     </row>
     <row r="4">
@@ -2324,24 +2324,24 @@
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>777.6145</v>
+        <v>752.597</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>780.346</v>
+        <v>757.809</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>780.6685</v>
+        <v>756.95</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>779.6900000000001</v>
+        <v>756.0335</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>777.2195</v>
+        <v>754.87</v>
       </c>
       <c r="H4" s="9" t="n"/>
       <c r="I4" s="9" t="n"/>
       <c r="J4" s="8" t="n">
-        <v>778.778</v>
+        <v>756.403</v>
       </c>
     </row>
     <row r="5">
@@ -2352,24 +2352,24 @@
         </is>
       </c>
       <c r="C5" s="8" t="n">
-        <v>2028.102</v>
+        <v>1771.5575</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>1001.4835</v>
+        <v>1012.2755</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>1579.266</v>
+        <v>1544.949</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>1552.726</v>
+        <v>1517.6855</v>
       </c>
       <c r="G5" s="8" t="n">
-        <v>1273.0575</v>
+        <v>1184.7615</v>
       </c>
       <c r="H5" s="9" t="n"/>
       <c r="I5" s="9" t="n"/>
       <c r="J5" s="8" t="n">
-        <v>1290.693</v>
+        <v>1247.413</v>
       </c>
     </row>
     <row r="6">
@@ -2384,24 +2384,24 @@
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>22.0915</v>
+        <v>21.9785</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>24.45</v>
+        <v>24.5645</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>22.25</v>
+        <v>22.7995</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>23.4705</v>
+        <v>22.1705</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>21.995</v>
+        <v>22.653</v>
       </c>
       <c r="H6" s="9" t="n"/>
       <c r="I6" s="9" t="n"/>
       <c r="J6" s="8" t="n">
-        <v>22.1495</v>
+        <v>22.806</v>
       </c>
     </row>
     <row r="7">
@@ -2412,24 +2412,24 @@
         </is>
       </c>
       <c r="C7" s="8" t="n">
-        <v>2197.456</v>
+        <v>741.4974999999999</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>796.7605</v>
+        <v>790.992</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>1195.838</v>
+        <v>2252.8125</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>1159.9735</v>
+        <v>1152.1975</v>
       </c>
       <c r="G7" s="8" t="n">
-        <v>1299.308</v>
+        <v>2062.2385</v>
       </c>
       <c r="H7" s="9" t="n"/>
       <c r="I7" s="9" t="n"/>
       <c r="J7" s="8" t="n">
-        <v>1226.864</v>
+        <v>1918.047</v>
       </c>
     </row>
     <row r="8">
@@ -2440,24 +2440,24 @@
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>1277.042</v>
+        <v>132.2875</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>34.0175</v>
+        <v>1829.6715</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>19.576</v>
+        <v>293.417</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>10.8475</v>
+        <v>125.386</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>3171.57</v>
+        <v>3042.0555</v>
       </c>
       <c r="H8" s="9" t="n"/>
       <c r="I8" s="9" t="n"/>
       <c r="J8" s="8" t="n">
-        <v>3605.0055</v>
+        <v>3452.935</v>
       </c>
     </row>
     <row r="9">
@@ -2468,24 +2468,24 @@
         </is>
       </c>
       <c r="C9" s="8" t="n">
-        <v>14.367</v>
+        <v>8.0075</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>5.5065</v>
+        <v>6.1145</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>5.2325</v>
+        <v>5.414</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>5.3295</v>
+        <v>5.2895</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>9.773</v>
+        <v>9.903</v>
       </c>
       <c r="H9" s="9" t="n"/>
       <c r="I9" s="9" t="n"/>
       <c r="J9" s="8" t="n">
-        <v>28.5115</v>
+        <v>27.853</v>
       </c>
     </row>
     <row r="10">
@@ -2496,24 +2496,24 @@
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>83.1515</v>
+        <v>82.1955</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>82.4295</v>
+        <v>82.663</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>82.315</v>
+        <v>83.27800000000001</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>82.2825</v>
+        <v>82.92100000000001</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>82.645</v>
+        <v>83.0035</v>
       </c>
       <c r="H10" s="9" t="n"/>
       <c r="I10" s="9" t="n"/>
       <c r="J10" s="8" t="n">
-        <v>82.99250000000001</v>
+        <v>83.575</v>
       </c>
     </row>
     <row r="11">
@@ -2524,24 +2524,24 @@
         </is>
       </c>
       <c r="C11" s="8" t="n">
-        <v>3603.054</v>
+        <v>986.3</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>943.283</v>
+        <v>2733.8415</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>1325.1885</v>
+        <v>2658.403</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>1282.534</v>
+        <v>1387.7285</v>
       </c>
       <c r="G11" s="8" t="n">
-        <v>4583.751</v>
+        <v>5220.1315</v>
       </c>
       <c r="H11" s="9" t="n"/>
       <c r="I11" s="9" t="n"/>
       <c r="J11" s="8" t="n">
-        <v>4966.076</v>
+        <v>5505.849</v>
       </c>
     </row>
     <row r="12">
@@ -2556,24 +2556,24 @@
         </is>
       </c>
       <c r="C12" s="8" t="n">
-        <v>248.096</v>
+        <v>248.3445</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>248.6595</v>
+        <v>250.8645</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>244.94</v>
+        <v>247.1135</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>244.906</v>
+        <v>248.662</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>254.489</v>
+        <v>250.4495</v>
       </c>
       <c r="H12" s="9" t="n"/>
       <c r="I12" s="9" t="n"/>
       <c r="J12" s="8" t="n">
-        <v>245.92</v>
+        <v>252.3425</v>
       </c>
     </row>
     <row r="13">
@@ -2584,24 +2584,24 @@
         </is>
       </c>
       <c r="C13" s="8" t="n">
-        <v>825.231</v>
+        <v>166.96</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>160.1735</v>
+        <v>157.073</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>179.194</v>
+        <v>468.833</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>169.853</v>
+        <v>158.9485</v>
       </c>
       <c r="G13" s="8" t="n">
-        <v>363.2235</v>
+        <v>606.278</v>
       </c>
       <c r="H13" s="9" t="n"/>
       <c r="I13" s="9" t="n"/>
       <c r="J13" s="8" t="n">
-        <v>440.3245</v>
+        <v>585.3915</v>
       </c>
     </row>
     <row r="14">
@@ -2612,24 +2612,24 @@
         </is>
       </c>
       <c r="C14" s="8" t="n">
-        <v>237.7165</v>
+        <v>237.5485</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>237.1095</v>
+        <v>236.966</v>
       </c>
       <c r="E14" s="8" t="n">
-        <v>237.7255</v>
+        <v>236.0865</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>235.049</v>
+        <v>260.0905</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>237.1875</v>
+        <v>237.5845</v>
       </c>
       <c r="H14" s="9" t="n"/>
       <c r="I14" s="9" t="n"/>
       <c r="J14" s="8" t="n">
-        <v>236.3645</v>
+        <v>237.6925</v>
       </c>
     </row>
     <row r="15">
@@ -2640,24 +2640,24 @@
         </is>
       </c>
       <c r="C15" s="8" t="n">
-        <v>63.421</v>
+        <v>59.425</v>
       </c>
       <c r="D15" s="8" t="n">
-        <v>64.346</v>
+        <v>61.6425</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>59.9845</v>
+        <v>60.2995</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>61.601</v>
+        <v>58.876</v>
       </c>
       <c r="G15" s="8" t="n">
-        <v>63.959</v>
+        <v>62.3555</v>
       </c>
       <c r="H15" s="9" t="n"/>
       <c r="I15" s="9" t="n"/>
       <c r="J15" s="8" t="n">
-        <v>62.981</v>
+        <v>62.6025</v>
       </c>
     </row>
     <row r="16">
@@ -2668,24 +2668,24 @@
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>1372.8635</v>
+        <v>712.918</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>710.62</v>
+        <v>706.628</v>
       </c>
       <c r="E16" s="8" t="n">
-        <v>720.902</v>
+        <v>1011.319</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>711.241</v>
+        <v>727.4915</v>
       </c>
       <c r="G16" s="8" t="n">
-        <v>920.9405</v>
+        <v>1156.5055</v>
       </c>
       <c r="H16" s="9" t="n"/>
       <c r="I16" s="9" t="n"/>
       <c r="J16" s="8" t="n">
-        <v>987.221</v>
+        <v>1137.0765</v>
       </c>
     </row>
     <row r="17">
@@ -2700,24 +2700,24 @@
         </is>
       </c>
       <c r="C17" s="8" t="n">
-        <v>286.2415</v>
+        <v>278.728</v>
       </c>
       <c r="D17" s="8" t="n">
-        <v>289.7485</v>
+        <v>322.153</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>316.9215</v>
+        <v>285.663</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>280.6995</v>
+        <v>279.536</v>
       </c>
       <c r="G17" s="8" t="n">
-        <v>290.349</v>
+        <v>304.087</v>
       </c>
       <c r="H17" s="9" t="n"/>
       <c r="I17" s="9" t="n"/>
       <c r="J17" s="8" t="n">
-        <v>287.2305</v>
+        <v>296.185</v>
       </c>
     </row>
     <row r="18">
@@ -2728,24 +2728,24 @@
         </is>
       </c>
       <c r="C18" s="8" t="n">
-        <v>3010.6125</v>
+        <v>189.7035</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>872.3145</v>
+        <v>1758.4335</v>
       </c>
       <c r="E18" s="8" t="n">
-        <v>561.0415</v>
+        <v>2420.751</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>527.3185</v>
+        <v>512.9085</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>2528.5685</v>
+        <v>2628.8265</v>
       </c>
       <c r="H18" s="9" t="n"/>
       <c r="I18" s="9" t="n"/>
       <c r="J18" s="8" t="n">
-        <v>2644.287</v>
+        <v>2587.23</v>
       </c>
     </row>
     <row r="19">
@@ -2756,24 +2756,24 @@
         </is>
       </c>
       <c r="C19" s="8" t="n">
-        <v>122.7625</v>
+        <v>119.7535</v>
       </c>
       <c r="D19" s="8" t="n">
-        <v>121.8615</v>
+        <v>127.378</v>
       </c>
       <c r="E19" s="8" t="n">
-        <v>126.5285</v>
+        <v>124.0705</v>
       </c>
       <c r="F19" s="8" t="n">
-        <v>122.011</v>
+        <v>123.5005</v>
       </c>
       <c r="G19" s="8" t="n">
-        <v>124.3115</v>
+        <v>124.439</v>
       </c>
       <c r="H19" s="9" t="n"/>
       <c r="I19" s="9" t="n"/>
       <c r="J19" s="8" t="n">
-        <v>123.1775</v>
+        <v>125.344</v>
       </c>
     </row>
     <row r="20">
@@ -2784,24 +2784,24 @@
         </is>
       </c>
       <c r="C20" s="8" t="n">
-        <v>3420.4895</v>
+        <v>589.2085</v>
       </c>
       <c r="D20" s="8" t="n">
-        <v>1290.4755</v>
+        <v>2208.1095</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>1006.026</v>
+        <v>2829.593</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>930.6085</v>
+        <v>915.737</v>
       </c>
       <c r="G20" s="8" t="n">
-        <v>2943.378</v>
+        <v>3057.966</v>
       </c>
       <c r="H20" s="9" t="n"/>
       <c r="I20" s="9" t="n"/>
       <c r="J20" s="8" t="n">
-        <v>3056.4685</v>
+        <v>3008.5785</v>
       </c>
     </row>
     <row r="21">
@@ -2816,24 +2816,24 @@
         </is>
       </c>
       <c r="C21" s="8" t="n">
-        <v>0.005</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="D21" s="8" t="n">
-        <v>2.011</v>
+        <v>2.106</v>
       </c>
       <c r="E21" s="8" t="n">
-        <v>0.944</v>
+        <v>0.958</v>
       </c>
       <c r="F21" s="8" t="n">
-        <v>0.907</v>
+        <v>1.008</v>
       </c>
       <c r="G21" s="8" t="n">
-        <v>2.716</v>
+        <v>2.867</v>
       </c>
       <c r="H21" s="9" t="n"/>
       <c r="I21" s="9" t="n"/>
       <c r="J21" s="8" t="n">
-        <v>1.502</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="22">
@@ -2844,24 +2844,24 @@
         </is>
       </c>
       <c r="C22" s="8" t="n">
-        <v>12.852</v>
+        <v>12.701</v>
       </c>
       <c r="D22" s="8" t="n">
-        <v>4.523</v>
+        <v>5.704</v>
       </c>
       <c r="E22" s="8" t="n">
-        <v>1.879</v>
+        <v>2.37</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>1.836</v>
+        <v>2.614</v>
       </c>
       <c r="G22" s="8" t="n">
-        <v>7.833</v>
+        <v>5.845</v>
       </c>
       <c r="H22" s="9" t="n"/>
       <c r="I22" s="9" t="n"/>
       <c r="J22" s="8" t="n">
-        <v>27.69</v>
+        <v>26.296</v>
       </c>
     </row>
     <row r="23">
@@ -2872,24 +2872,24 @@
         </is>
       </c>
       <c r="C23" s="8" t="n">
-        <v>84.88</v>
+        <v>91.173</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>10.394</v>
+        <v>23.905</v>
       </c>
       <c r="E23" s="8" t="n">
-        <v>2.864</v>
+        <v>33.432</v>
       </c>
       <c r="F23" s="8" t="n">
-        <v>2.684</v>
+        <v>15.748</v>
       </c>
       <c r="G23" s="8" t="n">
-        <v>192.749</v>
+        <v>177.337</v>
       </c>
       <c r="H23" s="9" t="n"/>
       <c r="I23" s="9" t="n"/>
       <c r="J23" s="8" t="n">
-        <v>517.647</v>
+        <v>488.858</v>
       </c>
     </row>
     <row r="24">
@@ -2900,24 +2900,24 @@
         </is>
       </c>
       <c r="C24" s="8" t="n">
-        <v>3.735</v>
+        <v>3.762</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>3.299</v>
+        <v>3.535</v>
       </c>
       <c r="E24" s="8" t="n">
-        <v>13.134</v>
+        <v>13.163</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>13.398</v>
+        <v>13.38</v>
       </c>
       <c r="G24" s="8" t="n">
-        <v>12.898</v>
+        <v>12.335</v>
       </c>
       <c r="H24" s="9" t="n"/>
       <c r="I24" s="9" t="n"/>
       <c r="J24" s="8" t="n">
-        <v>64.624</v>
+        <v>63.11</v>
       </c>
     </row>
     <row r="25">
@@ -2928,24 +2928,24 @@
         </is>
       </c>
       <c r="C25" s="8" t="n">
-        <v>32.847</v>
+        <v>32.97</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>7.106</v>
+        <v>7.169</v>
       </c>
       <c r="E25" s="8" t="n">
-        <v>5.239</v>
+        <v>5.818</v>
       </c>
       <c r="F25" s="8" t="n">
-        <v>5.797</v>
+        <v>5.976</v>
       </c>
       <c r="G25" s="8" t="n">
-        <v>12.286</v>
+        <v>12.303</v>
       </c>
       <c r="H25" s="9" t="n"/>
       <c r="I25" s="9" t="n"/>
       <c r="J25" s="8" t="n">
-        <v>16.994</v>
+        <v>16.633</v>
       </c>
     </row>
     <row r="26">
@@ -2956,24 +2956,24 @@
         </is>
       </c>
       <c r="C26" s="8" t="n">
-        <v>134.332</v>
+        <v>140.626</v>
       </c>
       <c r="D26" s="8" t="n">
-        <v>28.741</v>
+        <v>43.008</v>
       </c>
       <c r="E26" s="8" t="n">
-        <v>24.068</v>
+        <v>55.75</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>24.631</v>
+        <v>38.737</v>
       </c>
       <c r="G26" s="8" t="n">
-        <v>228.494</v>
+        <v>210.698</v>
       </c>
       <c r="H26" s="9" t="n"/>
       <c r="I26" s="9" t="n"/>
       <c r="J26" s="8" t="n">
-        <v>628.467</v>
+        <v>596.005</v>
       </c>
     </row>
     <row r="27">
@@ -2988,24 +2988,24 @@
         </is>
       </c>
       <c r="C27" s="8" t="n">
-        <v>89.1935</v>
+        <v>88.072</v>
       </c>
       <c r="D27" s="8" t="n">
-        <v>89.0235</v>
+        <v>136.1105</v>
       </c>
       <c r="E27" s="8" t="n">
-        <v>140.038</v>
+        <v>88.245</v>
       </c>
       <c r="F27" s="8" t="n">
-        <v>138.958</v>
+        <v>88.077</v>
       </c>
       <c r="G27" s="8" t="n">
-        <v>89.1425</v>
+        <v>88.4485</v>
       </c>
       <c r="H27" s="9" t="n"/>
       <c r="I27" s="9" t="n"/>
       <c r="J27" s="8" t="n">
-        <v>89.31</v>
+        <v>88.404</v>
       </c>
     </row>
     <row r="28">
@@ -3016,24 +3016,24 @@
         </is>
       </c>
       <c r="C28" s="8" t="n">
-        <v>355.2395</v>
+        <v>346.3885</v>
       </c>
       <c r="D28" s="8" t="n">
-        <v>352.3605</v>
+        <v>418.221</v>
       </c>
       <c r="E28" s="8" t="n">
-        <v>437.408</v>
+        <v>344.0195</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>428.826</v>
+        <v>348.794</v>
       </c>
       <c r="G28" s="8" t="n">
-        <v>351.9555</v>
+        <v>351.883</v>
       </c>
       <c r="H28" s="9" t="n"/>
       <c r="I28" s="9" t="n"/>
       <c r="J28" s="8" t="n">
-        <v>355.8005</v>
+        <v>349.57</v>
       </c>
     </row>
     <row r="29">
@@ -3044,24 +3044,24 @@
         </is>
       </c>
       <c r="C29" s="8" t="n">
-        <v>1233.663</v>
+        <v>174.9085</v>
       </c>
       <c r="D29" s="8" t="n">
-        <v>248.3075</v>
+        <v>263.103</v>
       </c>
       <c r="E29" s="8" t="n">
-        <v>540.5365</v>
+        <v>1416.3165</v>
       </c>
       <c r="F29" s="8" t="n">
-        <v>511.323</v>
+        <v>465.004</v>
       </c>
       <c r="G29" s="8" t="n">
-        <v>659.9450000000001</v>
+        <v>974.0940000000001</v>
       </c>
       <c r="H29" s="9" t="n"/>
       <c r="I29" s="9" t="n"/>
       <c r="J29" s="8" t="n">
-        <v>769.6325000000001</v>
+        <v>954.6965</v>
       </c>
     </row>
     <row r="30">
@@ -3072,24 +3072,24 @@
         </is>
       </c>
       <c r="C30" s="8" t="n">
-        <v>28.838</v>
+        <v>28.7695</v>
       </c>
       <c r="D30" s="8" t="n">
-        <v>29.663</v>
+        <v>34.0235</v>
       </c>
       <c r="E30" s="8" t="n">
-        <v>30.732</v>
+        <v>28.955</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>30.7325</v>
+        <v>29.241</v>
       </c>
       <c r="G30" s="8" t="n">
-        <v>28.8075</v>
+        <v>29.1405</v>
       </c>
       <c r="H30" s="9" t="n"/>
       <c r="I30" s="9" t="n"/>
       <c r="J30" s="8" t="n">
-        <v>29.0645</v>
+        <v>29.493</v>
       </c>
     </row>
     <row r="31">
@@ -3116,24 +3116,24 @@
         </is>
       </c>
       <c r="C32" s="8" t="n">
-        <v>1707.148</v>
+        <v>637.175</v>
       </c>
       <c r="D32" s="8" t="n">
-        <v>718.393</v>
+        <v>851.3105</v>
       </c>
       <c r="E32" s="8" t="n">
-        <v>1154.8775</v>
+        <v>1877.5465</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>1109.8655</v>
+        <v>930.5575</v>
       </c>
       <c r="G32" s="8" t="n">
-        <v>1132.7815</v>
+        <v>1444.4775</v>
       </c>
       <c r="H32" s="9" t="n"/>
       <c r="I32" s="9" t="n"/>
       <c r="J32" s="8" t="n">
-        <v>1244.1125</v>
+        <v>1421.486</v>
       </c>
     </row>
     <row r="33">
@@ -3148,24 +3148,24 @@
         </is>
       </c>
       <c r="C33" s="8" t="n">
-        <v>91.0385</v>
+        <v>91.32599999999999</v>
       </c>
       <c r="D33" s="8" t="n">
-        <v>89.5325</v>
+        <v>97.834</v>
       </c>
       <c r="E33" s="8" t="n">
-        <v>92.1405</v>
+        <v>89.58450000000001</v>
       </c>
       <c r="F33" s="8" t="n">
-        <v>90.604</v>
+        <v>90.59350000000001</v>
       </c>
       <c r="G33" s="8" t="n">
-        <v>99.27500000000001</v>
+        <v>93.1305</v>
       </c>
       <c r="H33" s="9" t="n"/>
       <c r="I33" s="9" t="n"/>
       <c r="J33" s="8" t="n">
-        <v>99.30249999999999</v>
+        <v>97.7265</v>
       </c>
     </row>
     <row r="34">
@@ -3176,24 +3176,24 @@
         </is>
       </c>
       <c r="C34" s="8" t="n">
-        <v>700.961</v>
+        <v>102.394</v>
       </c>
       <c r="D34" s="8" t="n">
-        <v>112.4955</v>
+        <v>115.203</v>
       </c>
       <c r="E34" s="8" t="n">
-        <v>312.994</v>
+        <v>711.3935</v>
       </c>
       <c r="F34" s="8" t="n">
-        <v>292.641</v>
+        <v>261.002</v>
       </c>
       <c r="G34" s="8" t="n">
-        <v>386.91</v>
+        <v>550.0170000000001</v>
       </c>
       <c r="H34" s="9" t="n"/>
       <c r="I34" s="9" t="n"/>
       <c r="J34" s="8" t="n">
-        <v>458.493</v>
+        <v>542.1375</v>
       </c>
     </row>
     <row r="35">
@@ -3204,24 +3204,24 @@
         </is>
       </c>
       <c r="C35" s="8" t="n">
-        <v>0.002</v>
+        <v>0.005</v>
       </c>
       <c r="D35" s="8" t="n">
-        <v>2.8435</v>
+        <v>2.874</v>
       </c>
       <c r="E35" s="8" t="n">
-        <v>0.952</v>
+        <v>1.1295</v>
       </c>
       <c r="F35" s="8" t="n">
-        <v>0.9235</v>
+        <v>0.91</v>
       </c>
       <c r="G35" s="8" t="n">
-        <v>1.672</v>
+        <v>1.337</v>
       </c>
       <c r="H35" s="9" t="n"/>
       <c r="I35" s="9" t="n"/>
       <c r="J35" s="8" t="n">
-        <v>1.3795</v>
+        <v>4.2565</v>
       </c>
     </row>
     <row r="36">
@@ -3232,24 +3232,24 @@
         </is>
       </c>
       <c r="C36" s="8" t="n">
-        <v>37.1105</v>
+        <v>29.3795</v>
       </c>
       <c r="D36" s="8" t="n">
-        <v>11.608</v>
+        <v>19.056</v>
       </c>
       <c r="E36" s="8" t="n">
-        <v>8.598000000000001</v>
+        <v>8.853</v>
       </c>
       <c r="F36" s="8" t="n">
-        <v>8.893000000000001</v>
+        <v>8.7235</v>
       </c>
       <c r="G36" s="8" t="n">
-        <v>18.4955</v>
+        <v>18.132</v>
       </c>
       <c r="H36" s="9" t="n"/>
       <c r="I36" s="9" t="n"/>
       <c r="J36" s="8" t="n">
-        <v>39.7435</v>
+        <v>50.1475</v>
       </c>
     </row>
     <row r="37">
@@ -3260,24 +3260,24 @@
         </is>
       </c>
       <c r="C37" s="8" t="n">
-        <v>208.238</v>
+        <v>206.362</v>
       </c>
       <c r="D37" s="8" t="n">
-        <v>207.7695</v>
+        <v>211.07</v>
       </c>
       <c r="E37" s="8" t="n">
-        <v>206.6585</v>
+        <v>208.6615</v>
       </c>
       <c r="F37" s="8" t="n">
-        <v>203.825</v>
+        <v>204.3935</v>
       </c>
       <c r="G37" s="8" t="n">
-        <v>204.854</v>
+        <v>209.014</v>
       </c>
       <c r="H37" s="9" t="n"/>
       <c r="I37" s="9" t="n"/>
       <c r="J37" s="8" t="n">
-        <v>206.15</v>
+        <v>210.673</v>
       </c>
     </row>
     <row r="38">
@@ -3288,24 +3288,24 @@
         </is>
       </c>
       <c r="C38" s="8" t="n">
-        <v>7.547</v>
+        <v>7.6185</v>
       </c>
       <c r="D38" s="8" t="n">
-        <v>7.371</v>
+        <v>7.337</v>
       </c>
       <c r="E38" s="8" t="n">
-        <v>7.7785</v>
+        <v>7.3625</v>
       </c>
       <c r="F38" s="8" t="n">
-        <v>7.4515</v>
+        <v>7.4385</v>
       </c>
       <c r="G38" s="8" t="n">
-        <v>7.159</v>
+        <v>7.3475</v>
       </c>
       <c r="H38" s="9" t="n"/>
       <c r="I38" s="9" t="n"/>
       <c r="J38" s="8" t="n">
-        <v>7.28</v>
+        <v>7.6295</v>
       </c>
     </row>
     <row r="39">
@@ -3316,24 +3316,24 @@
         </is>
       </c>
       <c r="C39" s="8" t="n">
-        <v>1044.876</v>
+        <v>437.0685</v>
       </c>
       <c r="D39" s="8" t="n">
-        <v>431.346</v>
+        <v>454.524</v>
       </c>
       <c r="E39" s="8" t="n">
-        <v>628.7455</v>
+        <v>1027.5375</v>
       </c>
       <c r="F39" s="8" t="n">
-        <v>604.7910000000001</v>
+        <v>572.5855</v>
       </c>
       <c r="G39" s="8" t="n">
-        <v>719.223</v>
+        <v>878.981</v>
       </c>
       <c r="H39" s="9" t="n"/>
       <c r="I39" s="9" t="n"/>
       <c r="J39" s="8" t="n">
-        <v>813.5465</v>
+        <v>912.8895</v>
       </c>
     </row>
     <row r="40">
@@ -3348,24 +3348,24 @@
         </is>
       </c>
       <c r="C40" s="8" t="n">
-        <v>604.455</v>
+        <v>852.3819999999999</v>
       </c>
       <c r="D40" s="8" t="n">
-        <v>607.1895</v>
+        <v>606.981</v>
       </c>
       <c r="E40" s="8" t="n">
-        <v>606.3869999999999</v>
+        <v>606.4705</v>
       </c>
       <c r="F40" s="8" t="n">
-        <v>604.671</v>
+        <v>610.2335</v>
       </c>
       <c r="G40" s="8" t="n">
-        <v>606.222</v>
+        <v>607.681</v>
       </c>
       <c r="H40" s="9" t="n"/>
       <c r="I40" s="9" t="n"/>
       <c r="J40" s="8" t="n">
-        <v>603.728</v>
+        <v>608.535</v>
       </c>
     </row>
     <row r="41">
@@ -3376,24 +3376,24 @@
         </is>
       </c>
       <c r="C41" s="8" t="n">
-        <v>17.4005</v>
+        <v>3.8035</v>
       </c>
       <c r="D41" s="8" t="n">
-        <v>6.3855</v>
+        <v>5.0495</v>
       </c>
       <c r="E41" s="8" t="n">
-        <v>1.6865</v>
+        <v>1.678</v>
       </c>
       <c r="F41" s="8" t="n">
-        <v>1.6265</v>
+        <v>1.6135</v>
       </c>
       <c r="G41" s="8" t="n">
-        <v>4.0765</v>
+        <v>2.9055</v>
       </c>
       <c r="H41" s="9" t="n"/>
       <c r="I41" s="9" t="n"/>
       <c r="J41" s="8" t="n">
-        <v>33.215</v>
+        <v>11.774</v>
       </c>
     </row>
     <row r="42">
@@ -3404,24 +3404,24 @@
         </is>
       </c>
       <c r="C42" s="8" t="n">
-        <v>867.301</v>
+        <v>41.119</v>
       </c>
       <c r="D42" s="8" t="n">
-        <v>263.486</v>
+        <v>493.86</v>
       </c>
       <c r="E42" s="8" t="n">
-        <v>255.4865</v>
+        <v>206.014</v>
       </c>
       <c r="F42" s="8" t="n">
-        <v>38.071</v>
+        <v>37.966</v>
       </c>
       <c r="G42" s="8" t="n">
-        <v>955.047</v>
+        <v>848.2965</v>
       </c>
       <c r="H42" s="9" t="n"/>
       <c r="I42" s="9" t="n"/>
       <c r="J42" s="8" t="n">
-        <v>1053.933</v>
+        <v>971.1605</v>
       </c>
     </row>
     <row r="43">
@@ -3432,24 +3432,24 @@
         </is>
       </c>
       <c r="C43" s="8" t="n">
-        <v>75.3425</v>
+        <v>86.669</v>
       </c>
       <c r="D43" s="8" t="n">
-        <v>42.6535</v>
+        <v>35.739</v>
       </c>
       <c r="E43" s="8" t="n">
-        <v>25.154</v>
+        <v>26.0505</v>
       </c>
       <c r="F43" s="8" t="n">
-        <v>24.8025</v>
+        <v>25.7945</v>
       </c>
       <c r="G43" s="8" t="n">
-        <v>49.0955</v>
+        <v>43.236</v>
       </c>
       <c r="H43" s="9" t="n"/>
       <c r="I43" s="9" t="n"/>
       <c r="J43" s="8" t="n">
-        <v>88.64400000000001</v>
+        <v>72.6875</v>
       </c>
     </row>
     <row r="44">
@@ -3460,24 +3460,24 @@
         </is>
       </c>
       <c r="C44" s="8" t="n">
-        <v>413.2565</v>
+        <v>418.314</v>
       </c>
       <c r="D44" s="8" t="n">
-        <v>419.0115</v>
+        <v>412.562</v>
       </c>
       <c r="E44" s="8" t="n">
-        <v>403.369</v>
+        <v>403.088</v>
       </c>
       <c r="F44" s="8" t="n">
-        <v>409.7575</v>
+        <v>418.924</v>
       </c>
       <c r="G44" s="8" t="n">
-        <v>411.2285</v>
+        <v>415.6475</v>
       </c>
       <c r="H44" s="9" t="n"/>
       <c r="I44" s="9" t="n"/>
       <c r="J44" s="8" t="n">
-        <v>413.478</v>
+        <v>414.3595</v>
       </c>
     </row>
     <row r="45">
@@ -3488,24 +3488,24 @@
         </is>
       </c>
       <c r="C45" s="8" t="n">
-        <v>1977.6165</v>
+        <v>1401.4595</v>
       </c>
       <c r="D45" s="8" t="n">
-        <v>1339.277</v>
+        <v>1553.859</v>
       </c>
       <c r="E45" s="8" t="n">
-        <v>1292.08</v>
+        <v>1245.2665</v>
       </c>
       <c r="F45" s="8" t="n">
-        <v>1079.6835</v>
+        <v>1094.998</v>
       </c>
       <c r="G45" s="8" t="n">
-        <v>2025.361</v>
+        <v>1918.92</v>
       </c>
       <c r="H45" s="9" t="n"/>
       <c r="I45" s="9" t="n"/>
       <c r="J45" s="8" t="n">
-        <v>2192.618</v>
+        <v>2077.558</v>
       </c>
     </row>
     <row r="46">
@@ -3520,24 +3520,24 @@
         </is>
       </c>
       <c r="C46" s="8" t="n">
-        <v>108.834</v>
+        <v>27.1415</v>
       </c>
       <c r="D46" s="8" t="n">
-        <v>34.511</v>
+        <v>32.8875</v>
       </c>
       <c r="E46" s="8" t="n">
-        <v>19.769</v>
+        <v>20.1445</v>
       </c>
       <c r="F46" s="8" t="n">
-        <v>11.008</v>
+        <v>10.767</v>
       </c>
       <c r="G46" s="8" t="n">
-        <v>63.611</v>
+        <v>63.1075</v>
       </c>
       <c r="H46" s="9" t="n"/>
       <c r="I46" s="9" t="n"/>
       <c r="J46" s="8" t="n">
-        <v>69.32850000000001</v>
+        <v>68.863</v>
       </c>
     </row>
     <row r="47">
@@ -3548,24 +3548,24 @@
         </is>
       </c>
       <c r="C47" s="8" t="n">
-        <v>78.89400000000001</v>
+        <v>78.2985</v>
       </c>
       <c r="D47" s="8" t="n">
-        <v>83.90900000000001</v>
+        <v>83.581</v>
       </c>
       <c r="E47" s="8" t="n">
-        <v>79.56999999999999</v>
+        <v>79.298</v>
       </c>
       <c r="F47" s="8" t="n">
-        <v>80.16500000000001</v>
+        <v>78.566</v>
       </c>
       <c r="G47" s="8" t="n">
-        <v>78.27200000000001</v>
+        <v>78.45950000000001</v>
       </c>
       <c r="H47" s="9" t="n"/>
       <c r="I47" s="9" t="n"/>
       <c r="J47" s="8" t="n">
-        <v>79.371</v>
+        <v>79.4115</v>
       </c>
     </row>
     <row r="48">
@@ -3576,24 +3576,24 @@
         </is>
       </c>
       <c r="C48" s="8" t="n">
-        <v>89.98399999999999</v>
+        <v>93.62649999999999</v>
       </c>
       <c r="D48" s="8" t="n">
-        <v>90.1735</v>
+        <v>90.98650000000001</v>
       </c>
       <c r="E48" s="8" t="n">
-        <v>89.9315</v>
+        <v>88.2325</v>
       </c>
       <c r="F48" s="8" t="n">
-        <v>91.13849999999999</v>
+        <v>89.099</v>
       </c>
       <c r="G48" s="8" t="n">
-        <v>89.0185</v>
+        <v>89.56999999999999</v>
       </c>
       <c r="H48" s="9" t="n"/>
       <c r="I48" s="9" t="n"/>
       <c r="J48" s="8" t="n">
-        <v>90.349</v>
+        <v>89.8185</v>
       </c>
     </row>
     <row r="49">
@@ -3604,24 +3604,24 @@
         </is>
       </c>
       <c r="C49" s="8" t="n">
-        <v>277.701</v>
+        <v>199.152</v>
       </c>
       <c r="D49" s="8" t="n">
-        <v>208.468</v>
+        <v>207.4225</v>
       </c>
       <c r="E49" s="8" t="n">
-        <v>189.4175</v>
+        <v>187.7505</v>
       </c>
       <c r="F49" s="8" t="n">
-        <v>182.1065</v>
+        <v>178.521</v>
       </c>
       <c r="G49" s="8" t="n">
-        <v>230.836</v>
+        <v>231.076</v>
       </c>
       <c r="H49" s="9" t="n"/>
       <c r="I49" s="9" t="n"/>
       <c r="J49" s="8" t="n">
-        <v>239.195</v>
+        <v>238.156</v>
       </c>
     </row>
     <row r="50">
@@ -3736,24 +3736,24 @@
         </is>
       </c>
       <c r="C53" s="8" t="n">
-        <v>39.0755</v>
+        <v>28.1305</v>
       </c>
       <c r="D53" s="8" t="n">
-        <v>44.7315</v>
+        <v>37.7875</v>
       </c>
       <c r="E53" s="8" t="n">
-        <v>32.192</v>
+        <v>30.688</v>
       </c>
       <c r="F53" s="8" t="n">
-        <v>33.0795</v>
+        <v>31.3265</v>
       </c>
       <c r="G53" s="8" t="n">
-        <v>37.267</v>
+        <v>36.7275</v>
       </c>
       <c r="H53" s="9" t="n"/>
       <c r="I53" s="9" t="n"/>
       <c r="J53" s="8" t="n">
-        <v>34.0715</v>
+        <v>33.2905</v>
       </c>
     </row>
     <row r="54">
@@ -3764,24 +3764,24 @@
         </is>
       </c>
       <c r="C54" s="8" t="n">
-        <v>19.165</v>
+        <v>19.244</v>
       </c>
       <c r="D54" s="8" t="n">
-        <v>23.8685</v>
+        <v>20.6725</v>
       </c>
       <c r="E54" s="8" t="n">
-        <v>19.7655</v>
+        <v>20.2135</v>
       </c>
       <c r="F54" s="8" t="n">
-        <v>21.875</v>
+        <v>19.1</v>
       </c>
       <c r="G54" s="8" t="n">
-        <v>21.257</v>
+        <v>23.5405</v>
       </c>
       <c r="H54" s="9" t="n"/>
       <c r="I54" s="9" t="n"/>
       <c r="J54" s="8" t="n">
-        <v>19.19</v>
+        <v>20.547</v>
       </c>
     </row>
     <row r="55">
@@ -3792,24 +3792,24 @@
         </is>
       </c>
       <c r="C55" s="8" t="n">
-        <v>0.9409999999999999</v>
+        <v>0.8985</v>
       </c>
       <c r="D55" s="8" t="n">
-        <v>1.0075</v>
+        <v>0.9105</v>
       </c>
       <c r="E55" s="8" t="n">
-        <v>1.007</v>
+        <v>0.9035</v>
       </c>
       <c r="F55" s="8" t="n">
-        <v>1</v>
+        <v>0.914</v>
       </c>
       <c r="G55" s="8" t="n">
-        <v>1.1835</v>
+        <v>1.191</v>
       </c>
       <c r="H55" s="9" t="n"/>
       <c r="I55" s="9" t="n"/>
       <c r="J55" s="8" t="n">
-        <v>0.9419999999999999</v>
+        <v>0.9195</v>
       </c>
     </row>
     <row r="56">
@@ -3820,24 +3820,24 @@
         </is>
       </c>
       <c r="C56" s="8" t="n">
-        <v>59.1735</v>
+        <v>48.2825</v>
       </c>
       <c r="D56" s="8" t="n">
-        <v>69.6125</v>
+        <v>59.3815</v>
       </c>
       <c r="E56" s="8" t="n">
-        <v>52.9695</v>
+        <v>51.8015</v>
       </c>
       <c r="F56" s="8" t="n">
-        <v>55.96</v>
+        <v>51.3375</v>
       </c>
       <c r="G56" s="8" t="n">
-        <v>59.709</v>
+        <v>61.514</v>
       </c>
       <c r="H56" s="9" t="n"/>
       <c r="I56" s="9" t="n"/>
       <c r="J56" s="8" t="n">
-        <v>54.347</v>
+        <v>54.7575</v>
       </c>
     </row>
     <row r="57">
@@ -3852,24 +3852,24 @@
         </is>
       </c>
       <c r="C57" s="8" t="n">
-        <v>80.377</v>
+        <v>81.78</v>
       </c>
       <c r="D57" s="8" t="n">
-        <v>30.196</v>
+        <v>30.1165</v>
       </c>
       <c r="E57" s="8" t="n">
-        <v>23.4155</v>
+        <v>24.1225</v>
       </c>
       <c r="F57" s="8" t="n">
-        <v>22.856</v>
+        <v>24.2605</v>
       </c>
       <c r="G57" s="8" t="n">
-        <v>51.2205</v>
+        <v>50.287</v>
       </c>
       <c r="H57" s="9" t="n"/>
       <c r="I57" s="9" t="n"/>
       <c r="J57" s="8" t="n">
-        <v>80.6755</v>
+        <v>79.8085</v>
       </c>
     </row>
     <row r="58">
@@ -3880,24 +3880,24 @@
         </is>
       </c>
       <c r="C58" s="8" t="n">
-        <v>27.9565</v>
+        <v>28.0925</v>
       </c>
       <c r="D58" s="8" t="n">
-        <v>28.104</v>
+        <v>28.085</v>
       </c>
       <c r="E58" s="8" t="n">
-        <v>28.0375</v>
+        <v>28.067</v>
       </c>
       <c r="F58" s="8" t="n">
-        <v>28.1695</v>
+        <v>28.052</v>
       </c>
       <c r="G58" s="8" t="n">
-        <v>27.9915</v>
+        <v>28.028</v>
       </c>
       <c r="H58" s="9" t="n"/>
       <c r="I58" s="9" t="n"/>
       <c r="J58" s="8" t="n">
-        <v>28.1395</v>
+        <v>28.136</v>
       </c>
     </row>
     <row r="59">
@@ -3908,24 +3908,24 @@
         </is>
       </c>
       <c r="C59" s="8" t="n">
-        <v>160.4965</v>
+        <v>161.345</v>
       </c>
       <c r="D59" s="8" t="n">
-        <v>162.0105</v>
+        <v>161.402</v>
       </c>
       <c r="E59" s="8" t="n">
-        <v>159.9325</v>
+        <v>161.0465</v>
       </c>
       <c r="F59" s="8" t="n">
-        <v>160.873</v>
+        <v>160.872</v>
       </c>
       <c r="G59" s="8" t="n">
-        <v>159.9815</v>
+        <v>160.5145</v>
       </c>
       <c r="H59" s="9" t="n"/>
       <c r="I59" s="9" t="n"/>
       <c r="J59" s="8" t="n">
-        <v>160.236</v>
+        <v>160.156</v>
       </c>
     </row>
     <row r="60">
@@ -3936,24 +3936,24 @@
         </is>
       </c>
       <c r="C60" s="8" t="n">
-        <v>269.1215</v>
+        <v>271.2215</v>
       </c>
       <c r="D60" s="8" t="n">
-        <v>220.4715</v>
+        <v>219.5055</v>
       </c>
       <c r="E60" s="8" t="n">
-        <v>212.381</v>
+        <v>213.709</v>
       </c>
       <c r="F60" s="8" t="n">
-        <v>212.9095</v>
+        <v>213.5735</v>
       </c>
       <c r="G60" s="8" t="n">
-        <v>239.585</v>
+        <v>239.0605</v>
       </c>
       <c r="H60" s="9" t="n"/>
       <c r="I60" s="9" t="n"/>
       <c r="J60" s="8" t="n">
-        <v>268.818</v>
+        <v>268.0645</v>
       </c>
     </row>
   </sheetData>
@@ -4695,7 +4695,7 @@
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
@@ -4815,7 +4815,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="62" customHeight="1">
+    <row r="3" ht="48" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Q3</t>
@@ -4832,16 +4832,14 @@
         <is>
           <t>orderkey: 4448.84 MB
 shipdate: 6586.64 MB
-shipdate_BPE: 188.47 MB
-total: 11223.95 MB</t>
+total: 11035.48 MB</t>
         </is>
       </c>
       <c r="D3" s="13" t="inlineStr">
         <is>
           <t>orderkey: 359.98 MB
 shipdate: 138.44 MB
-shipdate_BPE: 354.33 MB
-total: 852.75 MB</t>
+total: 498.42 MB</t>
         </is>
       </c>
       <c r="E3" s="13" t="inlineStr">
@@ -4988,7 +4986,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="90" customHeight="1">
+    <row r="6" ht="62" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Q6</t>
@@ -5007,9 +5005,7 @@
           <t>shipdate_GE: 48.83 MB
 discount: 89.91 MB
 quantity: 257.20 MB
-discount_BPE: 79.93 MB
-quantity_BPE: 79.58 MB
-total: 555.45 MB</t>
+total: 395.94 MB</t>
         </is>
       </c>
       <c r="D6" s="13" t="inlineStr">
@@ -5017,9 +5013,7 @@
           <t>shipdate_GE: 52.56 MB
 discount: 82.57 MB
 quantity: 120.34 MB
-discount_BPE: 150.25 MB
-quantity_BPE: 154.94 MB
-total: 560.67 MB</t>
+total: 255.48 MB</t>
         </is>
       </c>
       <c r="E6" s="13" t="inlineStr">
@@ -5695,7 +5689,7 @@
         </is>
       </c>
       <c r="E9" s="15" t="n">
-        <v>11223.952</v>
+        <v>11035.48</v>
       </c>
     </row>
     <row r="10">
@@ -5720,7 +5714,7 @@
         </is>
       </c>
       <c r="E10" s="15" t="n">
-        <v>852.75</v>
+        <v>498.421</v>
       </c>
     </row>
     <row r="11">
@@ -6145,7 +6139,7 @@
         </is>
       </c>
       <c r="E27" s="15" t="n">
-        <v>555.4544000000001</v>
+        <v>395.9385</v>
       </c>
     </row>
     <row r="28">
@@ -6170,7 +6164,7 @@
         </is>
       </c>
       <c r="E28" s="15" t="n">
-        <v>560.6653</v>
+        <v>255.4757</v>
       </c>
     </row>
     <row r="29">
@@ -7403,10 +7397,10 @@
         <v>1732.932</v>
       </c>
       <c r="C3" s="16" t="n">
-        <v>11223.952</v>
+        <v>11035.48</v>
       </c>
       <c r="D3" s="16" t="n">
-        <v>852.75</v>
+        <v>498.421</v>
       </c>
       <c r="E3" s="16" t="n">
         <v>395.597</v>
@@ -7493,10 +7487,10 @@
         <v>412.1922</v>
       </c>
       <c r="C6" s="16" t="n">
-        <v>555.4544000000001</v>
+        <v>395.9385</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>560.6653</v>
+        <v>255.4757</v>
       </c>
       <c r="E6" s="16" t="n">
         <v>255.4297</v>

</xml_diff>

<commit_message>
SparseDDC ultra-sparse fast path: bypass L1/L2/L3/L4 for ≤64-bit
</commit_message>
<xml_diff>
--- a/bm_resultL4.xlsx
+++ b/bm_resultL4.xlsx
@@ -1699,24 +1699,24 @@
         </is>
       </c>
       <c r="B2" s="8" t="n">
-        <v>1771.5575</v>
+        <v>1770.7075</v>
       </c>
       <c r="C2" s="8" t="n">
-        <v>1012.2755</v>
+        <v>910.842</v>
       </c>
       <c r="D2" s="8" t="n">
-        <v>1544.949</v>
+        <v>1542.4375</v>
       </c>
       <c r="E2" s="8" t="n">
-        <v>1517.6855</v>
+        <v>1515.896</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>1184.7615</v>
+        <v>1183.1345</v>
       </c>
       <c r="G2" s="9" t="n"/>
       <c r="H2" s="9" t="n"/>
       <c r="I2" s="8" t="n">
-        <v>1247.413</v>
+        <v>1251.1105</v>
       </c>
       <c r="J2" s="9" t="n"/>
     </row>
@@ -1727,24 +1727,24 @@
         </is>
       </c>
       <c r="B3" s="8" t="n">
-        <v>986.3</v>
+        <v>998.9295</v>
       </c>
       <c r="C3" s="8" t="n">
-        <v>2733.8415</v>
+        <v>2642.7335</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>2658.403</v>
+        <v>2647.1515</v>
       </c>
       <c r="E3" s="8" t="n">
-        <v>1387.7285</v>
+        <v>1410.4455</v>
       </c>
       <c r="F3" s="8" t="n">
-        <v>5220.1315</v>
+        <v>4915.181</v>
       </c>
       <c r="G3" s="9" t="n"/>
       <c r="H3" s="9" t="n"/>
       <c r="I3" s="8" t="n">
-        <v>5505.849</v>
+        <v>5581.2905</v>
       </c>
       <c r="J3" s="9" t="n"/>
     </row>
@@ -1755,24 +1755,24 @@
         </is>
       </c>
       <c r="B4" s="8" t="n">
-        <v>712.918</v>
+        <v>711.649</v>
       </c>
       <c r="C4" s="8" t="n">
-        <v>706.628</v>
+        <v>668.8935</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>1011.319</v>
+        <v>1008.782</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>727.4915</v>
+        <v>700.463</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>1156.5055</v>
+        <v>1152.927</v>
       </c>
       <c r="G4" s="9" t="n"/>
       <c r="H4" s="9" t="n"/>
       <c r="I4" s="8" t="n">
-        <v>1137.0765</v>
+        <v>1121.333</v>
       </c>
       <c r="J4" s="9" t="n"/>
     </row>
@@ -1783,24 +1783,24 @@
         </is>
       </c>
       <c r="B5" s="8" t="n">
-        <v>589.2085</v>
+        <v>599.105</v>
       </c>
       <c r="C5" s="8" t="n">
-        <v>2208.1095</v>
+        <v>2108.9535</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>2829.593</v>
+        <v>2824.7625</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>915.737</v>
+        <v>915.125</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>3057.966</v>
+        <v>3116.3675</v>
       </c>
       <c r="G5" s="9" t="n"/>
       <c r="H5" s="9" t="n"/>
       <c r="I5" s="8" t="n">
-        <v>3008.5785</v>
+        <v>3012.8215</v>
       </c>
       <c r="J5" s="9" t="n"/>
     </row>
@@ -1811,24 +1811,24 @@
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>140.626</v>
+        <v>141.255</v>
       </c>
       <c r="C6" s="8" t="n">
-        <v>43.008</v>
+        <v>40.402</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>55.75</v>
+        <v>57.085</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>38.737</v>
+        <v>38.755</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>210.698</v>
+        <v>213.217</v>
       </c>
       <c r="G6" s="9" t="n"/>
       <c r="H6" s="9" t="n"/>
       <c r="I6" s="8" t="n">
-        <v>596.005</v>
+        <v>592.515</v>
       </c>
       <c r="J6" s="9" t="n"/>
     </row>
@@ -1839,24 +1839,24 @@
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>637.175</v>
+        <v>636.266</v>
       </c>
       <c r="C7" s="8" t="n">
-        <v>851.3105</v>
+        <v>583.7695</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>1877.5465</v>
+        <v>1878.9945</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>930.5575</v>
+        <v>930.121</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>1444.4775</v>
+        <v>1425.4075</v>
       </c>
       <c r="G7" s="9" t="n"/>
       <c r="H7" s="9" t="n"/>
       <c r="I7" s="8" t="n">
-        <v>1421.486</v>
+        <v>1429.9245</v>
       </c>
       <c r="J7" s="9" t="n"/>
     </row>
@@ -1867,24 +1867,24 @@
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>437.0685</v>
+        <v>433.2185</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>454.524</v>
+        <v>403.4925</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>1027.5375</v>
+        <v>1041.9455</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>572.5855</v>
+        <v>569.976</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>878.981</v>
+        <v>873.5055</v>
       </c>
       <c r="G8" s="9" t="n"/>
       <c r="H8" s="9" t="n"/>
       <c r="I8" s="8" t="n">
-        <v>912.8895</v>
+        <v>880.7645</v>
       </c>
       <c r="J8" s="9" t="n"/>
     </row>
@@ -1895,24 +1895,24 @@
         </is>
       </c>
       <c r="B9" s="8" t="n">
-        <v>1401.4595</v>
+        <v>1149.375</v>
       </c>
       <c r="C9" s="8" t="n">
-        <v>1553.859</v>
+        <v>1578.578</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>1245.2665</v>
+        <v>1239.926</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>1094.998</v>
+        <v>1087.439</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>1918.92</v>
+        <v>1919.0865</v>
       </c>
       <c r="G9" s="9" t="n"/>
       <c r="H9" s="9" t="n"/>
       <c r="I9" s="8" t="n">
-        <v>2077.558</v>
+        <v>2085.74</v>
       </c>
       <c r="J9" s="9" t="n"/>
     </row>
@@ -1923,24 +1923,24 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>199.152</v>
+        <v>194.207</v>
       </c>
       <c r="C10" s="8" t="n">
-        <v>207.4225</v>
+        <v>205.01</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>187.7505</v>
+        <v>189.8705</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>178.521</v>
+        <v>177.102</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>231.076</v>
+        <v>230.475</v>
       </c>
       <c r="G10" s="9" t="n"/>
       <c r="H10" s="9" t="n"/>
       <c r="I10" s="8" t="n">
-        <v>238.156</v>
+        <v>237.3535</v>
       </c>
       <c r="J10" s="9" t="n"/>
     </row>
@@ -1985,24 +1985,24 @@
         </is>
       </c>
       <c r="B12" s="8" t="n">
-        <v>48.2825</v>
+        <v>48.277</v>
       </c>
       <c r="C12" s="8" t="n">
-        <v>59.3815</v>
+        <v>46.2445</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>51.8015</v>
+        <v>52.5005</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>51.3375</v>
+        <v>53.2565</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>61.514</v>
+        <v>57.1535</v>
       </c>
       <c r="G12" s="9" t="n"/>
       <c r="H12" s="9" t="n"/>
       <c r="I12" s="8" t="n">
-        <v>54.7575</v>
+        <v>54.098</v>
       </c>
       <c r="J12" s="9" t="n"/>
     </row>
@@ -2013,24 +2013,24 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>271.2215</v>
+        <v>270.6675</v>
       </c>
       <c r="C13" s="8" t="n">
-        <v>219.5055</v>
+        <v>215.509</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>213.709</v>
+        <v>212.107</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>213.5735</v>
+        <v>212.0205</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>239.0605</v>
+        <v>238.932</v>
       </c>
       <c r="G13" s="9" t="n"/>
       <c r="H13" s="9" t="n"/>
       <c r="I13" s="8" t="n">
-        <v>268.0645</v>
+        <v>269.153</v>
       </c>
       <c r="J13" s="9" t="n"/>
     </row>
@@ -2268,24 +2268,24 @@
         </is>
       </c>
       <c r="C2" s="8" t="n">
-        <v>25.379</v>
+        <v>25.697</v>
       </c>
       <c r="D2" s="8" t="n">
-        <v>75.07250000000001</v>
+        <v>70.967</v>
       </c>
       <c r="E2" s="8" t="n">
-        <v>35.203</v>
+        <v>34.924</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>12.917</v>
+        <v>12.7805</v>
       </c>
       <c r="G2" s="8" t="n">
-        <v>77.955</v>
+        <v>78.14100000000001</v>
       </c>
       <c r="H2" s="9" t="n"/>
       <c r="I2" s="9" t="n"/>
       <c r="J2" s="8" t="n">
-        <v>84.04000000000001</v>
+        <v>84.9545</v>
       </c>
     </row>
     <row r="3">
@@ -2296,24 +2296,24 @@
         </is>
       </c>
       <c r="C3" s="8" t="n">
-        <v>993.7465</v>
+        <v>989.5775</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>179.395</v>
+        <v>80.2315</v>
       </c>
       <c r="E3" s="8" t="n">
-        <v>752.8535000000001</v>
+        <v>751.0645</v>
       </c>
       <c r="F3" s="8" t="n">
-        <v>748.6395</v>
+        <v>749.671</v>
       </c>
       <c r="G3" s="8" t="n">
-        <v>351.736</v>
+        <v>352.484</v>
       </c>
       <c r="H3" s="9" t="n"/>
       <c r="I3" s="9" t="n"/>
       <c r="J3" s="8" t="n">
-        <v>406.8655</v>
+        <v>411.5745</v>
       </c>
     </row>
     <row r="4">
@@ -2324,24 +2324,24 @@
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>752.597</v>
+        <v>755.385</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>757.809</v>
+        <v>759.785</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>756.95</v>
+        <v>756.678</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>756.0335</v>
+        <v>753.8395</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>754.87</v>
+        <v>752.688</v>
       </c>
       <c r="H4" s="9" t="n"/>
       <c r="I4" s="9" t="n"/>
       <c r="J4" s="8" t="n">
-        <v>756.403</v>
+        <v>754.3985</v>
       </c>
     </row>
     <row r="5">
@@ -2352,24 +2352,24 @@
         </is>
       </c>
       <c r="C5" s="8" t="n">
-        <v>1771.5575</v>
+        <v>1770.7075</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>1012.2755</v>
+        <v>910.842</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>1544.949</v>
+        <v>1542.4375</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>1517.6855</v>
+        <v>1515.896</v>
       </c>
       <c r="G5" s="8" t="n">
-        <v>1184.7615</v>
+        <v>1183.1345</v>
       </c>
       <c r="H5" s="9" t="n"/>
       <c r="I5" s="9" t="n"/>
       <c r="J5" s="8" t="n">
-        <v>1247.413</v>
+        <v>1251.1105</v>
       </c>
     </row>
     <row r="6">
@@ -2384,24 +2384,24 @@
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>21.9785</v>
+        <v>22.0045</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>24.5645</v>
+        <v>23.885</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>22.7995</v>
+        <v>22.6195</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>22.1705</v>
+        <v>22.37</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>22.653</v>
+        <v>22.4295</v>
       </c>
       <c r="H6" s="9" t="n"/>
       <c r="I6" s="9" t="n"/>
       <c r="J6" s="8" t="n">
-        <v>22.806</v>
+        <v>22.862</v>
       </c>
     </row>
     <row r="7">
@@ -2412,24 +2412,24 @@
         </is>
       </c>
       <c r="C7" s="8" t="n">
-        <v>741.4974999999999</v>
+        <v>752.1420000000001</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>790.992</v>
+        <v>695.7954999999999</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>2252.8125</v>
+        <v>2242.619</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>1152.1975</v>
+        <v>1175.4295</v>
       </c>
       <c r="G7" s="8" t="n">
-        <v>2062.2385</v>
+        <v>1984.6425</v>
       </c>
       <c r="H7" s="9" t="n"/>
       <c r="I7" s="9" t="n"/>
       <c r="J7" s="8" t="n">
-        <v>1918.047</v>
+        <v>1959.9195</v>
       </c>
     </row>
     <row r="8">
@@ -2440,24 +2440,24 @@
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>132.2875</v>
+        <v>133.784</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>1829.6715</v>
+        <v>1836.6485</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>293.417</v>
+        <v>293.264</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>125.386</v>
+        <v>125.0125</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>3042.0555</v>
+        <v>2815.547</v>
       </c>
       <c r="H8" s="9" t="n"/>
       <c r="I8" s="9" t="n"/>
       <c r="J8" s="8" t="n">
-        <v>3452.935</v>
+        <v>3489.3805</v>
       </c>
     </row>
     <row r="9">
@@ -2468,24 +2468,24 @@
         </is>
       </c>
       <c r="C9" s="8" t="n">
-        <v>8.0075</v>
+        <v>8.083</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>6.1145</v>
+        <v>5.659</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>5.414</v>
+        <v>5.459</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>5.2895</v>
+        <v>5.3515</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>9.903</v>
+        <v>9.8065</v>
       </c>
       <c r="H9" s="9" t="n"/>
       <c r="I9" s="9" t="n"/>
       <c r="J9" s="8" t="n">
-        <v>27.853</v>
+        <v>28.1425</v>
       </c>
     </row>
     <row r="10">
@@ -2496,24 +2496,24 @@
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>82.1955</v>
+        <v>82.735</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>82.663</v>
+        <v>81.998</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>83.27800000000001</v>
+        <v>82.866</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>82.92100000000001</v>
+        <v>82.38800000000001</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>83.0035</v>
+        <v>82.754</v>
       </c>
       <c r="H10" s="9" t="n"/>
       <c r="I10" s="9" t="n"/>
       <c r="J10" s="8" t="n">
-        <v>83.575</v>
+        <v>83.23699999999999</v>
       </c>
     </row>
     <row r="11">
@@ -2524,24 +2524,24 @@
         </is>
       </c>
       <c r="C11" s="8" t="n">
-        <v>986.3</v>
+        <v>998.9295</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>2733.8415</v>
+        <v>2642.7335</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>2658.403</v>
+        <v>2647.1515</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>1387.7285</v>
+        <v>1410.4455</v>
       </c>
       <c r="G11" s="8" t="n">
-        <v>5220.1315</v>
+        <v>4915.181</v>
       </c>
       <c r="H11" s="9" t="n"/>
       <c r="I11" s="9" t="n"/>
       <c r="J11" s="8" t="n">
-        <v>5505.849</v>
+        <v>5581.2905</v>
       </c>
     </row>
     <row r="12">
@@ -2556,24 +2556,24 @@
         </is>
       </c>
       <c r="C12" s="8" t="n">
-        <v>248.3445</v>
+        <v>243.3005</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>250.8645</v>
+        <v>251.0175</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>247.1135</v>
+        <v>243.4275</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>248.662</v>
+        <v>242.933</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>250.4495</v>
+        <v>244.454</v>
       </c>
       <c r="H12" s="9" t="n"/>
       <c r="I12" s="9" t="n"/>
       <c r="J12" s="8" t="n">
-        <v>252.3425</v>
+        <v>242.656</v>
       </c>
     </row>
     <row r="13">
@@ -2584,24 +2584,24 @@
         </is>
       </c>
       <c r="C13" s="8" t="n">
-        <v>166.96</v>
+        <v>168.4515</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>157.073</v>
+        <v>117.795</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>468.833</v>
+        <v>467.4755</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>158.9485</v>
+        <v>161.489</v>
       </c>
       <c r="G13" s="8" t="n">
-        <v>606.278</v>
+        <v>605.947</v>
       </c>
       <c r="H13" s="9" t="n"/>
       <c r="I13" s="9" t="n"/>
       <c r="J13" s="8" t="n">
-        <v>585.3915</v>
+        <v>582.4835</v>
       </c>
     </row>
     <row r="14">
@@ -2612,24 +2612,24 @@
         </is>
       </c>
       <c r="C14" s="8" t="n">
-        <v>237.5485</v>
+        <v>239.6245</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>236.966</v>
+        <v>236.8985</v>
       </c>
       <c r="E14" s="8" t="n">
-        <v>236.0865</v>
+        <v>236.7835</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>260.0905</v>
+        <v>236.7</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>237.5845</v>
+        <v>236.8495</v>
       </c>
       <c r="H14" s="9" t="n"/>
       <c r="I14" s="9" t="n"/>
       <c r="J14" s="8" t="n">
-        <v>237.6925</v>
+        <v>235.067</v>
       </c>
     </row>
     <row r="15">
@@ -2640,24 +2640,24 @@
         </is>
       </c>
       <c r="C15" s="8" t="n">
-        <v>59.425</v>
+        <v>59.2865</v>
       </c>
       <c r="D15" s="8" t="n">
-        <v>61.6425</v>
+        <v>61.5465</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>60.2995</v>
+        <v>61.5625</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>58.876</v>
+        <v>60.1005</v>
       </c>
       <c r="G15" s="8" t="n">
-        <v>62.3555</v>
+        <v>63.5335</v>
       </c>
       <c r="H15" s="9" t="n"/>
       <c r="I15" s="9" t="n"/>
       <c r="J15" s="8" t="n">
-        <v>62.6025</v>
+        <v>60.901</v>
       </c>
     </row>
     <row r="16">
@@ -2668,24 +2668,24 @@
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>712.918</v>
+        <v>711.649</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>706.628</v>
+        <v>668.8935</v>
       </c>
       <c r="E16" s="8" t="n">
-        <v>1011.319</v>
+        <v>1008.782</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>727.4915</v>
+        <v>700.463</v>
       </c>
       <c r="G16" s="8" t="n">
-        <v>1156.5055</v>
+        <v>1152.927</v>
       </c>
       <c r="H16" s="9" t="n"/>
       <c r="I16" s="9" t="n"/>
       <c r="J16" s="8" t="n">
-        <v>1137.0765</v>
+        <v>1121.333</v>
       </c>
     </row>
     <row r="17">
@@ -2700,24 +2700,24 @@
         </is>
       </c>
       <c r="C17" s="8" t="n">
-        <v>278.728</v>
+        <v>284.968</v>
       </c>
       <c r="D17" s="8" t="n">
-        <v>322.153</v>
+        <v>313.9575</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>285.663</v>
+        <v>283.5675</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>279.536</v>
+        <v>282.5625</v>
       </c>
       <c r="G17" s="8" t="n">
-        <v>304.087</v>
+        <v>289.7045</v>
       </c>
       <c r="H17" s="9" t="n"/>
       <c r="I17" s="9" t="n"/>
       <c r="J17" s="8" t="n">
-        <v>296.185</v>
+        <v>285.8005</v>
       </c>
     </row>
     <row r="18">
@@ -2728,24 +2728,24 @@
         </is>
       </c>
       <c r="C18" s="8" t="n">
-        <v>189.7035</v>
+        <v>193.3805</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>1758.4335</v>
+        <v>1668.389</v>
       </c>
       <c r="E18" s="8" t="n">
-        <v>2420.751</v>
+        <v>2417.007</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>512.9085</v>
+        <v>510.526</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>2628.8265</v>
+        <v>2701.529</v>
       </c>
       <c r="H18" s="9" t="n"/>
       <c r="I18" s="9" t="n"/>
       <c r="J18" s="8" t="n">
-        <v>2587.23</v>
+        <v>2602.405</v>
       </c>
     </row>
     <row r="19">
@@ -2756,24 +2756,24 @@
         </is>
       </c>
       <c r="C19" s="8" t="n">
-        <v>119.7535</v>
+        <v>119.641</v>
       </c>
       <c r="D19" s="8" t="n">
-        <v>127.378</v>
+        <v>125.852</v>
       </c>
       <c r="E19" s="8" t="n">
-        <v>124.0705</v>
+        <v>124.1315</v>
       </c>
       <c r="F19" s="8" t="n">
-        <v>123.5005</v>
+        <v>122.0595</v>
       </c>
       <c r="G19" s="8" t="n">
-        <v>124.439</v>
+        <v>125.2965</v>
       </c>
       <c r="H19" s="9" t="n"/>
       <c r="I19" s="9" t="n"/>
       <c r="J19" s="8" t="n">
-        <v>125.344</v>
+        <v>124.216</v>
       </c>
     </row>
     <row r="20">
@@ -2784,24 +2784,24 @@
         </is>
       </c>
       <c r="C20" s="8" t="n">
-        <v>589.2085</v>
+        <v>599.105</v>
       </c>
       <c r="D20" s="8" t="n">
-        <v>2208.1095</v>
+        <v>2108.9535</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>2829.593</v>
+        <v>2824.7625</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>915.737</v>
+        <v>915.125</v>
       </c>
       <c r="G20" s="8" t="n">
-        <v>3057.966</v>
+        <v>3116.3675</v>
       </c>
       <c r="H20" s="9" t="n"/>
       <c r="I20" s="9" t="n"/>
       <c r="J20" s="8" t="n">
-        <v>3008.5785</v>
+        <v>3012.8215</v>
       </c>
     </row>
     <row r="21">
@@ -2816,24 +2816,24 @@
         </is>
       </c>
       <c r="C21" s="8" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.004</v>
       </c>
       <c r="D21" s="8" t="n">
-        <v>2.106</v>
+        <v>1.076</v>
       </c>
       <c r="E21" s="8" t="n">
-        <v>0.958</v>
+        <v>0.957</v>
       </c>
       <c r="F21" s="8" t="n">
-        <v>1.008</v>
+        <v>0.972</v>
       </c>
       <c r="G21" s="8" t="n">
-        <v>2.867</v>
+        <v>2.631</v>
       </c>
       <c r="H21" s="9" t="n"/>
       <c r="I21" s="9" t="n"/>
       <c r="J21" s="8" t="n">
-        <v>1.1</v>
+        <v>1.122</v>
       </c>
     </row>
     <row r="22">
@@ -2844,24 +2844,24 @@
         </is>
       </c>
       <c r="C22" s="8" t="n">
-        <v>12.701</v>
+        <v>12.509</v>
       </c>
       <c r="D22" s="8" t="n">
-        <v>5.704</v>
+        <v>5.175</v>
       </c>
       <c r="E22" s="8" t="n">
-        <v>2.37</v>
+        <v>2.402</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>2.614</v>
+        <v>2.347</v>
       </c>
       <c r="G22" s="8" t="n">
-        <v>5.845</v>
+        <v>5.889</v>
       </c>
       <c r="H22" s="9" t="n"/>
       <c r="I22" s="9" t="n"/>
       <c r="J22" s="8" t="n">
-        <v>26.296</v>
+        <v>26.174</v>
       </c>
     </row>
     <row r="23">
@@ -2872,24 +2872,24 @@
         </is>
       </c>
       <c r="C23" s="8" t="n">
-        <v>91.173</v>
+        <v>91.461</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>23.905</v>
+        <v>23.55</v>
       </c>
       <c r="E23" s="8" t="n">
-        <v>33.432</v>
+        <v>33.847</v>
       </c>
       <c r="F23" s="8" t="n">
-        <v>15.748</v>
+        <v>16.166</v>
       </c>
       <c r="G23" s="8" t="n">
-        <v>177.337</v>
+        <v>180.112</v>
       </c>
       <c r="H23" s="9" t="n"/>
       <c r="I23" s="9" t="n"/>
       <c r="J23" s="8" t="n">
-        <v>488.858</v>
+        <v>485.368</v>
       </c>
     </row>
     <row r="24">
@@ -2900,24 +2900,24 @@
         </is>
       </c>
       <c r="C24" s="8" t="n">
-        <v>3.762</v>
+        <v>3.787</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>3.535</v>
+        <v>2.165</v>
       </c>
       <c r="E24" s="8" t="n">
-        <v>13.163</v>
+        <v>13.397</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>13.38</v>
+        <v>13.286</v>
       </c>
       <c r="G24" s="8" t="n">
-        <v>12.335</v>
+        <v>12.299</v>
       </c>
       <c r="H24" s="9" t="n"/>
       <c r="I24" s="9" t="n"/>
       <c r="J24" s="8" t="n">
-        <v>63.11</v>
+        <v>63.313</v>
       </c>
     </row>
     <row r="25">
@@ -2928,24 +2928,24 @@
         </is>
       </c>
       <c r="C25" s="8" t="n">
-        <v>32.97</v>
+        <v>33.485</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>7.169</v>
+        <v>7.23</v>
       </c>
       <c r="E25" s="8" t="n">
-        <v>5.818</v>
+        <v>6.475</v>
       </c>
       <c r="F25" s="8" t="n">
         <v>5.976</v>
       </c>
       <c r="G25" s="8" t="n">
-        <v>12.303</v>
+        <v>12.275</v>
       </c>
       <c r="H25" s="9" t="n"/>
       <c r="I25" s="9" t="n"/>
       <c r="J25" s="8" t="n">
-        <v>16.633</v>
+        <v>16.528</v>
       </c>
     </row>
     <row r="26">
@@ -2956,24 +2956,24 @@
         </is>
       </c>
       <c r="C26" s="8" t="n">
-        <v>140.626</v>
+        <v>141.255</v>
       </c>
       <c r="D26" s="8" t="n">
-        <v>43.008</v>
+        <v>40.402</v>
       </c>
       <c r="E26" s="8" t="n">
-        <v>55.75</v>
+        <v>57.085</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>38.737</v>
+        <v>38.755</v>
       </c>
       <c r="G26" s="8" t="n">
-        <v>210.698</v>
+        <v>213.217</v>
       </c>
       <c r="H26" s="9" t="n"/>
       <c r="I26" s="9" t="n"/>
       <c r="J26" s="8" t="n">
-        <v>596.005</v>
+        <v>592.515</v>
       </c>
     </row>
     <row r="27">
@@ -2988,24 +2988,24 @@
         </is>
       </c>
       <c r="C27" s="8" t="n">
-        <v>88.072</v>
+        <v>88.008</v>
       </c>
       <c r="D27" s="8" t="n">
-        <v>136.1105</v>
+        <v>88.0305</v>
       </c>
       <c r="E27" s="8" t="n">
-        <v>88.245</v>
+        <v>88.23050000000001</v>
       </c>
       <c r="F27" s="8" t="n">
-        <v>88.077</v>
+        <v>87.86799999999999</v>
       </c>
       <c r="G27" s="8" t="n">
-        <v>88.4485</v>
+        <v>88.345</v>
       </c>
       <c r="H27" s="9" t="n"/>
       <c r="I27" s="9" t="n"/>
       <c r="J27" s="8" t="n">
-        <v>88.404</v>
+        <v>88.205</v>
       </c>
     </row>
     <row r="28">
@@ -3016,24 +3016,24 @@
         </is>
       </c>
       <c r="C28" s="8" t="n">
-        <v>346.3885</v>
+        <v>347.4085</v>
       </c>
       <c r="D28" s="8" t="n">
-        <v>418.221</v>
+        <v>342.185</v>
       </c>
       <c r="E28" s="8" t="n">
-        <v>344.0195</v>
+        <v>345.041</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>348.794</v>
+        <v>349.734</v>
       </c>
       <c r="G28" s="8" t="n">
-        <v>351.883</v>
+        <v>348.4885</v>
       </c>
       <c r="H28" s="9" t="n"/>
       <c r="I28" s="9" t="n"/>
       <c r="J28" s="8" t="n">
-        <v>349.57</v>
+        <v>346.4155</v>
       </c>
     </row>
     <row r="29">
@@ -3044,24 +3044,24 @@
         </is>
       </c>
       <c r="C29" s="8" t="n">
-        <v>174.9085</v>
+        <v>172.7905</v>
       </c>
       <c r="D29" s="8" t="n">
-        <v>263.103</v>
+        <v>124.841</v>
       </c>
       <c r="E29" s="8" t="n">
-        <v>1416.3165</v>
+        <v>1414.635</v>
       </c>
       <c r="F29" s="8" t="n">
-        <v>465.004</v>
+        <v>463.6225</v>
       </c>
       <c r="G29" s="8" t="n">
-        <v>974.0940000000001</v>
+        <v>958.927</v>
       </c>
       <c r="H29" s="9" t="n"/>
       <c r="I29" s="9" t="n"/>
       <c r="J29" s="8" t="n">
-        <v>954.6965</v>
+        <v>964.577</v>
       </c>
     </row>
     <row r="30">
@@ -3072,24 +3072,24 @@
         </is>
       </c>
       <c r="C30" s="8" t="n">
-        <v>28.7695</v>
+        <v>28.434</v>
       </c>
       <c r="D30" s="8" t="n">
-        <v>34.0235</v>
+        <v>29.366</v>
       </c>
       <c r="E30" s="8" t="n">
-        <v>28.955</v>
+        <v>28.963</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>29.241</v>
+        <v>28.976</v>
       </c>
       <c r="G30" s="8" t="n">
-        <v>29.1405</v>
+        <v>29.016</v>
       </c>
       <c r="H30" s="9" t="n"/>
       <c r="I30" s="9" t="n"/>
       <c r="J30" s="8" t="n">
-        <v>29.493</v>
+        <v>28.9855</v>
       </c>
     </row>
     <row r="31">
@@ -3116,24 +3116,24 @@
         </is>
       </c>
       <c r="C32" s="8" t="n">
-        <v>637.175</v>
+        <v>636.266</v>
       </c>
       <c r="D32" s="8" t="n">
-        <v>851.3105</v>
+        <v>583.7695</v>
       </c>
       <c r="E32" s="8" t="n">
-        <v>1877.5465</v>
+        <v>1878.9945</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>930.5575</v>
+        <v>930.121</v>
       </c>
       <c r="G32" s="8" t="n">
-        <v>1444.4775</v>
+        <v>1425.4075</v>
       </c>
       <c r="H32" s="9" t="n"/>
       <c r="I32" s="9" t="n"/>
       <c r="J32" s="8" t="n">
-        <v>1421.486</v>
+        <v>1429.9245</v>
       </c>
     </row>
     <row r="33">
@@ -3148,24 +3148,24 @@
         </is>
       </c>
       <c r="C33" s="8" t="n">
-        <v>91.32599999999999</v>
+        <v>90.5665</v>
       </c>
       <c r="D33" s="8" t="n">
-        <v>97.834</v>
+        <v>93.068</v>
       </c>
       <c r="E33" s="8" t="n">
-        <v>89.58450000000001</v>
+        <v>91.19450000000001</v>
       </c>
       <c r="F33" s="8" t="n">
-        <v>90.59350000000001</v>
+        <v>91.14100000000001</v>
       </c>
       <c r="G33" s="8" t="n">
-        <v>93.1305</v>
+        <v>92.14749999999999</v>
       </c>
       <c r="H33" s="9" t="n"/>
       <c r="I33" s="9" t="n"/>
       <c r="J33" s="8" t="n">
-        <v>97.7265</v>
+        <v>90.47499999999999</v>
       </c>
     </row>
     <row r="34">
@@ -3176,24 +3176,24 @@
         </is>
       </c>
       <c r="C34" s="8" t="n">
-        <v>102.394</v>
+        <v>102.3325</v>
       </c>
       <c r="D34" s="8" t="n">
-        <v>115.203</v>
+        <v>74.3775</v>
       </c>
       <c r="E34" s="8" t="n">
-        <v>711.3935</v>
+        <v>725.1905</v>
       </c>
       <c r="F34" s="8" t="n">
-        <v>261.002</v>
+        <v>258.775</v>
       </c>
       <c r="G34" s="8" t="n">
-        <v>550.0170000000001</v>
+        <v>544.628</v>
       </c>
       <c r="H34" s="9" t="n"/>
       <c r="I34" s="9" t="n"/>
       <c r="J34" s="8" t="n">
-        <v>542.1375</v>
+        <v>534.086</v>
       </c>
     </row>
     <row r="35">
@@ -3207,21 +3207,21 @@
         <v>0.005</v>
       </c>
       <c r="D35" s="8" t="n">
-        <v>2.874</v>
+        <v>3.2675</v>
       </c>
       <c r="E35" s="8" t="n">
-        <v>1.1295</v>
+        <v>1.11</v>
       </c>
       <c r="F35" s="8" t="n">
-        <v>0.91</v>
+        <v>0.9105</v>
       </c>
       <c r="G35" s="8" t="n">
-        <v>1.337</v>
+        <v>1.4905</v>
       </c>
       <c r="H35" s="9" t="n"/>
       <c r="I35" s="9" t="n"/>
       <c r="J35" s="8" t="n">
-        <v>4.2565</v>
+        <v>1.364</v>
       </c>
     </row>
     <row r="36">
@@ -3232,24 +3232,24 @@
         </is>
       </c>
       <c r="C36" s="8" t="n">
-        <v>29.3795</v>
+        <v>29.307</v>
       </c>
       <c r="D36" s="8" t="n">
-        <v>19.056</v>
+        <v>21.7685</v>
       </c>
       <c r="E36" s="8" t="n">
-        <v>8.853</v>
+        <v>8.943</v>
       </c>
       <c r="F36" s="8" t="n">
-        <v>8.7235</v>
+        <v>8.4155</v>
       </c>
       <c r="G36" s="8" t="n">
-        <v>18.132</v>
+        <v>18.062</v>
       </c>
       <c r="H36" s="9" t="n"/>
       <c r="I36" s="9" t="n"/>
       <c r="J36" s="8" t="n">
-        <v>50.1475</v>
+        <v>38.3315</v>
       </c>
     </row>
     <row r="37">
@@ -3260,24 +3260,24 @@
         </is>
       </c>
       <c r="C37" s="8" t="n">
-        <v>206.362</v>
+        <v>202.7535</v>
       </c>
       <c r="D37" s="8" t="n">
-        <v>211.07</v>
+        <v>201.792</v>
       </c>
       <c r="E37" s="8" t="n">
-        <v>208.6615</v>
+        <v>208.0205</v>
       </c>
       <c r="F37" s="8" t="n">
-        <v>204.3935</v>
+        <v>203.468</v>
       </c>
       <c r="G37" s="8" t="n">
-        <v>209.014</v>
+        <v>209.428</v>
       </c>
       <c r="H37" s="9" t="n"/>
       <c r="I37" s="9" t="n"/>
       <c r="J37" s="8" t="n">
-        <v>210.673</v>
+        <v>208.5205</v>
       </c>
     </row>
     <row r="38">
@@ -3288,24 +3288,24 @@
         </is>
       </c>
       <c r="C38" s="8" t="n">
-        <v>7.6185</v>
+        <v>7.507</v>
       </c>
       <c r="D38" s="8" t="n">
-        <v>7.337</v>
+        <v>7.289</v>
       </c>
       <c r="E38" s="8" t="n">
-        <v>7.3625</v>
+        <v>7.5045</v>
       </c>
       <c r="F38" s="8" t="n">
-        <v>7.4385</v>
+        <v>7.4755</v>
       </c>
       <c r="G38" s="8" t="n">
-        <v>7.3475</v>
+        <v>7.7025</v>
       </c>
       <c r="H38" s="9" t="n"/>
       <c r="I38" s="9" t="n"/>
       <c r="J38" s="8" t="n">
-        <v>7.6295</v>
+        <v>7.5935</v>
       </c>
     </row>
     <row r="39">
@@ -3316,24 +3316,24 @@
         </is>
       </c>
       <c r="C39" s="8" t="n">
-        <v>437.0685</v>
+        <v>433.2185</v>
       </c>
       <c r="D39" s="8" t="n">
-        <v>454.524</v>
+        <v>403.4925</v>
       </c>
       <c r="E39" s="8" t="n">
-        <v>1027.5375</v>
+        <v>1041.9455</v>
       </c>
       <c r="F39" s="8" t="n">
-        <v>572.5855</v>
+        <v>569.976</v>
       </c>
       <c r="G39" s="8" t="n">
-        <v>878.981</v>
+        <v>873.5055</v>
       </c>
       <c r="H39" s="9" t="n"/>
       <c r="I39" s="9" t="n"/>
       <c r="J39" s="8" t="n">
-        <v>912.8895</v>
+        <v>880.7645</v>
       </c>
     </row>
     <row r="40">
@@ -3348,24 +3348,24 @@
         </is>
       </c>
       <c r="C40" s="8" t="n">
-        <v>852.3819999999999</v>
+        <v>604.7435</v>
       </c>
       <c r="D40" s="8" t="n">
-        <v>606.981</v>
+        <v>607.3645</v>
       </c>
       <c r="E40" s="8" t="n">
-        <v>606.4705</v>
+        <v>607.0625</v>
       </c>
       <c r="F40" s="8" t="n">
-        <v>610.2335</v>
+        <v>606.5045</v>
       </c>
       <c r="G40" s="8" t="n">
-        <v>607.681</v>
+        <v>606.4965</v>
       </c>
       <c r="H40" s="9" t="n"/>
       <c r="I40" s="9" t="n"/>
       <c r="J40" s="8" t="n">
-        <v>608.535</v>
+        <v>605.836</v>
       </c>
     </row>
     <row r="41">
@@ -3376,24 +3376,24 @@
         </is>
       </c>
       <c r="C41" s="8" t="n">
-        <v>3.8035</v>
+        <v>3.8685</v>
       </c>
       <c r="D41" s="8" t="n">
-        <v>5.0495</v>
+        <v>4.9885</v>
       </c>
       <c r="E41" s="8" t="n">
-        <v>1.678</v>
+        <v>1.73</v>
       </c>
       <c r="F41" s="8" t="n">
-        <v>1.6135</v>
+        <v>1.652</v>
       </c>
       <c r="G41" s="8" t="n">
-        <v>2.9055</v>
+        <v>2.887</v>
       </c>
       <c r="H41" s="9" t="n"/>
       <c r="I41" s="9" t="n"/>
       <c r="J41" s="8" t="n">
-        <v>11.774</v>
+        <v>11.544</v>
       </c>
     </row>
     <row r="42">
@@ -3404,24 +3404,24 @@
         </is>
       </c>
       <c r="C42" s="8" t="n">
-        <v>41.119</v>
+        <v>42.2055</v>
       </c>
       <c r="D42" s="8" t="n">
-        <v>493.86</v>
+        <v>508.794</v>
       </c>
       <c r="E42" s="8" t="n">
-        <v>206.014</v>
+        <v>208.543</v>
       </c>
       <c r="F42" s="8" t="n">
-        <v>37.966</v>
+        <v>37.9475</v>
       </c>
       <c r="G42" s="8" t="n">
-        <v>848.2965</v>
+        <v>852.8795</v>
       </c>
       <c r="H42" s="9" t="n"/>
       <c r="I42" s="9" t="n"/>
       <c r="J42" s="8" t="n">
-        <v>971.1605</v>
+        <v>981.1115</v>
       </c>
     </row>
     <row r="43">
@@ -3432,24 +3432,24 @@
         </is>
       </c>
       <c r="C43" s="8" t="n">
-        <v>86.669</v>
+        <v>87.2945</v>
       </c>
       <c r="D43" s="8" t="n">
-        <v>35.739</v>
+        <v>41.1325</v>
       </c>
       <c r="E43" s="8" t="n">
-        <v>26.0505</v>
+        <v>25.879</v>
       </c>
       <c r="F43" s="8" t="n">
-        <v>25.7945</v>
+        <v>26.0975</v>
       </c>
       <c r="G43" s="8" t="n">
-        <v>43.236</v>
+        <v>43.8405</v>
       </c>
       <c r="H43" s="9" t="n"/>
       <c r="I43" s="9" t="n"/>
       <c r="J43" s="8" t="n">
-        <v>72.6875</v>
+        <v>73.476</v>
       </c>
     </row>
     <row r="44">
@@ -3460,24 +3460,24 @@
         </is>
       </c>
       <c r="C44" s="8" t="n">
-        <v>418.314</v>
+        <v>410.5865</v>
       </c>
       <c r="D44" s="8" t="n">
-        <v>412.562</v>
+        <v>416.956</v>
       </c>
       <c r="E44" s="8" t="n">
-        <v>403.088</v>
+        <v>397.999</v>
       </c>
       <c r="F44" s="8" t="n">
-        <v>418.924</v>
+        <v>413.887</v>
       </c>
       <c r="G44" s="8" t="n">
-        <v>415.6475</v>
+        <v>412.892</v>
       </c>
       <c r="H44" s="9" t="n"/>
       <c r="I44" s="9" t="n"/>
       <c r="J44" s="8" t="n">
-        <v>414.3595</v>
+        <v>413.535</v>
       </c>
     </row>
     <row r="45">
@@ -3488,24 +3488,24 @@
         </is>
       </c>
       <c r="C45" s="8" t="n">
-        <v>1401.4595</v>
+        <v>1149.375</v>
       </c>
       <c r="D45" s="8" t="n">
-        <v>1553.859</v>
+        <v>1578.578</v>
       </c>
       <c r="E45" s="8" t="n">
-        <v>1245.2665</v>
+        <v>1239.926</v>
       </c>
       <c r="F45" s="8" t="n">
-        <v>1094.998</v>
+        <v>1087.439</v>
       </c>
       <c r="G45" s="8" t="n">
-        <v>1918.92</v>
+        <v>1919.0865</v>
       </c>
       <c r="H45" s="9" t="n"/>
       <c r="I45" s="9" t="n"/>
       <c r="J45" s="8" t="n">
-        <v>2077.558</v>
+        <v>2085.74</v>
       </c>
     </row>
     <row r="46">
@@ -3520,24 +3520,24 @@
         </is>
       </c>
       <c r="C46" s="8" t="n">
-        <v>27.1415</v>
+        <v>26.81</v>
       </c>
       <c r="D46" s="8" t="n">
-        <v>32.8875</v>
+        <v>31.5715</v>
       </c>
       <c r="E46" s="8" t="n">
-        <v>20.1445</v>
+        <v>20.447</v>
       </c>
       <c r="F46" s="8" t="n">
-        <v>10.767</v>
+        <v>10.6105</v>
       </c>
       <c r="G46" s="8" t="n">
-        <v>63.1075</v>
+        <v>63.226</v>
       </c>
       <c r="H46" s="9" t="n"/>
       <c r="I46" s="9" t="n"/>
       <c r="J46" s="8" t="n">
-        <v>68.863</v>
+        <v>69.44450000000001</v>
       </c>
     </row>
     <row r="47">
@@ -3548,24 +3548,24 @@
         </is>
       </c>
       <c r="C47" s="8" t="n">
-        <v>78.2985</v>
+        <v>78.7985</v>
       </c>
       <c r="D47" s="8" t="n">
-        <v>83.581</v>
+        <v>83.3985</v>
       </c>
       <c r="E47" s="8" t="n">
-        <v>79.298</v>
+        <v>79.8075</v>
       </c>
       <c r="F47" s="8" t="n">
-        <v>78.566</v>
+        <v>78.48050000000001</v>
       </c>
       <c r="G47" s="8" t="n">
-        <v>78.45950000000001</v>
+        <v>78.39749999999999</v>
       </c>
       <c r="H47" s="9" t="n"/>
       <c r="I47" s="9" t="n"/>
       <c r="J47" s="8" t="n">
-        <v>79.4115</v>
+        <v>78.968</v>
       </c>
     </row>
     <row r="48">
@@ -3576,24 +3576,24 @@
         </is>
       </c>
       <c r="C48" s="8" t="n">
-        <v>93.62649999999999</v>
+        <v>88.42149999999999</v>
       </c>
       <c r="D48" s="8" t="n">
-        <v>90.98650000000001</v>
+        <v>90.021</v>
       </c>
       <c r="E48" s="8" t="n">
-        <v>88.2325</v>
+        <v>89.2405</v>
       </c>
       <c r="F48" s="8" t="n">
-        <v>89.099</v>
+        <v>87.89400000000001</v>
       </c>
       <c r="G48" s="8" t="n">
-        <v>89.56999999999999</v>
+        <v>88.886</v>
       </c>
       <c r="H48" s="9" t="n"/>
       <c r="I48" s="9" t="n"/>
       <c r="J48" s="8" t="n">
-        <v>89.8185</v>
+        <v>88.90349999999999</v>
       </c>
     </row>
     <row r="49">
@@ -3604,24 +3604,24 @@
         </is>
       </c>
       <c r="C49" s="8" t="n">
-        <v>199.152</v>
+        <v>194.207</v>
       </c>
       <c r="D49" s="8" t="n">
-        <v>207.4225</v>
+        <v>205.01</v>
       </c>
       <c r="E49" s="8" t="n">
-        <v>187.7505</v>
+        <v>189.8705</v>
       </c>
       <c r="F49" s="8" t="n">
-        <v>178.521</v>
+        <v>177.102</v>
       </c>
       <c r="G49" s="8" t="n">
-        <v>231.076</v>
+        <v>230.475</v>
       </c>
       <c r="H49" s="9" t="n"/>
       <c r="I49" s="9" t="n"/>
       <c r="J49" s="8" t="n">
-        <v>238.156</v>
+        <v>237.3535</v>
       </c>
     </row>
     <row r="50">
@@ -3736,24 +3736,24 @@
         </is>
       </c>
       <c r="C53" s="8" t="n">
-        <v>28.1305</v>
+        <v>28.306</v>
       </c>
       <c r="D53" s="8" t="n">
-        <v>37.7875</v>
+        <v>26.6265</v>
       </c>
       <c r="E53" s="8" t="n">
-        <v>30.688</v>
+        <v>31.7045</v>
       </c>
       <c r="F53" s="8" t="n">
-        <v>31.3265</v>
+        <v>31.947</v>
       </c>
       <c r="G53" s="8" t="n">
-        <v>36.7275</v>
+        <v>35.6265</v>
       </c>
       <c r="H53" s="9" t="n"/>
       <c r="I53" s="9" t="n"/>
       <c r="J53" s="8" t="n">
-        <v>33.2905</v>
+        <v>33.113</v>
       </c>
     </row>
     <row r="54">
@@ -3764,24 +3764,24 @@
         </is>
       </c>
       <c r="C54" s="8" t="n">
-        <v>19.244</v>
+        <v>19.061</v>
       </c>
       <c r="D54" s="8" t="n">
-        <v>20.6725</v>
+        <v>18.7185</v>
       </c>
       <c r="E54" s="8" t="n">
-        <v>20.2135</v>
+        <v>19.8115</v>
       </c>
       <c r="F54" s="8" t="n">
-        <v>19.1</v>
+        <v>20.3325</v>
       </c>
       <c r="G54" s="8" t="n">
-        <v>23.5405</v>
+        <v>20.6135</v>
       </c>
       <c r="H54" s="9" t="n"/>
       <c r="I54" s="9" t="n"/>
       <c r="J54" s="8" t="n">
-        <v>20.547</v>
+        <v>20.04</v>
       </c>
     </row>
     <row r="55">
@@ -3792,24 +3792,24 @@
         </is>
       </c>
       <c r="C55" s="8" t="n">
-        <v>0.8985</v>
+        <v>0.9075</v>
       </c>
       <c r="D55" s="8" t="n">
-        <v>0.9105</v>
+        <v>0.899</v>
       </c>
       <c r="E55" s="8" t="n">
-        <v>0.9035</v>
+        <v>0.98</v>
       </c>
       <c r="F55" s="8" t="n">
-        <v>0.914</v>
+        <v>0.9765</v>
       </c>
       <c r="G55" s="8" t="n">
-        <v>1.191</v>
+        <v>0.911</v>
       </c>
       <c r="H55" s="9" t="n"/>
       <c r="I55" s="9" t="n"/>
       <c r="J55" s="8" t="n">
-        <v>0.9195</v>
+        <v>0.9185</v>
       </c>
     </row>
     <row r="56">
@@ -3820,24 +3820,24 @@
         </is>
       </c>
       <c r="C56" s="8" t="n">
-        <v>48.2825</v>
+        <v>48.277</v>
       </c>
       <c r="D56" s="8" t="n">
-        <v>59.3815</v>
+        <v>46.2445</v>
       </c>
       <c r="E56" s="8" t="n">
-        <v>51.8015</v>
+        <v>52.5005</v>
       </c>
       <c r="F56" s="8" t="n">
-        <v>51.3375</v>
+        <v>53.2565</v>
       </c>
       <c r="G56" s="8" t="n">
-        <v>61.514</v>
+        <v>57.1535</v>
       </c>
       <c r="H56" s="9" t="n"/>
       <c r="I56" s="9" t="n"/>
       <c r="J56" s="8" t="n">
-        <v>54.7575</v>
+        <v>54.098</v>
       </c>
     </row>
     <row r="57">
@@ -3852,24 +3852,24 @@
         </is>
       </c>
       <c r="C57" s="8" t="n">
-        <v>81.78</v>
+        <v>81.229</v>
       </c>
       <c r="D57" s="8" t="n">
-        <v>30.1165</v>
+        <v>25.166</v>
       </c>
       <c r="E57" s="8" t="n">
-        <v>24.1225</v>
+        <v>23.817</v>
       </c>
       <c r="F57" s="8" t="n">
-        <v>24.2605</v>
+        <v>23.907</v>
       </c>
       <c r="G57" s="8" t="n">
-        <v>50.287</v>
+        <v>50.576</v>
       </c>
       <c r="H57" s="9" t="n"/>
       <c r="I57" s="9" t="n"/>
       <c r="J57" s="8" t="n">
-        <v>79.8085</v>
+        <v>80.7675</v>
       </c>
     </row>
     <row r="58">
@@ -3880,24 +3880,24 @@
         </is>
       </c>
       <c r="C58" s="8" t="n">
-        <v>28.0925</v>
+        <v>28.1515</v>
       </c>
       <c r="D58" s="8" t="n">
-        <v>28.085</v>
+        <v>28.1145</v>
       </c>
       <c r="E58" s="8" t="n">
-        <v>28.067</v>
+        <v>28.0155</v>
       </c>
       <c r="F58" s="8" t="n">
-        <v>28.052</v>
+        <v>28.0665</v>
       </c>
       <c r="G58" s="8" t="n">
-        <v>28.028</v>
+        <v>28.068</v>
       </c>
       <c r="H58" s="9" t="n"/>
       <c r="I58" s="9" t="n"/>
       <c r="J58" s="8" t="n">
-        <v>28.136</v>
+        <v>28.061</v>
       </c>
     </row>
     <row r="59">
@@ -3908,24 +3908,24 @@
         </is>
       </c>
       <c r="C59" s="8" t="n">
-        <v>161.345</v>
+        <v>161.2095</v>
       </c>
       <c r="D59" s="8" t="n">
-        <v>161.402</v>
+        <v>162.188</v>
       </c>
       <c r="E59" s="8" t="n">
-        <v>161.0465</v>
+        <v>159.499</v>
       </c>
       <c r="F59" s="8" t="n">
-        <v>160.872</v>
+        <v>159.2555</v>
       </c>
       <c r="G59" s="8" t="n">
-        <v>160.5145</v>
+        <v>159.9755</v>
       </c>
       <c r="H59" s="9" t="n"/>
       <c r="I59" s="9" t="n"/>
       <c r="J59" s="8" t="n">
-        <v>160.156</v>
+        <v>160.188</v>
       </c>
     </row>
     <row r="60">
@@ -3936,24 +3936,24 @@
         </is>
       </c>
       <c r="C60" s="8" t="n">
-        <v>271.2215</v>
+        <v>270.6675</v>
       </c>
       <c r="D60" s="8" t="n">
-        <v>219.5055</v>
+        <v>215.509</v>
       </c>
       <c r="E60" s="8" t="n">
-        <v>213.709</v>
+        <v>212.107</v>
       </c>
       <c r="F60" s="8" t="n">
-        <v>213.5735</v>
+        <v>212.0205</v>
       </c>
       <c r="G60" s="8" t="n">
-        <v>239.0605</v>
+        <v>238.932</v>
       </c>
       <c r="H60" s="9" t="n"/>
       <c r="I60" s="9" t="n"/>
       <c r="J60" s="8" t="n">
-        <v>268.0645</v>
+        <v>269.153</v>
       </c>
     </row>
   </sheetData>
@@ -4766,10 +4766,10 @@
       </c>
       <c r="C2" s="13" t="inlineStr">
         <is>
-          <t>shipdate: 6586.64 MB
+          <t>shipdate: 6586.70 MB
 linestatus: 20.63 MB
 returnflag: 29.78 MB
-total: 6637.05 MB</t>
+total: 6637.11 MB</t>
         </is>
       </c>
       <c r="D2" s="13" t="inlineStr">
@@ -4830,9 +4830,9 @@
       </c>
       <c r="C3" s="13" t="inlineStr">
         <is>
-          <t>orderkey: 4448.84 MB
-shipdate: 6586.64 MB
-total: 11035.48 MB</t>
+          <t>orderkey: 1679.94 MB
+shipdate: 6586.70 MB
+total: 8266.64 MB</t>
         </is>
       </c>
       <c r="D3" s="13" t="inlineStr">
@@ -4888,8 +4888,8 @@
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>orderkey: 4448.84 MB
-total: 4448.84 MB</t>
+          <t>orderkey: 1679.94 MB
+total: 1679.94 MB</t>
         </is>
       </c>
       <c r="D4" s="13" t="inlineStr">
@@ -4942,9 +4942,9 @@
       </c>
       <c r="C5" s="13" t="inlineStr">
         <is>
-          <t>orderkey: 4448.84 MB
-suppkey: 13176.00 MB
-total: 17624.84 MB</t>
+          <t>orderkey: 1679.94 MB
+suppkey: 13178.40 MB
+total: 14858.34 MB</t>
         </is>
       </c>
       <c r="D5" s="13" t="inlineStr">
@@ -5066,9 +5066,9 @@
       </c>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>orderkey: 4448.84 MB
-partkey: 13567.30 MB
-total: 18016.14 MB</t>
+          <t>orderkey: 1679.94 MB
+partkey: 431.94 MB
+total: 2111.88 MB</t>
         </is>
       </c>
       <c r="D7" s="13" t="inlineStr">
@@ -5125,9 +5125,9 @@
       </c>
       <c r="C8" s="13" t="inlineStr">
         <is>
-          <t>orderkey: 4448.84 MB
+          <t>orderkey: 1679.94 MB
 returnflag: 29.78 MB
-total: 4478.62 MB</t>
+total: 1709.72 MB</t>
         </is>
       </c>
       <c r="D8" s="13" t="inlineStr">
@@ -5185,8 +5185,8 @@
       <c r="C9" s="13" t="inlineStr">
         <is>
           <t>shipmode: 58.13 MB
-receiptdate: 6593.20 MB
-total: 6651.33 MB</t>
+receiptdate: 6593.22 MB
+total: 6651.35 MB</t>
         </is>
       </c>
       <c r="D9" s="13" t="inlineStr">
@@ -5242,8 +5242,8 @@
       </c>
       <c r="C10" s="13" t="inlineStr">
         <is>
-          <t>shipdate: 6586.64 MB
-total: 6586.64 MB</t>
+          <t>shipdate: 6586.70 MB
+total: 6586.70 MB</t>
         </is>
       </c>
       <c r="D10" s="13" t="inlineStr">
@@ -5346,8 +5346,8 @@
       </c>
       <c r="C12" s="13" t="inlineStr">
         <is>
-          <t>partkey: 13567.30 MB
-total: 13567.30 MB</t>
+          <t>partkey: 431.94 MB
+total: 431.94 MB</t>
         </is>
       </c>
       <c r="D12" s="13" t="inlineStr">
@@ -5539,7 +5539,7 @@
         </is>
       </c>
       <c r="E3" s="15" t="n">
-        <v>6637.049</v>
+        <v>6637.1092</v>
       </c>
     </row>
     <row r="4">
@@ -5689,7 +5689,7 @@
         </is>
       </c>
       <c r="E9" s="15" t="n">
-        <v>11035.48</v>
+        <v>8266.639999999999</v>
       </c>
     </row>
     <row r="10">
@@ -5839,7 +5839,7 @@
         </is>
       </c>
       <c r="E15" s="15" t="n">
-        <v>4448.84</v>
+        <v>1679.94</v>
       </c>
     </row>
     <row r="16">
@@ -5989,7 +5989,7 @@
         </is>
       </c>
       <c r="E21" s="15" t="n">
-        <v>17624.84</v>
+        <v>14858.34</v>
       </c>
     </row>
     <row r="22">
@@ -6139,7 +6139,7 @@
         </is>
       </c>
       <c r="E27" s="15" t="n">
-        <v>395.9385</v>
+        <v>395.9409</v>
       </c>
     </row>
     <row r="28">
@@ -6289,7 +6289,7 @@
         </is>
       </c>
       <c r="E33" s="15" t="n">
-        <v>18016.14</v>
+        <v>2111.884</v>
       </c>
     </row>
     <row r="34">
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="E39" s="15" t="n">
-        <v>4478.6165</v>
+        <v>1709.7166</v>
       </c>
     </row>
     <row r="40">
@@ -6589,7 +6589,7 @@
         </is>
       </c>
       <c r="E45" s="15" t="n">
-        <v>6651.326</v>
+        <v>6651.3462</v>
       </c>
     </row>
     <row r="46">
@@ -6739,7 +6739,7 @@
         </is>
       </c>
       <c r="E51" s="15" t="n">
-        <v>6586.64</v>
+        <v>6586.7</v>
       </c>
     </row>
     <row r="52">
@@ -7014,7 +7014,7 @@
         </is>
       </c>
       <c r="E62" s="15" t="n">
-        <v>13567.3</v>
+        <v>431.944</v>
       </c>
     </row>
     <row r="63">
@@ -7164,7 +7164,7 @@
         </is>
       </c>
       <c r="E68" s="15" t="n">
-        <v>100.6633</v>
+        <v>100.6636</v>
       </c>
     </row>
     <row r="69">
@@ -7283,7 +7283,7 @@
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
@@ -7367,7 +7367,7 @@
         <v>505.8297</v>
       </c>
       <c r="C2" s="16" t="n">
-        <v>6637.049</v>
+        <v>6637.1092</v>
       </c>
       <c r="D2" s="16" t="n">
         <v>175.999</v>
@@ -7397,7 +7397,7 @@
         <v>1732.932</v>
       </c>
       <c r="C3" s="16" t="n">
-        <v>11035.48</v>
+        <v>8266.639999999999</v>
       </c>
       <c r="D3" s="16" t="n">
         <v>498.421</v>
@@ -7427,7 +7427,7 @@
         <v>1265.8</v>
       </c>
       <c r="C4" s="16" t="n">
-        <v>4448.84</v>
+        <v>1679.94</v>
       </c>
       <c r="D4" s="16" t="n">
         <v>359.978</v>
@@ -7457,7 +7457,7 @@
         <v>1753.143</v>
       </c>
       <c r="C5" s="16" t="n">
-        <v>17624.84</v>
+        <v>14858.34</v>
       </c>
       <c r="D5" s="16" t="n">
         <v>832.8140000000001</v>
@@ -7487,7 +7487,7 @@
         <v>412.1922</v>
       </c>
       <c r="C6" s="16" t="n">
-        <v>395.9385</v>
+        <v>395.9409</v>
       </c>
       <c r="D6" s="16" t="n">
         <v>255.4757</v>
@@ -7517,7 +7517,7 @@
         <v>1897.681</v>
       </c>
       <c r="C7" s="16" t="n">
-        <v>18016.14</v>
+        <v>2111.884</v>
       </c>
       <c r="D7" s="16" t="n">
         <v>968.067</v>
@@ -7547,7 +7547,7 @@
         <v>1289.018</v>
       </c>
       <c r="C8" s="16" t="n">
-        <v>4478.6165</v>
+        <v>1709.7166</v>
       </c>
       <c r="D8" s="16" t="n">
         <v>382.5116</v>
@@ -7577,7 +7577,7 @@
         <v>514.1715</v>
       </c>
       <c r="C9" s="16" t="n">
-        <v>6651.326</v>
+        <v>6651.3462</v>
       </c>
       <c r="D9" s="16" t="n">
         <v>183.5719</v>
@@ -7607,7 +7607,7 @@
         <v>467.132</v>
       </c>
       <c r="C10" s="16" t="n">
-        <v>6586.64</v>
+        <v>6586.7</v>
       </c>
       <c r="D10" s="16" t="n">
         <v>138.443</v>
@@ -7671,7 +7671,7 @@
         <v>631.881</v>
       </c>
       <c r="C12" s="16" t="n">
-        <v>13567.3</v>
+        <v>431.944</v>
       </c>
       <c r="D12" s="16" t="n">
         <v>608.0890000000001</v>
@@ -7701,7 +7701,7 @@
         <v>77.3993</v>
       </c>
       <c r="C13" s="16" t="n">
-        <v>100.6633</v>
+        <v>100.6636</v>
       </c>
       <c r="D13" s="16" t="n">
         <v>75.1007</v>

</xml_diff>